<commit_message>
Update bracket sim outputs (2026-03-04)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.2</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>79.5</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>58.6</v>
+        <v>60.6</v>
       </c>
       <c r="J2" t="n">
-        <v>41.8</v>
+        <v>43.4</v>
       </c>
       <c r="K2" t="n">
-        <v>27.7</v>
+        <v>29.7</v>
       </c>
       <c r="L2" t="n">
-        <v>17</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="3">
@@ -551,19 +551,19 @@
         <v>89.7</v>
       </c>
       <c r="H3" t="n">
-        <v>65.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="I3" t="n">
         <v>35.8</v>
       </c>
       <c r="J3" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="K3" t="n">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="L3" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="4">
@@ -595,13 +595,13 @@
         <v>87.5</v>
       </c>
       <c r="H4" t="n">
-        <v>60.8</v>
+        <v>60.9</v>
       </c>
       <c r="I4" t="n">
-        <v>36.7</v>
+        <v>36.8</v>
       </c>
       <c r="J4" t="n">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="K4" t="n">
         <v>8.5</v>
@@ -639,19 +639,19 @@
         <v>87</v>
       </c>
       <c r="H5" t="n">
-        <v>54.2</v>
+        <v>51.8</v>
       </c>
       <c r="I5" t="n">
-        <v>21.1</v>
+        <v>20.1</v>
       </c>
       <c r="J5" t="n">
-        <v>11.4</v>
+        <v>10.6</v>
       </c>
       <c r="K5" t="n">
-        <v>5.3</v>
+        <v>4.7</v>
       </c>
       <c r="L5" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="6">
@@ -683,19 +683,19 @@
         <v>80.40000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>39.4</v>
+        <v>41.7</v>
       </c>
       <c r="I6" t="n">
-        <v>12.8</v>
+        <v>11.9</v>
       </c>
       <c r="J6" t="n">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="K6" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="L6" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -727,16 +727,16 @@
         <v>66.8</v>
       </c>
       <c r="H7" t="n">
-        <v>25.4</v>
+        <v>25.7</v>
       </c>
       <c r="I7" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="J7" t="n">
         <v>3.7</v>
       </c>
       <c r="K7" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="L7" t="n">
         <v>0.5</v>
@@ -768,19 +768,19 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>57.1</v>
+        <v>54.1</v>
       </c>
       <c r="H8" t="n">
-        <v>19.8</v>
+        <v>18.7</v>
       </c>
       <c r="I8" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="J8" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L8" t="n">
         <v>0.1</v>
@@ -815,10 +815,10 @@
         <v>44.5</v>
       </c>
       <c r="H9" t="n">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="I9" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="J9" t="n">
         <v>0.8</v>
@@ -859,19 +859,19 @@
         <v>55.5</v>
       </c>
       <c r="H10" t="n">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="J10" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="K10" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
@@ -900,16 +900,16 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>42.9</v>
+        <v>45.9</v>
       </c>
       <c r="H11" t="n">
-        <v>12.6</v>
+        <v>13.5</v>
       </c>
       <c r="I11" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K11" t="n">
         <v>0.2</v>
@@ -947,13 +947,13 @@
         <v>18.5</v>
       </c>
       <c r="H12" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="I12" t="n">
         <v>2.4</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K12" t="n">
         <v>0.2</v>
@@ -1123,7 +1123,7 @@
         <v>12.4</v>
       </c>
       <c r="H16" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="I16" t="n">
         <v>0.4</v>
@@ -1208,7 +1208,7 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="H18" t="n">
         <v>0.1</v>
@@ -1255,19 +1255,19 @@
         <v>92.09999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>67.59999999999999</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>36.1</v>
+        <v>35.9</v>
       </c>
       <c r="J19" t="n">
-        <v>16.4</v>
+        <v>16.8</v>
       </c>
       <c r="K19" t="n">
         <v>6.8</v>
       </c>
       <c r="L19" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="20">
@@ -1299,19 +1299,19 @@
         <v>96</v>
       </c>
       <c r="H20" t="n">
-        <v>72.59999999999999</v>
+        <v>75.8</v>
       </c>
       <c r="I20" t="n">
-        <v>44.4</v>
+        <v>45.5</v>
       </c>
       <c r="J20" t="n">
-        <v>28.3</v>
+        <v>29.9</v>
       </c>
       <c r="K20" t="n">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="L20" t="n">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1343,19 +1343,19 @@
         <v>87.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>58.1</v>
+        <v>61.2</v>
       </c>
       <c r="I21" t="n">
-        <v>31.1</v>
+        <v>33</v>
       </c>
       <c r="J21" t="n">
-        <v>19.4</v>
+        <v>20.7</v>
       </c>
       <c r="K21" t="n">
-        <v>9.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="22">
@@ -1384,22 +1384,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>84.59999999999999</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>54</v>
+        <v>49.8</v>
       </c>
       <c r="I22" t="n">
-        <v>31.1</v>
+        <v>28.5</v>
       </c>
       <c r="J22" t="n">
-        <v>15.5</v>
+        <v>12.1</v>
       </c>
       <c r="K22" t="n">
-        <v>6.8</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="23">
@@ -1431,16 +1431,16 @@
         <v>68.09999999999999</v>
       </c>
       <c r="H23" t="n">
-        <v>33</v>
+        <v>34.9</v>
       </c>
       <c r="I23" t="n">
-        <v>16.9</v>
+        <v>17.9</v>
       </c>
       <c r="J23" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="K23" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="L23" t="n">
         <v>0.9</v>
@@ -1472,22 +1472,22 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>63</v>
+        <v>62.4</v>
       </c>
       <c r="H24" t="n">
-        <v>26.5</v>
+        <v>23.1</v>
       </c>
       <c r="I24" t="n">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="J24" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="K24" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="L24" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="25">
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>59.3</v>
+        <v>56.8</v>
       </c>
       <c r="H25" t="n">
-        <v>17.8</v>
+        <v>13.9</v>
       </c>
       <c r="I25" t="n">
-        <v>8.199999999999999</v>
+        <v>5.7</v>
       </c>
       <c r="J25" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="L25" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -1560,13 +1560,13 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>45.5</v>
+        <v>44.2</v>
       </c>
       <c r="H26" t="n">
-        <v>13.1</v>
+        <v>12.7</v>
       </c>
       <c r="I26" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="J26" t="n">
         <v>1.1</v>
@@ -1604,19 +1604,19 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>54.5</v>
+        <v>55.8</v>
       </c>
       <c r="H27" t="n">
-        <v>18.6</v>
+        <v>20.7</v>
       </c>
       <c r="I27" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
       <c r="J27" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K27" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="L27" t="n">
         <v>0.2</v>
@@ -1648,19 +1648,19 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>40.7</v>
+        <v>43.2</v>
       </c>
       <c r="H28" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I28" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="K28" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L28" t="n">
         <v>0.1</v>
@@ -1692,16 +1692,16 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>37</v>
+        <v>37.6</v>
       </c>
       <c r="H29" t="n">
-        <v>12.9</v>
+        <v>13.4</v>
       </c>
       <c r="I29" t="n">
         <v>3.3</v>
       </c>
       <c r="J29" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="K29" t="n">
         <v>0.3</v>
@@ -1739,13 +1739,13 @@
         <v>31.9</v>
       </c>
       <c r="H30" t="n">
-        <v>8.5</v>
+        <v>10.7</v>
       </c>
       <c r="I30" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K30" t="n">
         <v>0.1</v>
@@ -1780,10 +1780,10 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>15.4</v>
+        <v>16.6</v>
       </c>
       <c r="H31" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="I31" t="n">
         <v>0.9</v>
@@ -1827,10 +1827,10 @@
         <v>12.4</v>
       </c>
       <c r="H32" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1871,7 +1871,7 @@
         <v>4</v>
       </c>
       <c r="H33" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I33" t="n">
         <v>0.1</v>
@@ -2000,22 +2000,22 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>97.5</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>79.5</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>57.8</v>
+        <v>56.7</v>
       </c>
       <c r="J36" t="n">
-        <v>39.2</v>
+        <v>38.8</v>
       </c>
       <c r="K36" t="n">
-        <v>25.1</v>
+        <v>23.7</v>
       </c>
       <c r="L36" t="n">
-        <v>14.7</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="37">
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>93.7</v>
+        <v>91.5</v>
       </c>
       <c r="H37" t="n">
-        <v>67.09999999999999</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="I37" t="n">
-        <v>46.6</v>
+        <v>47.1</v>
       </c>
       <c r="J37" t="n">
-        <v>24.5</v>
+        <v>24.8</v>
       </c>
       <c r="K37" t="n">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
       <c r="L37" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="38">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>81.2</v>
+        <v>79.8</v>
       </c>
       <c r="H38" t="n">
-        <v>50.4</v>
+        <v>48.9</v>
       </c>
       <c r="I38" t="n">
-        <v>22.1</v>
+        <v>19.5</v>
       </c>
       <c r="J38" t="n">
-        <v>8.6</v>
+        <v>7.5</v>
       </c>
       <c r="K38" t="n">
-        <v>3.6</v>
+        <v>2.8</v>
       </c>
       <c r="L38" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2138,13 +2138,13 @@
         <v>43.7</v>
       </c>
       <c r="I39" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="J39" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="K39" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="L39" t="n">
         <v>0.9</v>
@@ -2182,16 +2182,16 @@
         <v>48.5</v>
       </c>
       <c r="I40" t="n">
-        <v>17.7</v>
+        <v>18.3</v>
       </c>
       <c r="J40" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K40" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="L40" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
@@ -2220,22 +2220,22 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>60.6</v>
+        <v>58.2</v>
       </c>
       <c r="H41" t="n">
-        <v>29.7</v>
+        <v>28.5</v>
       </c>
       <c r="I41" t="n">
-        <v>11.1</v>
+        <v>10.7</v>
       </c>
       <c r="J41" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="K41" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L41" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="42">
@@ -2267,16 +2267,16 @@
         <v>55.2</v>
       </c>
       <c r="H42" t="n">
-        <v>17.7</v>
+        <v>18.4</v>
       </c>
       <c r="I42" t="n">
-        <v>9</v>
+        <v>9.6</v>
       </c>
       <c r="J42" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="K42" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
         <v>0.2</v>
@@ -2308,19 +2308,19 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>44.6</v>
+        <v>47.2</v>
       </c>
       <c r="H43" t="n">
-        <v>9.199999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="I43" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="J43" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="K43" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2352,16 +2352,16 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>55.4</v>
+        <v>52.8</v>
       </c>
       <c r="H44" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="I44" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="J44" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K44" t="n">
         <v>0.4</v>
@@ -2399,13 +2399,13 @@
         <v>44.8</v>
       </c>
       <c r="H45" t="n">
-        <v>14.7</v>
+        <v>15.4</v>
       </c>
       <c r="I45" t="n">
-        <v>6.3</v>
+        <v>7.4</v>
       </c>
       <c r="J45" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="K45" t="n">
         <v>0.6</v>
@@ -2440,16 +2440,16 @@
         <v>48.6</v>
       </c>
       <c r="G46" t="n">
-        <v>17.9</v>
+        <v>20.3</v>
       </c>
       <c r="H46" t="n">
-        <v>6.9</v>
+        <v>8.4</v>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="J46" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K46" t="n">
         <v>0.1</v>
@@ -2487,10 +2487,10 @@
         <v>21.5</v>
       </c>
       <c r="H47" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="J47" t="n">
         <v>0.5</v>
@@ -2534,7 +2534,7 @@
         <v>3.3</v>
       </c>
       <c r="I48" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>18.8</v>
+        <v>20.2</v>
       </c>
       <c r="H50" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="I50" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J50" t="n">
         <v>0.1</v>
@@ -2660,10 +2660,10 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>6.3</v>
+        <v>8.5</v>
       </c>
       <c r="H51" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="I51" t="n">
         <v>0.1</v>
@@ -2704,10 +2704,10 @@
         <v>56.2</v>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="H52" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>96.09999999999999</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H54" t="n">
-        <v>77</v>
+        <v>75.7</v>
       </c>
       <c r="I54" t="n">
-        <v>53.4</v>
+        <v>56.3</v>
       </c>
       <c r="J54" t="n">
-        <v>36.4</v>
+        <v>39.6</v>
       </c>
       <c r="K54" t="n">
-        <v>21.3</v>
+        <v>24.5</v>
       </c>
       <c r="L54" t="n">
-        <v>13.6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55">
@@ -2839,19 +2839,19 @@
         <v>93.5</v>
       </c>
       <c r="H55" t="n">
-        <v>63.3</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="I55" t="n">
-        <v>41.9</v>
+        <v>49.3</v>
       </c>
       <c r="J55" t="n">
-        <v>21.4</v>
+        <v>24.6</v>
       </c>
       <c r="K55" t="n">
-        <v>10.3</v>
+        <v>12.4</v>
       </c>
       <c r="L55" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="56">
@@ -2886,16 +2886,16 @@
         <v>47.1</v>
       </c>
       <c r="I56" t="n">
-        <v>20.5</v>
+        <v>17.5</v>
       </c>
       <c r="J56" t="n">
-        <v>7.3</v>
+        <v>5.8</v>
       </c>
       <c r="K56" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="L56" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>71.90000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="H57" t="n">
-        <v>43.1</v>
+        <v>42.1</v>
       </c>
       <c r="I57" t="n">
-        <v>18.1</v>
+        <v>15.2</v>
       </c>
       <c r="J57" t="n">
-        <v>10.2</v>
+        <v>8.1</v>
       </c>
       <c r="K57" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="L57" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="58">
@@ -2971,19 +2971,19 @@
         <v>74.3</v>
       </c>
       <c r="H58" t="n">
-        <v>41.1</v>
+        <v>41.3</v>
       </c>
       <c r="I58" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="J58" t="n">
-        <v>8.1</v>
+        <v>7</v>
       </c>
       <c r="K58" t="n">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
       <c r="L58" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -3018,16 +3018,16 @@
         <v>37.3</v>
       </c>
       <c r="I59" t="n">
-        <v>15.3</v>
+        <v>13.2</v>
       </c>
       <c r="J59" t="n">
-        <v>5.5</v>
+        <v>4.4</v>
       </c>
       <c r="K59" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="L59" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="60">
@@ -3059,16 +3059,16 @@
         <v>63.1</v>
       </c>
       <c r="H60" t="n">
-        <v>24.8</v>
+        <v>22.6</v>
       </c>
       <c r="I60" t="n">
-        <v>14.3</v>
+        <v>13.2</v>
       </c>
       <c r="J60" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="K60" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L60" t="n">
         <v>0.7</v>
@@ -3103,13 +3103,13 @@
         <v>51.4</v>
       </c>
       <c r="H61" t="n">
-        <v>11.7</v>
+        <v>12.4</v>
       </c>
       <c r="I61" t="n">
-        <v>4.5</v>
+        <v>4.8</v>
       </c>
       <c r="J61" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="K61" t="n">
         <v>0.4</v>
@@ -3147,13 +3147,13 @@
         <v>48.6</v>
       </c>
       <c r="H62" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="I62" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="J62" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K62" t="n">
         <v>0.3</v>
@@ -3191,16 +3191,16 @@
         <v>36.9</v>
       </c>
       <c r="H63" t="n">
-        <v>11.2</v>
+        <v>8.9</v>
       </c>
       <c r="I63" t="n">
-        <v>4.8</v>
+        <v>3.9</v>
       </c>
       <c r="J63" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="K63" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L63" t="n">
         <v>0.1</v>
@@ -3238,7 +3238,7 @@
         <v>9.6</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="J64" t="n">
         <v>0.4</v>
@@ -3279,10 +3279,10 @@
         <v>25.7</v>
       </c>
       <c r="H65" t="n">
-        <v>9</v>
+        <v>9.6</v>
       </c>
       <c r="I65" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="J65" t="n">
         <v>0.6</v>
@@ -3320,10 +3320,10 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="H66" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="I66" t="n">
         <v>1.6</v>
@@ -3370,10 +3370,10 @@
         <v>6</v>
       </c>
       <c r="I67" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="J67" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>3.9</v>
+        <v>6.1</v>
       </c>
       <c r="H69" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="I69" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-05)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,62 +429,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TeamID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>TeamName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Is_FirstFour</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pct_R64</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pct_R32</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pct_S16</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pct_E8</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pct_F4</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pct_Finals</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pct_Champion</t>
         </is>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-06)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -507,19 +507,19 @@
         <v>98.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>80.90000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="I2" t="n">
-        <v>61.2</v>
+        <v>61.1</v>
       </c>
       <c r="J2" t="n">
-        <v>43.8</v>
+        <v>43.4</v>
       </c>
       <c r="K2" t="n">
-        <v>30</v>
+        <v>30.4</v>
       </c>
       <c r="L2" t="n">
-        <v>18.3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -554,16 +554,16 @@
         <v>66.2</v>
       </c>
       <c r="I3" t="n">
-        <v>35.9</v>
+        <v>37</v>
       </c>
       <c r="J3" t="n">
-        <v>15</v>
+        <v>16.6</v>
       </c>
       <c r="K3" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="4">
@@ -592,31 +592,31 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>87.5</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>60.9</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>36.8</v>
+        <v>40.8</v>
       </c>
       <c r="J4" t="n">
-        <v>16</v>
+        <v>17.4</v>
       </c>
       <c r="K4" t="n">
-        <v>8.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>4</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1211</v>
+        <v>1104</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -636,19 +636,19 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>87</v>
+        <v>76.5</v>
       </c>
       <c r="H5" t="n">
-        <v>51.8</v>
+        <v>46.5</v>
       </c>
       <c r="I5" t="n">
-        <v>19.8</v>
+        <v>19.1</v>
       </c>
       <c r="J5" t="n">
-        <v>10.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="L5" t="n">
         <v>1.9</v>
@@ -656,11 +656,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1397</v>
+        <v>1385</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,31 +680,31 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>80.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>41.7</v>
+        <v>38.9</v>
       </c>
       <c r="I6" t="n">
-        <v>11.9</v>
+        <v>10.7</v>
       </c>
       <c r="J6" t="n">
-        <v>5.8</v>
+        <v>4.5</v>
       </c>
       <c r="K6" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1257</v>
+        <v>1246</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -724,31 +724,31 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>66.8</v>
+        <v>59.4</v>
       </c>
       <c r="H7" t="n">
-        <v>25.7</v>
+        <v>20.2</v>
       </c>
       <c r="I7" t="n">
-        <v>12.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>3.8</v>
+        <v>2.3</v>
       </c>
       <c r="K7" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1437</v>
+        <v>1274</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -768,19 +768,19 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>54.1</v>
+        <v>56.7</v>
       </c>
       <c r="H8" t="n">
-        <v>18.4</v>
+        <v>19.3</v>
       </c>
       <c r="I8" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="J8" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L8" t="n">
         <v>0.1</v>
@@ -788,11 +788,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1387</v>
+        <v>1429</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Utah St</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -812,31 +812,31 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>45.3</v>
+        <v>56.2</v>
       </c>
       <c r="H9" t="n">
-        <v>8</v>
+        <v>10.8</v>
       </c>
       <c r="I9" t="n">
-        <v>2.3</v>
+        <v>4.8</v>
       </c>
       <c r="J9" t="n">
-        <v>0.7</v>
+        <v>1.7</v>
       </c>
       <c r="K9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L9" t="n">
         <v>0.2</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1234</v>
+        <v>1417</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -856,31 +856,31 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>54.7</v>
+        <v>43.8</v>
       </c>
       <c r="H10" t="n">
-        <v>11.1</v>
+        <v>6.6</v>
       </c>
       <c r="I10" t="n">
-        <v>4.1</v>
+        <v>2.7</v>
       </c>
       <c r="J10" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1395</v>
+        <v>1281</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -900,19 +900,19 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>45.9</v>
+        <v>43.3</v>
       </c>
       <c r="H11" t="n">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L11" t="n">
         <v>0.1</v>
@@ -920,11 +920,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1365</v>
+        <v>1374</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -941,34 +941,34 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>53.1</v>
+        <v>47.6</v>
       </c>
       <c r="G12" t="n">
-        <v>17.5</v>
+        <v>18.2</v>
       </c>
       <c r="H12" t="n">
-        <v>6.3</v>
+        <v>5.3</v>
       </c>
       <c r="I12" t="n">
-        <v>2.3</v>
+        <v>1.7</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K12" t="n">
         <v>0.1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1326</v>
+        <v>1231</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ohio St</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -985,16 +985,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>46.9</v>
+        <v>52.4</v>
       </c>
       <c r="G13" t="n">
-        <v>15.7</v>
+        <v>22.4</v>
       </c>
       <c r="H13" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="I13" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="J13" t="n">
         <v>0.4</v>
@@ -1008,11 +1008,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1463</v>
+        <v>1125</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>Belmont</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1032,19 +1032,19 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>19.6</v>
+        <v>26.5</v>
       </c>
       <c r="H14" t="n">
-        <v>3.7</v>
+        <v>9.4</v>
       </c>
       <c r="I14" t="n">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="J14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K14" t="n">
         <v>0.1</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1076,13 +1076,13 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>13</v>
+        <v>23.5</v>
       </c>
       <c r="H15" t="n">
-        <v>2.8</v>
+        <v>5.2</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="J15" t="n">
         <v>0.1</v>
@@ -1096,11 +1096,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1295</v>
+        <v>1407</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1120,16 +1120,16 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>12.4</v>
+        <v>10.4</v>
       </c>
       <c r="H16" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="I16" t="n">
         <v>0.4</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1167,10 +1167,10 @@
         <v>10.3</v>
       </c>
       <c r="H17" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>92.09999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>65.90000000000001</v>
+        <v>62.6</v>
       </c>
       <c r="I19" t="n">
-        <v>35.2</v>
+        <v>38.8</v>
       </c>
       <c r="J19" t="n">
-        <v>16.9</v>
+        <v>18.6</v>
       </c>
       <c r="K19" t="n">
-        <v>6.9</v>
+        <v>7.4</v>
       </c>
       <c r="L19" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="20">
@@ -1299,19 +1299,19 @@
         <v>96</v>
       </c>
       <c r="H20" t="n">
-        <v>75.8</v>
+        <v>78</v>
       </c>
       <c r="I20" t="n">
-        <v>47.2</v>
+        <v>48.6</v>
       </c>
       <c r="J20" t="n">
-        <v>31</v>
+        <v>32.4</v>
       </c>
       <c r="K20" t="n">
-        <v>16.7</v>
+        <v>16.9</v>
       </c>
       <c r="L20" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1340,19 +1340,19 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>87.59999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>60.8</v>
+        <v>60.3</v>
       </c>
       <c r="I21" t="n">
-        <v>31.1</v>
+        <v>30.8</v>
       </c>
       <c r="J21" t="n">
-        <v>19.3</v>
+        <v>18.7</v>
       </c>
       <c r="K21" t="n">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="L21" t="n">
         <v>4.4</v>
@@ -1360,11 +1360,11 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1403</v>
+        <v>1438</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1384,31 +1384,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>83.40000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="H22" t="n">
-        <v>49.3</v>
+        <v>40.2</v>
       </c>
       <c r="I22" t="n">
-        <v>27.9</v>
+        <v>17.5</v>
       </c>
       <c r="J22" t="n">
-        <v>11.7</v>
+        <v>6</v>
       </c>
       <c r="K22" t="n">
-        <v>4.8</v>
+        <v>1.8</v>
       </c>
       <c r="L22" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1116</v>
+        <v>1397</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1428,31 +1428,31 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>70.8</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>36.2</v>
+        <v>51.9</v>
       </c>
       <c r="I23" t="n">
-        <v>19.1</v>
+        <v>26.3</v>
       </c>
       <c r="J23" t="n">
-        <v>7.6</v>
+        <v>10.7</v>
       </c>
       <c r="K23" t="n">
-        <v>2.8</v>
+        <v>3.9</v>
       </c>
       <c r="L23" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1140</v>
+        <v>1257</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BYU</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1472,19 +1472,19 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>62.4</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H24" t="n">
-        <v>23.5</v>
+        <v>28.2</v>
       </c>
       <c r="I24" t="n">
-        <v>8.699999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="J24" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
       <c r="K24" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="L24" t="n">
         <v>0.4</v>
@@ -1492,11 +1492,11 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1429</v>
+        <v>1437</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Utah St</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1516,19 +1516,19 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>56.8</v>
+        <v>47.7</v>
       </c>
       <c r="H25" t="n">
-        <v>13.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I25" t="n">
-        <v>5.7</v>
+        <v>3.3</v>
       </c>
       <c r="J25" t="n">
-        <v>2.1</v>
+        <v>1.2</v>
       </c>
       <c r="K25" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="L25" t="n">
         <v>0.1</v>
@@ -1536,11 +1536,11 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1274</v>
+        <v>1387</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1560,31 +1560,31 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>44.2</v>
+        <v>45.1</v>
       </c>
       <c r="H26" t="n">
-        <v>12.7</v>
+        <v>15.3</v>
       </c>
       <c r="I26" t="n">
-        <v>5.1</v>
+        <v>6.8</v>
       </c>
       <c r="J26" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="K26" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1208</v>
+        <v>1234</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1604,31 +1604,31 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>55.8</v>
+        <v>54.9</v>
       </c>
       <c r="H27" t="n">
-        <v>20.7</v>
+        <v>21.2</v>
       </c>
       <c r="I27" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="J27" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="K27" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1417</v>
+        <v>1401</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1648,19 +1648,19 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>43.2</v>
+        <v>52.3</v>
       </c>
       <c r="H28" t="n">
-        <v>9.699999999999999</v>
+        <v>11.6</v>
       </c>
       <c r="I28" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="J28" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="K28" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L28" t="n">
         <v>0.1</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1401</v>
+        <v>1365</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1682,41 +1682,41 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>56.1</v>
       </c>
       <c r="G29" t="n">
-        <v>37.6</v>
+        <v>18.5</v>
       </c>
       <c r="H29" t="n">
-        <v>13.4</v>
+        <v>6.8</v>
       </c>
       <c r="I29" t="n">
-        <v>3.3</v>
+        <v>1.8</v>
       </c>
       <c r="J29" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="K29" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1378</v>
+        <v>1307</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1726,29 +1726,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>100</v>
+        <v>43.9</v>
       </c>
       <c r="G30" t="n">
-        <v>29.2</v>
+        <v>13.1</v>
       </c>
       <c r="H30" t="n">
-        <v>9.800000000000001</v>
+        <v>3.3</v>
       </c>
       <c r="I30" t="n">
-        <v>2.8</v>
+        <v>0.7</v>
       </c>
       <c r="J30" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -1756,11 +1756,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1372</v>
+        <v>1251</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SF Austin</t>
+          <t>Liberty</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E31" t="b">
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>16.6</v>
+        <v>15.6</v>
       </c>
       <c r="H31" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="I31" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1800,11 +1800,11 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1407</v>
+        <v>1465</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Cal Baptist</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E32" t="b">
@@ -1824,16 +1824,16 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>12.4</v>
+        <v>19.5</v>
       </c>
       <c r="H32" t="n">
-        <v>2.3</v>
+        <v>4.6</v>
       </c>
       <c r="I32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J32" t="n">
         <v>0.1</v>
-      </c>
-      <c r="J32" t="n">
-        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1467</v>
+        <v>1295</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Merrimack</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -1868,13 +1868,13 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>4</v>
+        <v>9.1</v>
       </c>
       <c r="H33" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="I33" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1888,11 +1888,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1254</v>
+        <v>1467</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Merrimack</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1902,23 +1902,23 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>52.2</v>
+        <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1420</v>
+        <v>1398</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1946,23 +1946,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>47.8</v>
+        <v>60</v>
       </c>
       <c r="G35" t="n">
-        <v>4.7</v>
+        <v>6.2</v>
       </c>
       <c r="H35" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1976,55 +1976,55 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1276</v>
+        <v>1254</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G36" t="n">
-        <v>95.90000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="H36" t="n">
-        <v>78.09999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="I36" t="n">
-        <v>56.7</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>38.6</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>23.6</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>13.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1222</v>
+        <v>1276</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E37" t="b">
@@ -2044,31 +2044,31 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>91.5</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="H37" t="n">
-        <v>66.8</v>
+        <v>80</v>
       </c>
       <c r="I37" t="n">
-        <v>48.1</v>
+        <v>59.3</v>
       </c>
       <c r="J37" t="n">
-        <v>25.4</v>
+        <v>38.6</v>
       </c>
       <c r="K37" t="n">
-        <v>14.2</v>
+        <v>22.5</v>
       </c>
       <c r="L37" t="n">
-        <v>7</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1304</v>
+        <v>1222</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E38" t="b">
@@ -2088,31 +2088,31 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>79.8</v>
+        <v>93.5</v>
       </c>
       <c r="H38" t="n">
-        <v>48.1</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="I38" t="n">
-        <v>19</v>
+        <v>45.5</v>
       </c>
       <c r="J38" t="n">
-        <v>7.2</v>
+        <v>24.6</v>
       </c>
       <c r="K38" t="n">
-        <v>2.7</v>
+        <v>13.2</v>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1438</v>
+        <v>1304</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E39" t="b">
@@ -2132,31 +2132,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H39" t="n">
-        <v>43.7</v>
+        <v>47.9</v>
       </c>
       <c r="I39" t="n">
-        <v>15.9</v>
+        <v>19.1</v>
       </c>
       <c r="J39" t="n">
-        <v>6.6</v>
+        <v>7.5</v>
       </c>
       <c r="K39" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="L39" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1435</v>
+        <v>1242</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E40" t="b">
@@ -2176,31 +2176,31 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>84.8</v>
+        <v>72.7</v>
       </c>
       <c r="H40" t="n">
-        <v>48.5</v>
+        <v>40.3</v>
       </c>
       <c r="I40" t="n">
-        <v>18.3</v>
+        <v>14.3</v>
       </c>
       <c r="J40" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="K40" t="n">
-        <v>3.2</v>
+        <v>1.9</v>
       </c>
       <c r="L40" t="n">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1314</v>
+        <v>1116</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E41" t="b">
@@ -2220,31 +2220,31 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>60.6</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H41" t="n">
-        <v>29.7</v>
+        <v>39.1</v>
       </c>
       <c r="I41" t="n">
-        <v>10.8</v>
+        <v>13.6</v>
       </c>
       <c r="J41" t="n">
-        <v>4.2</v>
+        <v>6.2</v>
       </c>
       <c r="K41" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="L41" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1458</v>
+        <v>1435</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E42" t="b">
@@ -2264,31 +2264,31 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>56.2</v>
+        <v>72.2</v>
       </c>
       <c r="H42" t="n">
-        <v>18.8</v>
+        <v>44.1</v>
       </c>
       <c r="I42" t="n">
-        <v>9.9</v>
+        <v>18.6</v>
       </c>
       <c r="J42" t="n">
-        <v>3.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K42" t="n">
-        <v>1.1</v>
+        <v>2.9</v>
       </c>
       <c r="L42" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1416</v>
+        <v>1388</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E43" t="b">
@@ -2308,31 +2308,31 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>47.2</v>
+        <v>63.4</v>
       </c>
       <c r="H43" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="I43" t="n">
         <v>10.2</v>
       </c>
-      <c r="I43" t="n">
-        <v>3.8</v>
-      </c>
       <c r="J43" t="n">
-        <v>1.1</v>
+        <v>4</v>
       </c>
       <c r="K43" t="n">
-        <v>0.3</v>
+        <v>1.4</v>
       </c>
       <c r="L43" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1301</v>
+        <v>1155</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E44" t="b">
@@ -2352,31 +2352,31 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>52.8</v>
+        <v>54.2</v>
       </c>
       <c r="H44" t="n">
-        <v>11.4</v>
+        <v>9.4</v>
       </c>
       <c r="I44" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="J44" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L44" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1400</v>
+        <v>1416</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E45" t="b">
@@ -2396,19 +2396,19 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>43.8</v>
+        <v>45.8</v>
       </c>
       <c r="H45" t="n">
-        <v>13.9</v>
+        <v>10.2</v>
       </c>
       <c r="I45" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
       <c r="J45" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="K45" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L45" t="n">
         <v>0.1</v>
@@ -2416,11 +2416,11 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1307</v>
+        <v>1326</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Ohio St</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2430,41 +2430,41 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>48.6</v>
+        <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>17.9</v>
+        <v>36.5</v>
       </c>
       <c r="H46" t="n">
-        <v>7</v>
+        <v>11.7</v>
       </c>
       <c r="I46" t="n">
-        <v>1.8</v>
+        <v>4.9</v>
       </c>
       <c r="J46" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="K46" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L46" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L46" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1231</v>
+        <v>1275</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2474,41 +2474,41 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>51.4</v>
+        <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>21.5</v>
+        <v>27.8</v>
       </c>
       <c r="H47" t="n">
-        <v>9.199999999999999</v>
+        <v>6.6</v>
       </c>
       <c r="I47" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="J47" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="K47" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1251</v>
+        <v>1378</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>15.2</v>
+        <v>31.6</v>
       </c>
       <c r="H48" t="n">
-        <v>3.3</v>
+        <v>12.2</v>
       </c>
       <c r="I48" t="n">
-        <v>0.4</v>
+        <v>3.1</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1465</v>
+        <v>1219</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cal Baptist</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2572,16 +2572,16 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>19</v>
+        <v>27.3</v>
       </c>
       <c r="H49" t="n">
-        <v>4.4</v>
+        <v>8.5</v>
       </c>
       <c r="I49" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2592,11 +2592,11 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1414</v>
+        <v>1298</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>UC Irvine</t>
+          <t>Navy</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2616,19 +2616,19 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>20.2</v>
+        <v>12</v>
       </c>
       <c r="H50" t="n">
-        <v>6</v>
+        <v>1.4</v>
       </c>
       <c r="I50" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="J50" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
@@ -2636,11 +2636,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1340</v>
+        <v>1190</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Portland St</t>
+          <t>ETSU</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2660,7 +2660,7 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>8.5</v>
+        <v>6.5</v>
       </c>
       <c r="H51" t="n">
         <v>0.6</v>
@@ -2704,10 +2704,10 @@
         <v>56.2</v>
       </c>
       <c r="G52" t="n">
-        <v>3.6</v>
+        <v>3.9</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>93.90000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>75.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>56.3</v>
+        <v>56.5</v>
       </c>
       <c r="J54" t="n">
-        <v>39.6</v>
+        <v>38.8</v>
       </c>
       <c r="K54" t="n">
-        <v>24.4</v>
+        <v>24</v>
       </c>
       <c r="L54" t="n">
-        <v>16</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="55">
@@ -2836,31 +2836,31 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>93.5</v>
+        <v>91.8</v>
       </c>
       <c r="H55" t="n">
-        <v>67.90000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="I55" t="n">
-        <v>49.3</v>
+        <v>42.4</v>
       </c>
       <c r="J55" t="n">
-        <v>24.6</v>
+        <v>21.5</v>
       </c>
       <c r="K55" t="n">
-        <v>12.4</v>
+        <v>10.9</v>
       </c>
       <c r="L55" t="n">
-        <v>6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1242</v>
+        <v>1211</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2880,31 +2880,31 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>76.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="H56" t="n">
-        <v>47.1</v>
+        <v>62.6</v>
       </c>
       <c r="I56" t="n">
-        <v>17.5</v>
+        <v>32.5</v>
       </c>
       <c r="J56" t="n">
-        <v>5.8</v>
+        <v>15.1</v>
       </c>
       <c r="K56" t="n">
-        <v>1.9</v>
+        <v>7.5</v>
       </c>
       <c r="L56" t="n">
-        <v>0.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1104</v>
+        <v>1403</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2924,19 +2924,19 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>71.09999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="H57" t="n">
-        <v>42.1</v>
+        <v>52.4</v>
       </c>
       <c r="I57" t="n">
-        <v>15.2</v>
+        <v>19.9</v>
       </c>
       <c r="J57" t="n">
-        <v>8.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K57" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="L57" t="n">
         <v>1.5</v>
@@ -2944,11 +2944,11 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1385</v>
+        <v>1314</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2968,31 +2968,31 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>74.3</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>41.3</v>
+        <v>33.6</v>
       </c>
       <c r="I58" t="n">
-        <v>15.7</v>
+        <v>9.4</v>
       </c>
       <c r="J58" t="n">
-        <v>7.1</v>
+        <v>3.4</v>
       </c>
       <c r="K58" t="n">
-        <v>2.9</v>
+        <v>1.3</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1246</v>
+        <v>1458</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3012,31 +3012,31 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>72.2</v>
+        <v>56.7</v>
       </c>
       <c r="H59" t="n">
-        <v>37.3</v>
+        <v>20.9</v>
       </c>
       <c r="I59" t="n">
-        <v>13.2</v>
+        <v>7.4</v>
       </c>
       <c r="J59" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="K59" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="L59" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1388</v>
+        <v>1140</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>BYU</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3056,31 +3056,31 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>63.1</v>
+        <v>63.4</v>
       </c>
       <c r="H60" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="I60" t="n">
-        <v>13.2</v>
+        <v>9.6</v>
       </c>
       <c r="J60" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="K60" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="L60" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1155</v>
+        <v>1208</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3100,31 +3100,31 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>51.4</v>
+        <v>55</v>
       </c>
       <c r="H61" t="n">
-        <v>12.4</v>
+        <v>15.5</v>
       </c>
       <c r="I61" t="n">
-        <v>4.8</v>
+        <v>7.3</v>
       </c>
       <c r="J61" t="n">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="K61" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="L61" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1281</v>
+        <v>1301</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3144,13 +3144,13 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>48.6</v>
+        <v>45</v>
       </c>
       <c r="H62" t="n">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="I62" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="J62" t="n">
         <v>1.1</v>
@@ -3164,11 +3164,11 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1374</v>
+        <v>1395</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3188,31 +3188,31 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>36.9</v>
+        <v>36.6</v>
       </c>
       <c r="H63" t="n">
-        <v>8.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I63" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="J63" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="K63" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L63" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1275</v>
+        <v>1400</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3232,31 +3232,31 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>27.8</v>
+        <v>43.3</v>
       </c>
       <c r="H64" t="n">
-        <v>9.6</v>
+        <v>14.2</v>
       </c>
       <c r="I64" t="n">
-        <v>1.9</v>
+        <v>4.4</v>
       </c>
       <c r="J64" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="K64" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L64" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L64" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1125</v>
+        <v>1463</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Belmont</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>25.7</v>
+        <v>28.4</v>
       </c>
       <c r="H65" t="n">
-        <v>9.6</v>
+        <v>8.6</v>
       </c>
       <c r="I65" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="J65" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3296,11 +3296,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1219</v>
+        <v>1372</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>SF Austin</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3320,19 +3320,19 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>28.9</v>
+        <v>16.7</v>
       </c>
       <c r="H66" t="n">
-        <v>7</v>
+        <v>5.4</v>
       </c>
       <c r="I66" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="J66" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K66" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3340,11 +3340,11 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1298</v>
+        <v>1414</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Navy</t>
+          <t>UC Irvine</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3364,13 +3364,13 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>23.4</v>
+        <v>10.5</v>
       </c>
       <c r="H67" t="n">
-        <v>6</v>
+        <v>2.3</v>
       </c>
       <c r="I67" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="J67" t="n">
         <v>0.1</v>
@@ -3384,11 +3384,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1190</v>
+        <v>1340</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ETSU</t>
+          <t>Portland St</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3408,10 +3408,10 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>6.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H68" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="I68" t="n">
         <v>0.1</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1398</v>
+        <v>1420</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="H69" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="I69" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-07)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.90000000000001</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>82.5</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>61</v>
+        <v>62.4</v>
       </c>
       <c r="J2" t="n">
-        <v>43.4</v>
+        <v>46.9</v>
       </c>
       <c r="K2" t="n">
-        <v>30.3</v>
+        <v>33.5</v>
       </c>
       <c r="L2" t="n">
-        <v>18.9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>89.7</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>66.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>37</v>
+        <v>37.8</v>
       </c>
       <c r="J3" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="K3" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="L3" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>89.59999999999999</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>66.90000000000001</v>
+        <v>62.6</v>
       </c>
       <c r="I4" t="n">
-        <v>40.8</v>
+        <v>38.4</v>
       </c>
       <c r="J4" t="n">
-        <v>17.5</v>
+        <v>15.8</v>
       </c>
       <c r="K4" t="n">
-        <v>9.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="L4" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="5">
@@ -636,19 +636,19 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>76.5</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>45.3</v>
+        <v>46.5</v>
       </c>
       <c r="I5" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="J5" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="L5" t="n">
         <v>1.8</v>
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>80.09999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="H6" t="n">
-        <v>42.3</v>
+        <v>40.6</v>
       </c>
       <c r="I6" t="n">
-        <v>11.6</v>
+        <v>10.3</v>
       </c>
       <c r="J6" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
       <c r="K6" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7">
@@ -724,19 +724,19 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>59.4</v>
+        <v>63.2</v>
       </c>
       <c r="H7" t="n">
-        <v>20.2</v>
+        <v>24</v>
       </c>
       <c r="I7" t="n">
-        <v>8.199999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="K7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="L7" t="n">
         <v>0.2</v>
@@ -768,16 +768,16 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>56.7</v>
+        <v>56.5</v>
       </c>
       <c r="H8" t="n">
-        <v>19.3</v>
+        <v>19.6</v>
       </c>
       <c r="I8" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="J8" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="K8" t="n">
         <v>0.4</v>
@@ -812,19 +812,19 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>56.2</v>
+        <v>56.8</v>
       </c>
       <c r="H9" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
       <c r="I9" t="n">
-        <v>4.7</v>
+        <v>3.9</v>
       </c>
       <c r="J9" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="K9" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L9" t="n">
         <v>0.2</v>
@@ -856,19 +856,19 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>43.8</v>
+        <v>43.2</v>
       </c>
       <c r="H10" t="n">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="I10" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L10" t="n">
         <v>0.1</v>
@@ -900,13 +900,13 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>43.3</v>
+        <v>43.5</v>
       </c>
       <c r="H11" t="n">
-        <v>12.5</v>
+        <v>12.9</v>
       </c>
       <c r="I11" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="J11" t="n">
         <v>0.7</v>
@@ -915,7 +915,7 @@
         <v>0.1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -941,19 +941,19 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>47.6</v>
+        <v>46.5</v>
       </c>
       <c r="G12" t="n">
-        <v>18.2</v>
+        <v>16.6</v>
       </c>
       <c r="H12" t="n">
-        <v>5.3</v>
+        <v>4.9</v>
       </c>
       <c r="I12" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K12" t="n">
         <v>0.1</v>
@@ -985,19 +985,19 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>52.4</v>
+        <v>53.5</v>
       </c>
       <c r="G13" t="n">
-        <v>22.4</v>
+        <v>20.2</v>
       </c>
       <c r="H13" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="I13" t="n">
         <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K13" t="n">
         <v>0.1</v>
@@ -1032,16 +1032,16 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>19.9</v>
+        <v>23.5</v>
       </c>
       <c r="H14" t="n">
-        <v>6.9</v>
+        <v>7.3</v>
       </c>
       <c r="I14" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1076,16 +1076,16 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="H15" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1120,10 +1120,10 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>10.4</v>
+        <v>11.9</v>
       </c>
       <c r="H16" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="I16" t="n">
         <v>0.4</v>
@@ -1164,10 +1164,10 @@
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="I17" t="n">
         <v>0.2</v>
@@ -1208,13 +1208,13 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>1.1</v>
+        <v>4.1</v>
       </c>
       <c r="H18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I18" t="n">
         <v>0.1</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>91.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="H19" t="n">
-        <v>62.6</v>
+        <v>62.2</v>
       </c>
       <c r="I19" t="n">
-        <v>38.2</v>
+        <v>38.6</v>
       </c>
       <c r="J19" t="n">
-        <v>18.3</v>
+        <v>18.7</v>
       </c>
       <c r="K19" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
       <c r="L19" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H20" t="n">
-        <v>78</v>
+        <v>79.7</v>
       </c>
       <c r="I20" t="n">
-        <v>48.4</v>
+        <v>50.3</v>
       </c>
       <c r="J20" t="n">
-        <v>32.2</v>
+        <v>33.2</v>
       </c>
       <c r="K20" t="n">
-        <v>16.8</v>
+        <v>16.4</v>
       </c>
       <c r="L20" t="n">
-        <v>8.800000000000001</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>93.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>61.8</v>
+        <v>61.3</v>
       </c>
       <c r="I21" t="n">
-        <v>31.5</v>
+        <v>31.2</v>
       </c>
       <c r="J21" t="n">
-        <v>19.2</v>
+        <v>18.5</v>
       </c>
       <c r="K21" t="n">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="L21" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="22">
@@ -1384,22 +1384,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>90.59999999999999</v>
+        <v>92.3</v>
       </c>
       <c r="H22" t="n">
-        <v>45.3</v>
+        <v>46.5</v>
       </c>
       <c r="I22" t="n">
-        <v>19.6</v>
+        <v>19.4</v>
       </c>
       <c r="J22" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="23">
@@ -1428,22 +1428,22 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>84.40000000000001</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="H23" t="n">
-        <v>50.3</v>
+        <v>49</v>
       </c>
       <c r="I23" t="n">
-        <v>25.7</v>
+        <v>25</v>
       </c>
       <c r="J23" t="n">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="K23" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="L23" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="24">
@@ -1472,19 +1472,19 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>68.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="H24" t="n">
-        <v>27.6</v>
+        <v>27.3</v>
       </c>
       <c r="I24" t="n">
-        <v>10.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
       <c r="K24" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="L24" t="n">
         <v>0.4</v>
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>47.7</v>
+        <v>46.7</v>
       </c>
       <c r="H25" t="n">
-        <v>9.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I25" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="J25" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="K25" t="n">
         <v>0.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1560,22 +1560,22 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>45.1</v>
+        <v>44.3</v>
       </c>
       <c r="H26" t="n">
-        <v>15.3</v>
+        <v>14.8</v>
       </c>
       <c r="I26" t="n">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="J26" t="n">
         <v>1.7</v>
       </c>
       <c r="K26" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="27">
@@ -1604,22 +1604,22 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>54.9</v>
+        <v>55.7</v>
       </c>
       <c r="H27" t="n">
-        <v>21.2</v>
+        <v>22.1</v>
       </c>
       <c r="I27" t="n">
-        <v>8.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J27" t="n">
         <v>3.3</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="L27" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="28">
@@ -1648,13 +1648,13 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>52.3</v>
+        <v>53.3</v>
       </c>
       <c r="H28" t="n">
-        <v>11.6</v>
+        <v>11.2</v>
       </c>
       <c r="I28" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="J28" t="n">
         <v>1.2</v>
@@ -1689,22 +1689,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>56.1</v>
+        <v>56.6</v>
       </c>
       <c r="G29" t="n">
-        <v>18.5</v>
+        <v>20.3</v>
       </c>
       <c r="H29" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="I29" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="J29" t="n">
         <v>0.6</v>
       </c>
       <c r="K29" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -1733,13 +1733,13 @@
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>43.9</v>
+        <v>43.4</v>
       </c>
       <c r="G30" t="n">
-        <v>13.1</v>
+        <v>12.4</v>
       </c>
       <c r="H30" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="I30" t="n">
         <v>0.6</v>
@@ -1780,13 +1780,13 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>15.6</v>
+        <v>16.9</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="I31" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J31" t="n">
         <v>0.1</v>
@@ -1824,16 +1824,16 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>9.4</v>
+        <v>7.7</v>
       </c>
       <c r="H32" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="I32" t="n">
         <v>0.2</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>6.9</v>
+        <v>7.6</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -1912,16 +1912,16 @@
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="H34" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I34" t="n">
         <v>0.1</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>60</v>
+        <v>58.5</v>
       </c>
       <c r="G35" t="n">
-        <v>6.2</v>
+        <v>6.8</v>
       </c>
       <c r="H35" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="I35" t="n">
         <v>0.1</v>
@@ -1997,7 +1997,7 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>40</v>
+        <v>41.5</v>
       </c>
       <c r="G36" t="n">
         <v>2.4</v>
@@ -2047,19 +2047,19 @@
         <v>95.59999999999999</v>
       </c>
       <c r="H37" t="n">
-        <v>80</v>
+        <v>80.2</v>
       </c>
       <c r="I37" t="n">
-        <v>59.1</v>
+        <v>60.7</v>
       </c>
       <c r="J37" t="n">
-        <v>38.5</v>
+        <v>40.3</v>
       </c>
       <c r="K37" t="n">
-        <v>22.4</v>
+        <v>23.2</v>
       </c>
       <c r="L37" t="n">
-        <v>12.4</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="38">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>93.5</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>67.40000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="I38" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="J38" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="K38" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="L38" t="n">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="39">
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>88</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>47.9</v>
+        <v>47.8</v>
       </c>
       <c r="I39" t="n">
-        <v>19.1</v>
+        <v>19.3</v>
       </c>
       <c r="J39" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="K39" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="L39" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>81</v>
+        <v>77.3</v>
       </c>
       <c r="H40" t="n">
-        <v>45</v>
+        <v>41.9</v>
       </c>
       <c r="I40" t="n">
-        <v>15.7</v>
+        <v>13.6</v>
       </c>
       <c r="J40" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="K40" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="L40" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="41">
@@ -2220,19 +2220,19 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>68.40000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="H41" t="n">
-        <v>39</v>
+        <v>42.2</v>
       </c>
       <c r="I41" t="n">
-        <v>13.6</v>
+        <v>14.8</v>
       </c>
       <c r="J41" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="K41" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="L41" t="n">
         <v>0.8</v>
@@ -2264,7 +2264,7 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>72.2</v>
+        <v>75.3</v>
       </c>
       <c r="H42" t="n">
         <v>44.1</v>
@@ -2273,13 +2273,13 @@
         <v>18.6</v>
       </c>
       <c r="J42" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="K42" t="n">
         <v>2.9</v>
       </c>
       <c r="L42" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="43">
@@ -2308,22 +2308,22 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>63.4</v>
+        <v>59.3</v>
       </c>
       <c r="H43" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="I43" t="n">
-        <v>10.2</v>
+        <v>9.9</v>
       </c>
       <c r="J43" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K43" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L43" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="44">
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>54.2</v>
+        <v>52.8</v>
       </c>
       <c r="H44" t="n">
-        <v>9.4</v>
+        <v>10</v>
       </c>
       <c r="I44" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="J44" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
@@ -2396,19 +2396,19 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>45.8</v>
+        <v>47.2</v>
       </c>
       <c r="H45" t="n">
-        <v>10.2</v>
+        <v>9.5</v>
       </c>
       <c r="I45" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="J45" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K45" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L45" t="n">
         <v>0</v>
@@ -2440,16 +2440,16 @@
         <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>36.5</v>
+        <v>40.7</v>
       </c>
       <c r="H46" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="I46" t="n">
         <v>4.9</v>
       </c>
       <c r="J46" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="K46" t="n">
         <v>0.4</v>
@@ -2484,13 +2484,13 @@
         <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>27.8</v>
+        <v>24.6</v>
       </c>
       <c r="H47" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
       <c r="I47" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="J47" t="n">
         <v>0.2</v>
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>31.6</v>
+        <v>27.5</v>
       </c>
       <c r="H48" t="n">
-        <v>11.9</v>
+        <v>10.5</v>
       </c>
       <c r="I48" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="J48" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K48" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2572,13 +2572,13 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>19</v>
+        <v>22.7</v>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="I49" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="J49" t="n">
         <v>0.1</v>
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>12</v>
+        <v>10.4</v>
       </c>
       <c r="H50" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I50" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2660,10 +2660,10 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>6.5</v>
+        <v>4.6</v>
       </c>
       <c r="H51" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="I51" t="n">
         <v>0.1</v>
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>56.2</v>
+        <v>57.4</v>
       </c>
       <c r="G52" t="n">
-        <v>3.9</v>
+        <v>2.8</v>
       </c>
       <c r="H52" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2745,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>43.8</v>
+        <v>42.6</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>93.59999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="H54" t="n">
-        <v>72.90000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="I54" t="n">
-        <v>56.6</v>
+        <v>56.9</v>
       </c>
       <c r="J54" t="n">
-        <v>38.9</v>
+        <v>38.7</v>
       </c>
       <c r="K54" t="n">
-        <v>24.1</v>
+        <v>24.3</v>
       </c>
       <c r="L54" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="55">
@@ -2836,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>91.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>68.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="I55" t="n">
-        <v>42.4</v>
+        <v>43.6</v>
       </c>
       <c r="J55" t="n">
-        <v>21.6</v>
+        <v>21.3</v>
       </c>
       <c r="K55" t="n">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="L55" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="56">
@@ -2880,22 +2880,22 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>89.5</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>62.6</v>
+        <v>60.9</v>
       </c>
       <c r="I56" t="n">
-        <v>32.5</v>
+        <v>31.6</v>
       </c>
       <c r="J56" t="n">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="K56" t="n">
-        <v>7.5</v>
+        <v>7.2</v>
       </c>
       <c r="L56" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>76.3</v>
+        <v>74</v>
       </c>
       <c r="H57" t="n">
-        <v>48.7</v>
+        <v>49.5</v>
       </c>
       <c r="I57" t="n">
-        <v>18.4</v>
+        <v>18</v>
       </c>
       <c r="J57" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="K57" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="L57" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="58">
@@ -2968,13 +2968,13 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>72.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>36.7</v>
+        <v>33.8</v>
       </c>
       <c r="I58" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="J58" t="n">
         <v>3.7</v>
@@ -3012,16 +3012,16 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>56.7</v>
+        <v>57.1</v>
       </c>
       <c r="H59" t="n">
-        <v>20.9</v>
+        <v>22.9</v>
       </c>
       <c r="I59" t="n">
-        <v>7.4</v>
+        <v>8</v>
       </c>
       <c r="J59" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="K59" t="n">
         <v>0.8</v>
@@ -3056,22 +3056,22 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>63.4</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="H60" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="I60" t="n">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="J60" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="K60" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L60" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="61">
@@ -3100,22 +3100,22 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>55</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="H61" t="n">
-        <v>15.5</v>
+        <v>17.6</v>
       </c>
       <c r="I61" t="n">
-        <v>7.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J61" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="K61" t="n">
         <v>0.9</v>
       </c>
       <c r="L61" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="62">
@@ -3144,22 +3144,22 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>45</v>
+        <v>34.9</v>
       </c>
       <c r="H62" t="n">
-        <v>10.7</v>
+        <v>7.5</v>
       </c>
       <c r="I62" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="J62" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="K62" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L62" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -3188,19 +3188,19 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>36.6</v>
+        <v>34.4</v>
       </c>
       <c r="H63" t="n">
-        <v>9.300000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="I63" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="J63" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="K63" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
@@ -3232,13 +3232,13 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>43.3</v>
+        <v>42.9</v>
       </c>
       <c r="H64" t="n">
-        <v>14.2</v>
+        <v>13.7</v>
       </c>
       <c r="I64" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="J64" t="n">
         <v>1.3</v>
@@ -3276,19 +3276,19 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>27.2</v>
+        <v>28.1</v>
       </c>
       <c r="H65" t="n">
-        <v>8.800000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="I65" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="J65" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K65" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
@@ -3320,13 +3320,13 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>23.7</v>
+        <v>26</v>
       </c>
       <c r="H66" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="J66" t="n">
         <v>0.2</v>
@@ -3364,13 +3364,13 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>10.5</v>
+        <v>11.9</v>
       </c>
       <c r="H67" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J67" t="n">
         <v>0.1</v>
@@ -3408,13 +3408,13 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>8.199999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="H68" t="n">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>6.4</v>
+        <v>5.2</v>
       </c>
       <c r="H69" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="I69" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-08)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>95.90000000000001</v>
+        <v>96.8</v>
       </c>
       <c r="H2" t="n">
-        <v>83.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="I2" t="n">
-        <v>62.4</v>
+        <v>60.4</v>
       </c>
       <c r="J2" t="n">
-        <v>46.9</v>
+        <v>45.1</v>
       </c>
       <c r="K2" t="n">
-        <v>33.5</v>
+        <v>31.8</v>
       </c>
       <c r="L2" t="n">
-        <v>21</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="3">
@@ -551,19 +551,19 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>65.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>37.8</v>
+        <v>37.4</v>
       </c>
       <c r="J3" t="n">
-        <v>16</v>
+        <v>15.7</v>
       </c>
       <c r="K3" t="n">
-        <v>8.5</v>
+        <v>8.1</v>
       </c>
       <c r="L3" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="4">
@@ -595,16 +595,16 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>62.6</v>
+        <v>61.7</v>
       </c>
       <c r="I4" t="n">
-        <v>38.4</v>
+        <v>38.3</v>
       </c>
       <c r="J4" t="n">
-        <v>15.8</v>
+        <v>16.1</v>
       </c>
       <c r="K4" t="n">
-        <v>8.1</v>
+        <v>8.4</v>
       </c>
       <c r="L4" t="n">
         <v>3.9</v>
@@ -642,16 +642,16 @@
         <v>46.5</v>
       </c>
       <c r="I5" t="n">
-        <v>18.9</v>
+        <v>19.9</v>
       </c>
       <c r="J5" t="n">
-        <v>9.199999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="K5" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="L5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -683,10 +683,10 @@
         <v>76.5</v>
       </c>
       <c r="H6" t="n">
-        <v>40.6</v>
+        <v>41</v>
       </c>
       <c r="I6" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="J6" t="n">
         <v>4.3</v>
@@ -695,16 +695,16 @@
         <v>1.8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1246</v>
+        <v>1458</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -724,31 +724,31 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>63.2</v>
+        <v>59.6</v>
       </c>
       <c r="H7" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="I7" t="n">
-        <v>9.800000000000001</v>
+        <v>10.4</v>
       </c>
       <c r="J7" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="K7" t="n">
         <v>0.9</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1274</v>
+        <v>1437</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -768,19 +768,19 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>56.5</v>
+        <v>58.4</v>
       </c>
       <c r="H8" t="n">
-        <v>19.6</v>
+        <v>17.9</v>
       </c>
       <c r="I8" t="n">
-        <v>6.3</v>
+        <v>5.7</v>
       </c>
       <c r="J8" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L8" t="n">
         <v>0.1</v>
@@ -812,31 +812,31 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>56.8</v>
+        <v>47</v>
       </c>
       <c r="H9" t="n">
-        <v>9.6</v>
+        <v>7.9</v>
       </c>
       <c r="I9" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="J9" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1417</v>
+        <v>1234</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -856,19 +856,19 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>43.2</v>
+        <v>53</v>
       </c>
       <c r="H10" t="n">
-        <v>6.3</v>
+        <v>10.5</v>
       </c>
       <c r="I10" t="n">
-        <v>2.5</v>
+        <v>4.6</v>
       </c>
       <c r="J10" t="n">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="L10" t="n">
         <v>0.1</v>
@@ -900,13 +900,13 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>43.5</v>
+        <v>41.6</v>
       </c>
       <c r="H11" t="n">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="I11" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="J11" t="n">
         <v>0.7</v>
@@ -920,11 +920,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1374</v>
+        <v>1365</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -941,19 +941,19 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>46.5</v>
+        <v>53.1</v>
       </c>
       <c r="G12" t="n">
-        <v>16.6</v>
+        <v>22.6</v>
       </c>
       <c r="H12" t="n">
-        <v>4.9</v>
+        <v>7.4</v>
       </c>
       <c r="I12" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="K12" t="n">
         <v>0.1</v>
@@ -964,11 +964,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1231</v>
+        <v>1374</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -985,19 +985,19 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>53.5</v>
+        <v>46.9</v>
       </c>
       <c r="G13" t="n">
-        <v>20.2</v>
+        <v>17.8</v>
       </c>
       <c r="H13" t="n">
-        <v>6.2</v>
+        <v>5.1</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="J13" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K13" t="n">
         <v>0.1</v>
@@ -1035,10 +1035,10 @@
         <v>23.5</v>
       </c>
       <c r="H14" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="I14" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0.2</v>
@@ -1052,11 +1052,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1423</v>
+        <v>1372</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UNC Wilmington</t>
+          <t>SF Austin</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1079,13 +1079,13 @@
         <v>23.6</v>
       </c>
       <c r="H15" t="n">
-        <v>5.7</v>
+        <v>4.9</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1123,13 +1123,13 @@
         <v>11.9</v>
       </c>
       <c r="H16" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
         <v>11.8</v>
       </c>
       <c r="H17" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="I17" t="n">
         <v>0.2</v>
@@ -1184,11 +1184,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1146</v>
+        <v>1398</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cent Arkansas</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1208,7 +1208,7 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="n">
         <v>0.3</v>
@@ -1228,11 +1228,11 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1163</v>
+        <v>1196</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1252,31 +1252,31 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>90.8</v>
+        <v>96.8</v>
       </c>
       <c r="H19" t="n">
-        <v>62.2</v>
+        <v>76.5</v>
       </c>
       <c r="I19" t="n">
-        <v>38.6</v>
+        <v>56.7</v>
       </c>
       <c r="J19" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="K19" t="n">
         <v>18.7</v>
       </c>
-      <c r="K19" t="n">
-        <v>7.9</v>
-      </c>
       <c r="L19" t="n">
-        <v>3.1</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1196</v>
+        <v>1222</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1296,31 +1296,31 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>95</v>
+        <v>95.2</v>
       </c>
       <c r="H20" t="n">
-        <v>79.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>50.3</v>
+        <v>47</v>
       </c>
       <c r="J20" t="n">
-        <v>33.2</v>
+        <v>26.3</v>
       </c>
       <c r="K20" t="n">
-        <v>16.4</v>
+        <v>12.6</v>
       </c>
       <c r="L20" t="n">
-        <v>8.4</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1345</v>
+        <v>1304</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1343,28 +1343,28 @@
         <v>92.40000000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>61.3</v>
+        <v>47.7</v>
       </c>
       <c r="I21" t="n">
-        <v>31.2</v>
+        <v>19.1</v>
       </c>
       <c r="J21" t="n">
-        <v>18.5</v>
+        <v>7.3</v>
       </c>
       <c r="K21" t="n">
-        <v>8.6</v>
+        <v>2.2</v>
       </c>
       <c r="L21" t="n">
-        <v>3.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1438</v>
+        <v>1242</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1384,31 +1384,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>92.3</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>46.5</v>
+        <v>41.2</v>
       </c>
       <c r="I22" t="n">
-        <v>19.4</v>
+        <v>13.7</v>
       </c>
       <c r="J22" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="K22" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="L22" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1397</v>
+        <v>1116</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1428,22 +1428,22 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>83.09999999999999</v>
+        <v>72</v>
       </c>
       <c r="H23" t="n">
-        <v>49</v>
+        <v>42.2</v>
       </c>
       <c r="I23" t="n">
-        <v>25</v>
+        <v>17.1</v>
       </c>
       <c r="J23" t="n">
-        <v>10.2</v>
+        <v>7.7</v>
       </c>
       <c r="K23" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="L23" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1472,31 +1472,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>67.3</v>
+        <v>71.2</v>
       </c>
       <c r="H24" t="n">
-        <v>27.3</v>
+        <v>40.6</v>
       </c>
       <c r="I24" t="n">
-        <v>9.300000000000001</v>
+        <v>16.8</v>
       </c>
       <c r="J24" t="n">
-        <v>4.3</v>
+        <v>6.5</v>
       </c>
       <c r="K24" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1437</v>
+        <v>1388</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1516,31 +1516,31 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>46.7</v>
+        <v>66.5</v>
       </c>
       <c r="H25" t="n">
-        <v>8.300000000000001</v>
+        <v>23.1</v>
       </c>
       <c r="I25" t="n">
-        <v>2.8</v>
+        <v>11</v>
       </c>
       <c r="J25" t="n">
-        <v>0.9</v>
+        <v>4.3</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1387</v>
+        <v>1274</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1560,31 +1560,31 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>44.3</v>
+        <v>43.3</v>
       </c>
       <c r="H26" t="n">
-        <v>14.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I26" t="n">
-        <v>6.3</v>
+        <v>3.5</v>
       </c>
       <c r="J26" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1234</v>
+        <v>1326</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Ohio St</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1604,19 +1604,19 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>55.7</v>
+        <v>56.7</v>
       </c>
       <c r="H27" t="n">
-        <v>22.1</v>
+        <v>14.6</v>
       </c>
       <c r="I27" t="n">
-        <v>9.699999999999999</v>
+        <v>5.7</v>
       </c>
       <c r="J27" t="n">
-        <v>3.3</v>
+        <v>2</v>
       </c>
       <c r="K27" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="L27" t="n">
         <v>0.2</v>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1648,16 +1648,16 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>53.3</v>
+        <v>33.5</v>
       </c>
       <c r="H28" t="n">
-        <v>11.2</v>
+        <v>9</v>
       </c>
       <c r="I28" t="n">
         <v>3.7</v>
       </c>
       <c r="J28" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K28" t="n">
         <v>0.3</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1365</v>
+        <v>1416</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1682,26 +1682,26 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>56.6</v>
+        <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>20.3</v>
+        <v>28.8</v>
       </c>
       <c r="H29" t="n">
-        <v>7.4</v>
+        <v>10.9</v>
       </c>
       <c r="I29" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="J29" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="K29" t="n">
         <v>0.1</v>
@@ -1712,11 +1712,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1307</v>
+        <v>1378</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1726,29 +1726,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>43.4</v>
+        <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>12.4</v>
+        <v>28</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>10.4</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6</v>
+        <v>2.5</v>
       </c>
       <c r="J30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K30" t="n">
         <v>0.1</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -1756,11 +1756,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1372</v>
+        <v>1423</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SF Austin</t>
+          <t>UNC Wilmington</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E31" t="b">
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>16.9</v>
+        <v>23.1</v>
       </c>
       <c r="H31" t="n">
-        <v>3.3</v>
+        <v>6.2</v>
       </c>
       <c r="I31" t="n">
         <v>0.8</v>
       </c>
       <c r="J31" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1800,11 +1800,11 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1295</v>
+        <v>1190</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>ETSU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E32" t="b">
@@ -1824,16 +1824,16 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="H32" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1133</v>
+        <v>1146</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bradley</t>
+          <t>Cent Arkansas</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -1868,10 +1868,10 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>7.6</v>
+        <v>4.8</v>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I33" t="n">
         <v>0.1</v>
@@ -1888,11 +1888,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1467</v>
+        <v>1224</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Merrimack</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1902,26 +1902,26 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>100</v>
+        <v>57.2</v>
       </c>
       <c r="G34" t="n">
-        <v>5.1</v>
+        <v>2.7</v>
       </c>
       <c r="H34" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1398</v>
+        <v>1126</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>Bethune-Cookman</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1946,23 +1946,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>58.5</v>
+        <v>42.8</v>
       </c>
       <c r="G35" t="n">
-        <v>6.8</v>
+        <v>0.5</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1976,55 +1976,55 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1254</v>
+        <v>1276</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>41.5</v>
+        <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>2.4</v>
+        <v>95.5</v>
       </c>
       <c r="H36" t="n">
-        <v>0.2</v>
+        <v>76</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>55.6</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>39.2</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>22.6</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1276</v>
+        <v>1163</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E37" t="b">
@@ -2044,31 +2044,31 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>95.59999999999999</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>80.2</v>
+        <v>60.8</v>
       </c>
       <c r="I37" t="n">
-        <v>60.7</v>
+        <v>31.3</v>
       </c>
       <c r="J37" t="n">
-        <v>40.2</v>
+        <v>13.2</v>
       </c>
       <c r="K37" t="n">
-        <v>23.2</v>
+        <v>5</v>
       </c>
       <c r="L37" t="n">
-        <v>13.3</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1222</v>
+        <v>1345</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E38" t="b">
@@ -2088,31 +2088,31 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>95.40000000000001</v>
+        <v>92</v>
       </c>
       <c r="H38" t="n">
-        <v>67.59999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="I38" t="n">
-        <v>45.5</v>
+        <v>41.8</v>
       </c>
       <c r="J38" t="n">
-        <v>24.5</v>
+        <v>19.1</v>
       </c>
       <c r="K38" t="n">
-        <v>13.4</v>
+        <v>9</v>
       </c>
       <c r="L38" t="n">
-        <v>6.6</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1304</v>
+        <v>1438</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E39" t="b">
@@ -2132,31 +2132,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>89.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="H39" t="n">
-        <v>48.7</v>
+        <v>48</v>
       </c>
       <c r="I39" t="n">
-        <v>19.8</v>
+        <v>17.5</v>
       </c>
       <c r="J39" t="n">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K39" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="L39" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1242</v>
+        <v>1397</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E40" t="b">
@@ -2176,31 +2176,31 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>77.3</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H40" t="n">
-        <v>41.9</v>
+        <v>48</v>
       </c>
       <c r="I40" t="n">
-        <v>13.6</v>
+        <v>17.6</v>
       </c>
       <c r="J40" t="n">
-        <v>5.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K40" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="L40" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1116</v>
+        <v>1314</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E41" t="b">
@@ -2220,31 +2220,31 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>72.5</v>
+        <v>60.6</v>
       </c>
       <c r="H41" t="n">
-        <v>42.2</v>
+        <v>19.5</v>
       </c>
       <c r="I41" t="n">
-        <v>14.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J41" t="n">
-        <v>6.5</v>
+        <v>3.2</v>
       </c>
       <c r="K41" t="n">
-        <v>2.4</v>
+        <v>1.1</v>
       </c>
       <c r="L41" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1435</v>
+        <v>1208</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E42" t="b">
@@ -2264,31 +2264,31 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>75.3</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>44.1</v>
+        <v>25.9</v>
       </c>
       <c r="I42" t="n">
-        <v>18.6</v>
+        <v>9.9</v>
       </c>
       <c r="J42" t="n">
-        <v>7.9</v>
+        <v>2.9</v>
       </c>
       <c r="K42" t="n">
-        <v>2.9</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E43" t="b">
@@ -2308,31 +2308,31 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>59.3</v>
+        <v>55</v>
       </c>
       <c r="H43" t="n">
-        <v>20.2</v>
+        <v>13.6</v>
       </c>
       <c r="I43" t="n">
-        <v>9.800000000000001</v>
+        <v>5.3</v>
       </c>
       <c r="J43" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="K43" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
       <c r="L43" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1155</v>
+        <v>1395</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E44" t="b">
@@ -2352,31 +2352,31 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="H44" t="n">
-        <v>10.3</v>
+        <v>10</v>
       </c>
       <c r="I44" t="n">
-        <v>4.4</v>
+        <v>3.5</v>
       </c>
       <c r="J44" t="n">
         <v>1.1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1416</v>
+        <v>1301</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E45" t="b">
@@ -2396,13 +2396,13 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="H45" t="n">
-        <v>9.1</v>
+        <v>11.4</v>
       </c>
       <c r="I45" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="J45" t="n">
         <v>0.9</v>
@@ -2416,11 +2416,11 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1326</v>
+        <v>1433</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ohio St</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2430,41 +2430,41 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>100</v>
+        <v>45.1</v>
       </c>
       <c r="G46" t="n">
-        <v>40.7</v>
+        <v>15.2</v>
       </c>
       <c r="H46" t="n">
-        <v>11.6</v>
+        <v>4.8</v>
       </c>
       <c r="I46" t="n">
-        <v>4.9</v>
+        <v>1.6</v>
       </c>
       <c r="J46" t="n">
-        <v>1.6</v>
+        <v>0.3</v>
       </c>
       <c r="K46" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1275</v>
+        <v>1120</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2474,41 +2474,41 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>100</v>
+        <v>54.9</v>
       </c>
       <c r="G47" t="n">
-        <v>24.6</v>
+        <v>24.2</v>
       </c>
       <c r="H47" t="n">
-        <v>5.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>1.2</v>
+        <v>3.4</v>
       </c>
       <c r="J47" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1378</v>
+        <v>1251</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>Liberty</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>27.5</v>
+        <v>16.4</v>
       </c>
       <c r="H48" t="n">
-        <v>10.5</v>
+        <v>2.9</v>
       </c>
       <c r="I48" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
       <c r="J48" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1251</v>
+        <v>1295</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2572,16 +2572,16 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>22.7</v>
+        <v>7.8</v>
       </c>
       <c r="H49" t="n">
-        <v>5.4</v>
+        <v>1.1</v>
       </c>
       <c r="I49" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2616,10 +2616,10 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>10.4</v>
+        <v>8.1</v>
       </c>
       <c r="H50" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
         <v>0.1</v>
@@ -2636,11 +2636,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1190</v>
+        <v>1467</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ETSU</t>
+          <t>Merrimack</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2660,13 +2660,13 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>4.6</v>
+        <v>11.6</v>
       </c>
       <c r="H51" t="n">
-        <v>0.5</v>
+        <v>1.8</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2680,11 +2680,11 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1224</v>
+        <v>1420</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>57.4</v>
+        <v>48.5</v>
       </c>
       <c r="G52" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2724,11 +2724,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1126</v>
+        <v>1254</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Bethune-Cookman</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2745,10 +2745,10 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>42.6</v>
+        <v>51.5</v>
       </c>
       <c r="G53" t="n">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="H53" t="n">
         <v>0.1</v>
@@ -2795,19 +2795,19 @@
         <v>94.8</v>
       </c>
       <c r="H54" t="n">
-        <v>74.2</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>56.9</v>
+        <v>57.6</v>
       </c>
       <c r="J54" t="n">
-        <v>38.7</v>
+        <v>39.3</v>
       </c>
       <c r="K54" t="n">
-        <v>24.3</v>
+        <v>25.6</v>
       </c>
       <c r="L54" t="n">
-        <v>16.1</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="55">
@@ -2836,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>94.09999999999999</v>
+        <v>92.5</v>
       </c>
       <c r="H55" t="n">
-        <v>69.2</v>
+        <v>66</v>
       </c>
       <c r="I55" t="n">
-        <v>43.6</v>
+        <v>41.3</v>
       </c>
       <c r="J55" t="n">
-        <v>21.3</v>
+        <v>19.8</v>
       </c>
       <c r="K55" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="L55" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
@@ -2883,19 +2883,19 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>60.9</v>
+        <v>64</v>
       </c>
       <c r="I56" t="n">
-        <v>31.6</v>
+        <v>32.4</v>
       </c>
       <c r="J56" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="K56" t="n">
         <v>7.3</v>
       </c>
       <c r="L56" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="57">
@@ -2927,16 +2927,16 @@
         <v>74</v>
       </c>
       <c r="H57" t="n">
-        <v>49.5</v>
+        <v>44.9</v>
       </c>
       <c r="I57" t="n">
-        <v>18</v>
+        <v>16.2</v>
       </c>
       <c r="J57" t="n">
-        <v>8.9</v>
+        <v>8</v>
       </c>
       <c r="K57" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="L57" t="n">
         <v>1.4</v>
@@ -2944,11 +2944,11 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1314</v>
+        <v>1435</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2968,31 +2968,31 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>71.90000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>33.8</v>
+        <v>40.7</v>
       </c>
       <c r="I58" t="n">
-        <v>10.2</v>
+        <v>14.5</v>
       </c>
       <c r="J58" t="n">
-        <v>3.7</v>
+        <v>6.5</v>
       </c>
       <c r="K58" t="n">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="L58" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1458</v>
+        <v>1246</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3012,22 +3012,22 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>57.1</v>
+        <v>73.3</v>
       </c>
       <c r="H59" t="n">
-        <v>22.9</v>
+        <v>26.8</v>
       </c>
       <c r="I59" t="n">
-        <v>8</v>
+        <v>9.1</v>
       </c>
       <c r="J59" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="K59" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L59" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="60">
@@ -3059,28 +3059,28 @@
         <v>65.59999999999999</v>
       </c>
       <c r="H60" t="n">
-        <v>20.5</v>
+        <v>22.8</v>
       </c>
       <c r="I60" t="n">
-        <v>8.9</v>
+        <v>11.2</v>
       </c>
       <c r="J60" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="K60" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="L60" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1208</v>
+        <v>1155</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3100,31 +3100,31 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>65.09999999999999</v>
+        <v>42</v>
       </c>
       <c r="H61" t="n">
-        <v>17.6</v>
+        <v>9.6</v>
       </c>
       <c r="I61" t="n">
-        <v>8.300000000000001</v>
+        <v>3.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3</v>
+        <v>0.9</v>
       </c>
       <c r="K61" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="L61" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1301</v>
+        <v>1417</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3144,31 +3144,31 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>34.9</v>
+        <v>58</v>
       </c>
       <c r="H62" t="n">
-        <v>7.5</v>
+        <v>13.9</v>
       </c>
       <c r="I62" t="n">
-        <v>3</v>
+        <v>5.8</v>
       </c>
       <c r="J62" t="n">
-        <v>0.9</v>
+        <v>2.1</v>
       </c>
       <c r="K62" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L62" t="n">
         <v>0.2</v>
-      </c>
-      <c r="L62" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1395</v>
+        <v>1401</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3191,16 +3191,16 @@
         <v>34.4</v>
       </c>
       <c r="H63" t="n">
-        <v>9.5</v>
+        <v>9.6</v>
       </c>
       <c r="I63" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="J63" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="K63" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
@@ -3208,11 +3208,11 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1400</v>
+        <v>1275</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3232,22 +3232,22 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>42.9</v>
+        <v>26.7</v>
       </c>
       <c r="H64" t="n">
-        <v>13.7</v>
+        <v>5.2</v>
       </c>
       <c r="I64" t="n">
-        <v>4.2</v>
+        <v>1.1</v>
       </c>
       <c r="J64" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="K64" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>28.1</v>
+        <v>23.9</v>
       </c>
       <c r="H65" t="n">
-        <v>10.4</v>
+        <v>7.7</v>
       </c>
       <c r="I65" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="J65" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3323,7 +3323,7 @@
         <v>26</v>
       </c>
       <c r="H66" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="I66" t="n">
         <v>1.1</v>
@@ -3332,7 +3332,7 @@
         <v>0.2</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3367,13 +3367,13 @@
         <v>11.9</v>
       </c>
       <c r="H67" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="I67" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3384,11 +3384,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1340</v>
+        <v>1227</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Portland St</t>
+          <t>IL Chicago</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3408,16 +3408,16 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>5.9</v>
+        <v>7.5</v>
       </c>
       <c r="H68" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1420</v>
+        <v>1340</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Portland St</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3455,10 +3455,10 @@
         <v>5.2</v>
       </c>
       <c r="H69" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="I69" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-09)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -513,13 +513,13 @@
         <v>60.9</v>
       </c>
       <c r="J2" t="n">
-        <v>45.1</v>
+        <v>45.2</v>
       </c>
       <c r="K2" t="n">
         <v>31.9</v>
       </c>
       <c r="L2" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="3">
@@ -551,16 +551,16 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>67.40000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="I3" t="n">
-        <v>36.9</v>
+        <v>37.3</v>
       </c>
       <c r="J3" t="n">
-        <v>15.7</v>
+        <v>16</v>
       </c>
       <c r="K3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="L3" t="n">
         <v>3.6</v>
@@ -598,16 +598,16 @@
         <v>64.7</v>
       </c>
       <c r="I4" t="n">
-        <v>39.8</v>
+        <v>38.8</v>
       </c>
       <c r="J4" t="n">
-        <v>16.6</v>
+        <v>16.3</v>
       </c>
       <c r="K4" t="n">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="L4" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="5">
@@ -639,16 +639,16 @@
         <v>83.2</v>
       </c>
       <c r="H5" t="n">
-        <v>47.1</v>
+        <v>46.8</v>
       </c>
       <c r="I5" t="n">
-        <v>16.1</v>
+        <v>16</v>
       </c>
       <c r="J5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="K5" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L5" t="n">
         <v>1.4</v>
@@ -689,7 +689,7 @@
         <v>13.6</v>
       </c>
       <c r="J6" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="K6" t="n">
         <v>2.5</v>
@@ -730,7 +730,7 @@
         <v>22.7</v>
       </c>
       <c r="I7" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J7" t="n">
         <v>2.5</v>
@@ -771,13 +771,13 @@
         <v>54.7</v>
       </c>
       <c r="H8" t="n">
-        <v>17.4</v>
+        <v>18.5</v>
       </c>
       <c r="I8" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="J8" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K8" t="n">
         <v>0.3</v>
@@ -821,10 +821,10 @@
         <v>4.3</v>
       </c>
       <c r="J9" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="K9" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L9" t="n">
         <v>0.1</v>
@@ -941,7 +941,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>53.1</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
         <v>22.6</v>
@@ -994,10 +994,10 @@
         <v>4.9</v>
       </c>
       <c r="I13" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K13" t="n">
         <v>0.1</v>
@@ -1035,7 +1035,7 @@
         <v>27.7</v>
       </c>
       <c r="H14" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="I14" t="n">
         <v>1.5</v>
@@ -1261,13 +1261,13 @@
         <v>59.2</v>
       </c>
       <c r="J19" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="K19" t="n">
         <v>19.4</v>
       </c>
       <c r="L19" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1302,16 +1302,16 @@
         <v>68.90000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>48.1</v>
+        <v>47.4</v>
       </c>
       <c r="J20" t="n">
-        <v>26.8</v>
+        <v>26.3</v>
       </c>
       <c r="K20" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="L20" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>77</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>41.1</v>
+        <v>44</v>
       </c>
       <c r="I21" t="n">
-        <v>16.6</v>
+        <v>18.8</v>
       </c>
       <c r="J21" t="n">
-        <v>6.2</v>
+        <v>7.1</v>
       </c>
       <c r="K21" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="L21" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="22">
@@ -1475,19 +1475,19 @@
         <v>62.9</v>
       </c>
       <c r="H24" t="n">
-        <v>37.9</v>
+        <v>36.1</v>
       </c>
       <c r="I24" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J24" t="n">
-        <v>6.5</v>
+        <v>6.1</v>
       </c>
       <c r="K24" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="L24" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="25">
@@ -1522,10 +1522,10 @@
         <v>23</v>
       </c>
       <c r="I25" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="J25" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="K25" t="n">
         <v>1.2</v>
@@ -1654,7 +1654,7 @@
         <v>7.5</v>
       </c>
       <c r="I28" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="J28" t="n">
         <v>0.5</v>
@@ -1695,10 +1695,10 @@
         <v>12.9</v>
       </c>
       <c r="H29" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="I29" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="J29" t="n">
         <v>0.2</v>
@@ -1739,10 +1739,10 @@
         <v>24.2</v>
       </c>
       <c r="H30" t="n">
-        <v>11</v>
+        <v>10.7</v>
       </c>
       <c r="I30" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="J30" t="n">
         <v>1.1</v>
@@ -1868,13 +1868,13 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>23</v>
+        <v>19.9</v>
       </c>
       <c r="H33" t="n">
-        <v>4.8</v>
+        <v>4.1</v>
       </c>
       <c r="I33" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J33" t="n">
         <v>0.1</v>
@@ -2050,16 +2050,16 @@
         <v>77.5</v>
       </c>
       <c r="I37" t="n">
-        <v>58</v>
+        <v>58.1</v>
       </c>
       <c r="J37" t="n">
-        <v>40.5</v>
+        <v>40.7</v>
       </c>
       <c r="K37" t="n">
-        <v>23.2</v>
+        <v>23.8</v>
       </c>
       <c r="L37" t="n">
-        <v>13.4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38">
@@ -2091,16 +2091,16 @@
         <v>88.40000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>49.3</v>
+        <v>50</v>
       </c>
       <c r="I38" t="n">
-        <v>25.3</v>
+        <v>25.9</v>
       </c>
       <c r="J38" t="n">
-        <v>10.7</v>
+        <v>10.9</v>
       </c>
       <c r="K38" t="n">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="L38" t="n">
         <v>1.6</v>
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>92</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>68.8</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="I39" t="n">
-        <v>43.1</v>
+        <v>41.9</v>
       </c>
       <c r="J39" t="n">
-        <v>20.7</v>
+        <v>20.2</v>
       </c>
       <c r="K39" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="40">
@@ -2185,13 +2185,13 @@
         <v>12.8</v>
       </c>
       <c r="J40" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="K40" t="n">
         <v>1.9</v>
       </c>
       <c r="L40" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="41">
@@ -2232,7 +2232,7 @@
         <v>8.300000000000001</v>
       </c>
       <c r="K41" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="L41" t="n">
         <v>1.1</v>
@@ -2267,10 +2267,10 @@
         <v>72.59999999999999</v>
       </c>
       <c r="H42" t="n">
-        <v>23</v>
+        <v>23.3</v>
       </c>
       <c r="I42" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="J42" t="n">
         <v>3.6</v>
@@ -2308,16 +2308,16 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>47.1</v>
+        <v>49.2</v>
       </c>
       <c r="H43" t="n">
-        <v>22.7</v>
+        <v>23.8</v>
       </c>
       <c r="I43" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="J43" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="K43" t="n">
         <v>1.1</v>
@@ -2440,22 +2440,22 @@
         <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>52.9</v>
+        <v>50.7</v>
       </c>
       <c r="H46" t="n">
-        <v>26.4</v>
+        <v>24.3</v>
       </c>
       <c r="I46" t="n">
-        <v>10.7</v>
+        <v>10</v>
       </c>
       <c r="J46" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="K46" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L46" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="47">
@@ -2531,7 +2531,7 @@
         <v>24.4</v>
       </c>
       <c r="H48" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
       <c r="I48" t="n">
         <v>1.6</v>
@@ -2575,7 +2575,7 @@
         <v>22.7</v>
       </c>
       <c r="H49" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="I49" t="n">
         <v>0.4</v>
@@ -2616,16 +2616,16 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>8.1</v>
+        <v>10.4</v>
       </c>
       <c r="H50" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="I50" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2663,10 +2663,10 @@
         <v>11.6</v>
       </c>
       <c r="H51" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="I51" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2801,13 +2801,13 @@
         <v>56</v>
       </c>
       <c r="J54" t="n">
-        <v>38.3</v>
+        <v>38.4</v>
       </c>
       <c r="K54" t="n">
-        <v>24.8</v>
+        <v>24.9</v>
       </c>
       <c r="L54" t="n">
-        <v>16.1</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="55">
@@ -2839,19 +2839,19 @@
         <v>88.7</v>
       </c>
       <c r="H55" t="n">
-        <v>69.5</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="I55" t="n">
-        <v>43.3</v>
+        <v>41.7</v>
       </c>
       <c r="J55" t="n">
-        <v>20.4</v>
+        <v>19.7</v>
       </c>
       <c r="K55" t="n">
-        <v>11.1</v>
+        <v>10.3</v>
       </c>
       <c r="L55" t="n">
-        <v>5.3</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="56">
@@ -2886,13 +2886,13 @@
         <v>55.8</v>
       </c>
       <c r="I56" t="n">
-        <v>30.2</v>
+        <v>30.4</v>
       </c>
       <c r="J56" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="K56" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="L56" t="n">
         <v>3</v>
@@ -2933,13 +2933,13 @@
         <v>21.2</v>
       </c>
       <c r="J57" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="K57" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="L57" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="58">
@@ -3018,13 +3018,13 @@
         <v>31.2</v>
       </c>
       <c r="I59" t="n">
-        <v>12.7</v>
+        <v>13.3</v>
       </c>
       <c r="J59" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="K59" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="L59" t="n">
         <v>0.5</v>
@@ -3106,7 +3106,7 @@
         <v>12.6</v>
       </c>
       <c r="I61" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="J61" t="n">
         <v>1.6</v>
@@ -3191,13 +3191,13 @@
         <v>53.9</v>
       </c>
       <c r="H63" t="n">
-        <v>14.4</v>
+        <v>16.1</v>
       </c>
       <c r="I63" t="n">
-        <v>5.1</v>
+        <v>5.7</v>
       </c>
       <c r="J63" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="K63" t="n">
         <v>0.4</v>
@@ -3238,7 +3238,7 @@
         <v>9.5</v>
       </c>
       <c r="I64" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="J64" t="n">
         <v>0.4</v>
@@ -3285,7 +3285,7 @@
         <v>0.7</v>
       </c>
       <c r="J65" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-10)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -554,16 +554,16 @@
         <v>65.2</v>
       </c>
       <c r="I3" t="n">
-        <v>38.8</v>
+        <v>39.3</v>
       </c>
       <c r="J3" t="n">
-        <v>16.7</v>
+        <v>16.8</v>
       </c>
       <c r="K3" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="L3" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>92.5</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>64.09999999999999</v>
+        <v>61.1</v>
       </c>
       <c r="I4" t="n">
-        <v>36.4</v>
+        <v>34.7</v>
       </c>
       <c r="J4" t="n">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
       <c r="K4" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
       <c r="L4" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5">
@@ -645,7 +645,7 @@
         <v>14</v>
       </c>
       <c r="J5" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="K5" t="n">
         <v>3.1</v>
@@ -689,13 +689,13 @@
         <v>14.9</v>
       </c>
       <c r="J6" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="K6" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="7">
@@ -727,10 +727,10 @@
         <v>64.59999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>24.7</v>
+        <v>25.6</v>
       </c>
       <c r="I7" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="J7" t="n">
         <v>3.2</v>
@@ -771,10 +771,10 @@
         <v>57.7</v>
       </c>
       <c r="H8" t="n">
-        <v>20.6</v>
+        <v>20.4</v>
       </c>
       <c r="I8" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="J8" t="n">
         <v>1.4</v>
@@ -783,7 +783,7 @@
         <v>0.4</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -821,7 +821,7 @@
         <v>4.5</v>
       </c>
       <c r="J9" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="K9" t="n">
         <v>0.5</v>
@@ -903,10 +903,10 @@
         <v>42.3</v>
       </c>
       <c r="H11" t="n">
-        <v>12.4</v>
+        <v>12.7</v>
       </c>
       <c r="I11" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="J11" t="n">
         <v>0.8</v>
@@ -947,16 +947,16 @@
         <v>20</v>
       </c>
       <c r="H12" t="n">
-        <v>6.3</v>
+        <v>6.7</v>
       </c>
       <c r="I12" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="J12" t="n">
         <v>0.5</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -991,10 +991,10 @@
         <v>15.4</v>
       </c>
       <c r="H13" t="n">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="I13" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="J13" t="n">
         <v>0.2</v>
@@ -1096,11 +1096,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1190</v>
+        <v>1460</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ETSU</t>
+          <t>Wright St</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1120,16 +1120,16 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>7.5</v>
+        <v>11.9</v>
       </c>
       <c r="H16" t="n">
-        <v>0.7</v>
+        <v>2.1</v>
       </c>
       <c r="I16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J16" t="n">
         <v>0.1</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1140,11 +1140,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1398</v>
+        <v>1474</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>Queens NC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1167,7 +1167,7 @@
         <v>11.8</v>
       </c>
       <c r="H17" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="I17" t="n">
         <v>0.1</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>98.59999999999999</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>78.09999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="I19" t="n">
-        <v>59.3</v>
+        <v>58.1</v>
       </c>
       <c r="J19" t="n">
-        <v>38.5</v>
+        <v>37.8</v>
       </c>
       <c r="K19" t="n">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
       <c r="L19" t="n">
-        <v>9.800000000000001</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="20">
@@ -1305,7 +1305,7 @@
         <v>48.8</v>
       </c>
       <c r="J20" t="n">
-        <v>27.2</v>
+        <v>27.3</v>
       </c>
       <c r="K20" t="n">
         <v>13.2</v>
@@ -1390,13 +1390,13 @@
         <v>46.3</v>
       </c>
       <c r="I22" t="n">
-        <v>15.2</v>
+        <v>15.5</v>
       </c>
       <c r="J22" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
       <c r="K22" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="L22" t="n">
         <v>0.4</v>
@@ -1434,10 +1434,10 @@
         <v>45.1</v>
       </c>
       <c r="I23" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="J23" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="K23" t="n">
         <v>1.9</v>
@@ -1481,10 +1481,10 @@
         <v>16.2</v>
       </c>
       <c r="J24" t="n">
-        <v>6.6</v>
+        <v>6.7</v>
       </c>
       <c r="K24" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="L24" t="n">
         <v>0.7</v>
@@ -1525,7 +1525,7 @@
         <v>10.4</v>
       </c>
       <c r="J25" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="K25" t="n">
         <v>1.2</v>
@@ -1563,13 +1563,13 @@
         <v>53.6</v>
       </c>
       <c r="H26" t="n">
-        <v>13</v>
+        <v>13.7</v>
       </c>
       <c r="I26" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="J26" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="K26" t="n">
         <v>0.5</v>
@@ -1607,13 +1607,13 @@
         <v>46.4</v>
       </c>
       <c r="H27" t="n">
-        <v>8.800000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="I27" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>0.2</v>
@@ -1748,7 +1748,7 @@
         <v>1.1</v>
       </c>
       <c r="K30" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L30" t="n">
         <v>0.1</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1250</v>
+        <v>1202</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Lehigh</t>
+          <t>Furman</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>34.6</v>
+        <v>57.1</v>
       </c>
       <c r="G35" t="n">
-        <v>0.6</v>
+        <v>1.4</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -1976,11 +1976,11 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1126</v>
+        <v>1224</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bethune-Cookman</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1997,13 +1997,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>65.40000000000001</v>
+        <v>42.9</v>
       </c>
       <c r="G36" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>95.7</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H37" t="n">
-        <v>80.5</v>
+        <v>81.7</v>
       </c>
       <c r="I37" t="n">
-        <v>60.5</v>
+        <v>61.4</v>
       </c>
       <c r="J37" t="n">
-        <v>42.9</v>
+        <v>43.6</v>
       </c>
       <c r="K37" t="n">
-        <v>24.9</v>
+        <v>25.4</v>
       </c>
       <c r="L37" t="n">
-        <v>14.6</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="38">
@@ -2141,13 +2141,13 @@
         <v>42.7</v>
       </c>
       <c r="J39" t="n">
-        <v>19.7</v>
+        <v>19.5</v>
       </c>
       <c r="K39" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="L39" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="40">
@@ -2182,7 +2182,7 @@
         <v>39.6</v>
       </c>
       <c r="I40" t="n">
-        <v>12.4</v>
+        <v>12.2</v>
       </c>
       <c r="J40" t="n">
         <v>5.3</v>
@@ -2226,10 +2226,10 @@
         <v>47.6</v>
       </c>
       <c r="I41" t="n">
-        <v>17.2</v>
+        <v>16.9</v>
       </c>
       <c r="J41" t="n">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
       <c r="K41" t="n">
         <v>3.2</v>
@@ -2317,7 +2317,7 @@
         <v>9.5</v>
       </c>
       <c r="J43" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="K43" t="n">
         <v>0.9</v>
@@ -2355,10 +2355,10 @@
         <v>52.8</v>
       </c>
       <c r="H44" t="n">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I44" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="J44" t="n">
         <v>1</v>
@@ -2399,16 +2399,16 @@
         <v>47.2</v>
       </c>
       <c r="H45" t="n">
-        <v>10.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I45" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="J45" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="K45" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L45" t="n">
         <v>0.1</v>
@@ -2537,7 +2537,7 @@
         <v>1.6</v>
       </c>
       <c r="J48" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K48" t="n">
         <v>0.1</v>
@@ -2680,11 +2680,11 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1224</v>
+        <v>1250</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>Lehigh</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2701,16 +2701,16 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>55.6</v>
+        <v>34.2</v>
       </c>
       <c r="G52" t="n">
-        <v>2.8</v>
+        <v>0.5</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2724,11 +2724,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1254</v>
+        <v>1126</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Bethune-Cookman</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2745,13 +2745,13 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>44.4</v>
+        <v>65.8</v>
       </c>
       <c r="G53" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
       <c r="H53" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2807,7 +2807,7 @@
         <v>23.9</v>
       </c>
       <c r="L54" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="55">
@@ -2886,7 +2886,7 @@
         <v>55.8</v>
       </c>
       <c r="I56" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="J56" t="n">
         <v>13.7</v>
@@ -2936,10 +2936,10 @@
         <v>11.8</v>
       </c>
       <c r="K57" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="L57" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="58">
@@ -3059,7 +3059,7 @@
         <v>51.1</v>
       </c>
       <c r="H60" t="n">
-        <v>15.3</v>
+        <v>15.5</v>
       </c>
       <c r="I60" t="n">
         <v>5.8</v>
@@ -3103,7 +3103,7 @@
         <v>53.2</v>
       </c>
       <c r="H61" t="n">
-        <v>14.3</v>
+        <v>14.5</v>
       </c>
       <c r="I61" t="n">
         <v>5.2</v>
@@ -3147,7 +3147,7 @@
         <v>46.8</v>
       </c>
       <c r="H62" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="I62" t="n">
         <v>3.8</v>
@@ -3191,16 +3191,16 @@
         <v>48.9</v>
       </c>
       <c r="H63" t="n">
-        <v>14.4</v>
+        <v>15.2</v>
       </c>
       <c r="I63" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="J63" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K63" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L63" t="n">
         <v>0.1</v>
@@ -3285,7 +3285,7 @@
         <v>0.7</v>
       </c>
       <c r="J65" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3384,11 +3384,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1460</v>
+        <v>1398</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Wright St</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3411,13 +3411,13 @@
         <v>11.3</v>
       </c>
       <c r="H68" t="n">
-        <v>2.4</v>
+        <v>1.4</v>
       </c>
       <c r="I68" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J68" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1474</v>
+        <v>1254</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Queens NC</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3455,10 +3455,10 @@
         <v>4.9</v>
       </c>
       <c r="H69" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="I69" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-11)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>96.8</v>
+        <v>97.2</v>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="I2" t="n">
-        <v>60.5</v>
+        <v>69</v>
       </c>
       <c r="J2" t="n">
-        <v>44.8</v>
+        <v>50.5</v>
       </c>
       <c r="K2" t="n">
-        <v>31.6</v>
+        <v>35</v>
       </c>
       <c r="L2" t="n">
-        <v>19.6</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="3">
@@ -551,28 +551,28 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>65.2</v>
+        <v>63.5</v>
       </c>
       <c r="I3" t="n">
-        <v>39.3</v>
+        <v>37.6</v>
       </c>
       <c r="J3" t="n">
-        <v>16.8</v>
+        <v>15.2</v>
       </c>
       <c r="K3" t="n">
-        <v>8.699999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="L3" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1235</v>
+        <v>1104</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Iowa St</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -592,31 +592,31 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>88.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>60.9</v>
+        <v>56.7</v>
       </c>
       <c r="I4" t="n">
-        <v>34.5</v>
+        <v>33</v>
       </c>
       <c r="J4" t="n">
         <v>14.8</v>
       </c>
       <c r="K4" t="n">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
       <c r="L4" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1403</v>
+        <v>1242</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -636,31 +636,31 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>80.90000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>44</v>
+        <v>38.1</v>
       </c>
       <c r="I5" t="n">
-        <v>14</v>
+        <v>9.4</v>
       </c>
       <c r="J5" t="n">
-        <v>7.1</v>
+        <v>3.9</v>
       </c>
       <c r="K5" t="n">
-        <v>3.1</v>
+        <v>1.4</v>
       </c>
       <c r="L5" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1116</v>
+        <v>1435</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,31 +680,31 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>72.3</v>
+        <v>75.3</v>
       </c>
       <c r="H6" t="n">
-        <v>41.2</v>
+        <v>47.7</v>
       </c>
       <c r="I6" t="n">
-        <v>14.9</v>
+        <v>12.5</v>
       </c>
       <c r="J6" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="K6" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1458</v>
+        <v>1314</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -724,19 +724,19 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>64.5</v>
+        <v>63.1</v>
       </c>
       <c r="H7" t="n">
-        <v>25.5</v>
+        <v>26.6</v>
       </c>
       <c r="I7" t="n">
-        <v>11.4</v>
+        <v>10.7</v>
       </c>
       <c r="J7" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="K7" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="L7" t="n">
         <v>0.3</v>
@@ -768,16 +768,16 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>57.7</v>
+        <v>50</v>
       </c>
       <c r="H8" t="n">
-        <v>20.4</v>
+        <v>18</v>
       </c>
       <c r="I8" t="n">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="J8" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="K8" t="n">
         <v>0.4</v>
@@ -788,11 +788,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1208</v>
+        <v>1429</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Utah St</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -812,31 +812,31 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>51.3</v>
+        <v>47</v>
       </c>
       <c r="H9" t="n">
-        <v>10</v>
+        <v>6.5</v>
       </c>
       <c r="I9" t="n">
-        <v>4.5</v>
+        <v>2.9</v>
       </c>
       <c r="J9" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="L9" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1326</v>
+        <v>1234</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ohio St</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -856,19 +856,19 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>48.7</v>
+        <v>53</v>
       </c>
       <c r="H10" t="n">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="I10" t="n">
-        <v>3.6</v>
+        <v>4.3</v>
       </c>
       <c r="J10" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="K10" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="L10" t="n">
         <v>0.1</v>
@@ -876,11 +876,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1301</v>
+        <v>1365</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -900,19 +900,19 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>42.3</v>
+        <v>50</v>
       </c>
       <c r="H11" t="n">
-        <v>12.7</v>
+        <v>17.2</v>
       </c>
       <c r="I11" t="n">
-        <v>3.9</v>
+        <v>7.2</v>
       </c>
       <c r="J11" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="L11" t="n">
         <v>0.1</v>
@@ -920,11 +920,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1365</v>
+        <v>1416</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -941,34 +941,34 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>55.6</v>
+        <v>44.2</v>
       </c>
       <c r="G12" t="n">
-        <v>20.9</v>
+        <v>15.9</v>
       </c>
       <c r="H12" t="n">
-        <v>7.2</v>
+        <v>5.6</v>
       </c>
       <c r="I12" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1374</v>
+        <v>1231</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>Indiana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -985,19 +985,19 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>44.4</v>
+        <v>55.8</v>
       </c>
       <c r="G13" t="n">
-        <v>14.6</v>
+        <v>20.9</v>
       </c>
       <c r="H13" t="n">
-        <v>4.3</v>
+        <v>7.6</v>
       </c>
       <c r="I13" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="K13" t="n">
         <v>0.1</v>
@@ -1008,11 +1008,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1378</v>
+        <v>1219</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1032,16 +1032,16 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>27.7</v>
+        <v>24.7</v>
       </c>
       <c r="H14" t="n">
-        <v>9.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="J14" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="K14" t="n">
         <v>0.1</v>
@@ -1052,11 +1052,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1372</v>
+        <v>1220</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SF Austin</t>
+          <t>Hofstra</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1076,13 +1076,13 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>19.1</v>
+        <v>24.9</v>
       </c>
       <c r="H15" t="n">
-        <v>4.9</v>
+        <v>5.9</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
         <v>0.1</v>
@@ -1096,11 +1096,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1460</v>
+        <v>1407</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wright St</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1120,16 +1120,16 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>11.9</v>
+        <v>17.4</v>
       </c>
       <c r="H16" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1140,11 +1140,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1474</v>
+        <v>1420</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Queens NC</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1167,7 +1167,7 @@
         <v>11.8</v>
       </c>
       <c r="H17" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="I17" t="n">
         <v>0.1</v>
@@ -1184,11 +1184,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1420</v>
+        <v>1224</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1198,20 +1198,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>100</v>
+        <v>44.1</v>
       </c>
       <c r="G18" t="n">
-        <v>3.2</v>
+        <v>1.4</v>
       </c>
       <c r="H18" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
@@ -1228,55 +1228,55 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1196</v>
+        <v>1186</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>E Washington</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>100</v>
+        <v>55.9</v>
       </c>
       <c r="G19" t="n">
-        <v>96.59999999999999</v>
+        <v>1.4</v>
       </c>
       <c r="H19" t="n">
-        <v>76.5</v>
+        <v>0.1</v>
       </c>
       <c r="I19" t="n">
-        <v>58.1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>37.8</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>19.3</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>9.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1222</v>
+        <v>1196</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1296,31 +1296,31 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>94.09999999999999</v>
+        <v>98.5</v>
       </c>
       <c r="H20" t="n">
-        <v>71.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>48.9</v>
+        <v>51.9</v>
       </c>
       <c r="J20" t="n">
-        <v>27.4</v>
+        <v>33.9</v>
       </c>
       <c r="K20" t="n">
-        <v>13.3</v>
+        <v>16.8</v>
       </c>
       <c r="L20" t="n">
-        <v>6.9</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1304</v>
+        <v>1222</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -1340,31 +1340,31 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>77</v>
+        <v>96.2</v>
       </c>
       <c r="H21" t="n">
-        <v>41.1</v>
+        <v>71.2</v>
       </c>
       <c r="I21" t="n">
-        <v>17.2</v>
+        <v>48</v>
       </c>
       <c r="J21" t="n">
-        <v>6.7</v>
+        <v>25</v>
       </c>
       <c r="K21" t="n">
-        <v>2.2</v>
+        <v>11.7</v>
       </c>
       <c r="L21" t="n">
-        <v>0.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1438</v>
+        <v>1304</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1384,31 +1384,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>89.8</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>46.3</v>
+        <v>47</v>
       </c>
       <c r="I22" t="n">
-        <v>15.5</v>
+        <v>19.7</v>
       </c>
       <c r="J22" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="K22" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="L22" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1385</v>
+        <v>1345</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1428,31 +1428,31 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>76.8</v>
+        <v>89.8</v>
       </c>
       <c r="H23" t="n">
-        <v>45.1</v>
+        <v>61.4</v>
       </c>
       <c r="I23" t="n">
-        <v>16.4</v>
+        <v>30.3</v>
       </c>
       <c r="J23" t="n">
-        <v>6.7</v>
+        <v>16.8</v>
       </c>
       <c r="K23" t="n">
-        <v>1.9</v>
+        <v>7.2</v>
       </c>
       <c r="L23" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1257</v>
+        <v>1385</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1472,31 +1472,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>62.9</v>
+        <v>68.7</v>
       </c>
       <c r="H24" t="n">
-        <v>37.9</v>
+        <v>27.1</v>
       </c>
       <c r="I24" t="n">
-        <v>16.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>6.7</v>
+        <v>3.6</v>
       </c>
       <c r="K24" t="n">
-        <v>2.3</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1388</v>
+        <v>1257</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -1516,31 +1516,31 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>64.5</v>
+        <v>71.2</v>
       </c>
       <c r="H25" t="n">
-        <v>20.1</v>
+        <v>41.4</v>
       </c>
       <c r="I25" t="n">
-        <v>9.800000000000001</v>
+        <v>17.5</v>
       </c>
       <c r="J25" t="n">
-        <v>3.4</v>
+        <v>6.8</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1429</v>
+        <v>1388</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Utah St</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E26" t="b">
@@ -1560,31 +1560,31 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>53.6</v>
+        <v>66.5</v>
       </c>
       <c r="H26" t="n">
-        <v>13.7</v>
+        <v>19.9</v>
       </c>
       <c r="I26" t="n">
-        <v>5.3</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>1.5</v>
+        <v>3.3</v>
       </c>
       <c r="K26" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1395</v>
+        <v>1274</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -1604,19 +1604,19 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>46.4</v>
+        <v>51</v>
       </c>
       <c r="H27" t="n">
         <v>9.5</v>
       </c>
       <c r="I27" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K27" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1281</v>
+        <v>1395</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E28" t="b">
@@ -1648,19 +1648,19 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>35.5</v>
+        <v>49</v>
       </c>
       <c r="H28" t="n">
-        <v>7.5</v>
+        <v>9.5</v>
       </c>
       <c r="I28" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="J28" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="K28" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1433</v>
+        <v>1400</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VCU</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1682,41 +1682,41 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>44.1</v>
+        <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>12.9</v>
+        <v>33.5</v>
       </c>
       <c r="H29" t="n">
-        <v>5.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I29" t="n">
-        <v>1.2</v>
+        <v>3.1</v>
       </c>
       <c r="J29" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="K29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L29" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1120</v>
+        <v>1281</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1726,41 +1726,41 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>55.9</v>
+        <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>24.2</v>
+        <v>28.8</v>
       </c>
       <c r="H30" t="n">
-        <v>11</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I30" t="n">
-        <v>3.6</v>
+        <v>2.3</v>
       </c>
       <c r="J30" t="n">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="K30" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="L30" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1463</v>
+        <v>1378</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>23.2</v>
+        <v>31.3</v>
       </c>
       <c r="H31" t="n">
-        <v>6.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>2.1</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="K31" t="n">
         <v>0.1</v>
@@ -1827,10 +1827,10 @@
         <v>10.2</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1414</v>
+        <v>1460</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>UC Irvine</t>
+          <t>Wright St</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1868,16 +1868,16 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>23</v>
+        <v>11.6</v>
       </c>
       <c r="H33" t="n">
-        <v>4.9</v>
+        <v>1.7</v>
       </c>
       <c r="I33" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="J33" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1888,11 +1888,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1340</v>
+        <v>1202</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Portland St</t>
+          <t>Furman</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1912,13 +1912,13 @@
         <v>100</v>
       </c>
       <c r="G34" t="n">
-        <v>5.9</v>
+        <v>3.8</v>
       </c>
       <c r="H34" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1202</v>
+        <v>1126</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Furman</t>
+          <t>Bethune-Cookman</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>57.1</v>
+        <v>67</v>
       </c>
       <c r="G35" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -1976,11 +1976,11 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1224</v>
+        <v>1250</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>Lehigh</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1997,13 +1997,13 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>42.9</v>
+        <v>33</v>
       </c>
       <c r="G36" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="H36" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>97.09999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="H37" t="n">
-        <v>81.7</v>
+        <v>78.3</v>
       </c>
       <c r="I37" t="n">
-        <v>61.4</v>
+        <v>57.8</v>
       </c>
       <c r="J37" t="n">
-        <v>43.6</v>
+        <v>39.1</v>
       </c>
       <c r="K37" t="n">
-        <v>25.4</v>
+        <v>22.9</v>
       </c>
       <c r="L37" t="n">
-        <v>14.8</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="38">
@@ -2088,31 +2088,31 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>88.40000000000001</v>
+        <v>94</v>
       </c>
       <c r="H38" t="n">
-        <v>50</v>
+        <v>64.8</v>
       </c>
       <c r="I38" t="n">
-        <v>24.4</v>
+        <v>33</v>
       </c>
       <c r="J38" t="n">
-        <v>10</v>
+        <v>13.2</v>
       </c>
       <c r="K38" t="n">
-        <v>3.9</v>
+        <v>5.2</v>
       </c>
       <c r="L38" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1345</v>
+        <v>1235</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Iowa St</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2132,31 +2132,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>89.59999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>67.09999999999999</v>
+        <v>60.7</v>
       </c>
       <c r="I39" t="n">
-        <v>42.7</v>
+        <v>38.5</v>
       </c>
       <c r="J39" t="n">
-        <v>19.5</v>
+        <v>19.1</v>
       </c>
       <c r="K39" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="L39" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1242</v>
+        <v>1403</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2176,31 +2176,31 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>77.3</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>39.6</v>
+        <v>41.7</v>
       </c>
       <c r="I40" t="n">
-        <v>12.2</v>
+        <v>15.1</v>
       </c>
       <c r="J40" t="n">
-        <v>5.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K40" t="n">
-        <v>1.9</v>
+        <v>3.3</v>
       </c>
       <c r="L40" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1435</v>
+        <v>1397</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2220,10 +2220,10 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>75.59999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="H41" t="n">
-        <v>47.6</v>
+        <v>48</v>
       </c>
       <c r="I41" t="n">
         <v>16.9</v>
@@ -2232,7 +2232,7 @@
         <v>8.4</v>
       </c>
       <c r="K41" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="L41" t="n">
         <v>1.1</v>
@@ -2240,11 +2240,11 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1314</v>
+        <v>1458</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2264,31 +2264,31 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>72.59999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="H42" t="n">
-        <v>23.3</v>
+        <v>27.5</v>
       </c>
       <c r="I42" t="n">
-        <v>10.4</v>
+        <v>13.6</v>
       </c>
       <c r="J42" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="K42" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="L42" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1246</v>
+        <v>1208</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2308,16 +2308,16 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>47.1</v>
+        <v>66</v>
       </c>
       <c r="H43" t="n">
-        <v>22.6</v>
+        <v>24.2</v>
       </c>
       <c r="I43" t="n">
-        <v>9.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J43" t="n">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
       <c r="K43" t="n">
         <v>0.9</v>
@@ -2328,11 +2328,11 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1155</v>
+        <v>1326</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Ohio St</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2352,31 +2352,31 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>52.8</v>
+        <v>62.9</v>
       </c>
       <c r="H44" t="n">
-        <v>8.300000000000001</v>
+        <v>15.1</v>
       </c>
       <c r="I44" t="n">
-        <v>3.2</v>
+        <v>6.2</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>2.2</v>
       </c>
       <c r="K44" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L44" t="n">
         <v>0.2</v>
-      </c>
-      <c r="L44" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1387</v>
+        <v>1155</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2396,31 +2396,31 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>47.2</v>
+        <v>37.1</v>
       </c>
       <c r="H45" t="n">
-        <v>9.800000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="I45" t="n">
-        <v>4</v>
+        <v>2.1</v>
       </c>
       <c r="J45" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="K45" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L45" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1234</v>
+        <v>1301</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2440,31 +2440,31 @@
         <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>52.9</v>
+        <v>34</v>
       </c>
       <c r="H46" t="n">
-        <v>25.4</v>
+        <v>10.2</v>
       </c>
       <c r="I46" t="n">
-        <v>10.4</v>
+        <v>2.9</v>
       </c>
       <c r="J46" t="n">
-        <v>3.2</v>
+        <v>0.7</v>
       </c>
       <c r="K46" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="L46" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1275</v>
+        <v>1374</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2474,29 +2474,29 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>100</v>
+        <v>55.6</v>
       </c>
       <c r="G47" t="n">
-        <v>27.4</v>
+        <v>18.8</v>
       </c>
       <c r="H47" t="n">
-        <v>6.3</v>
+        <v>5.8</v>
       </c>
       <c r="I47" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="J47" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
@@ -2504,11 +2504,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1219</v>
+        <v>1433</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2518,29 +2518,29 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>100</v>
+        <v>44.4</v>
       </c>
       <c r="G48" t="n">
-        <v>24.4</v>
+        <v>13.5</v>
       </c>
       <c r="H48" t="n">
-        <v>8.6</v>
+        <v>3.9</v>
       </c>
       <c r="I48" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="J48" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K48" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1295</v>
+        <v>1320</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -2572,16 +2572,16 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>22.7</v>
+        <v>18.7</v>
       </c>
       <c r="H49" t="n">
-        <v>4.2</v>
+        <v>4.7</v>
       </c>
       <c r="I49" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2592,11 +2592,11 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1220</v>
+        <v>1430</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Hofstra</t>
+          <t>Utah Valley</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -2616,16 +2616,16 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>10.4</v>
+        <v>25.6</v>
       </c>
       <c r="H50" t="n">
-        <v>3.3</v>
+        <v>5.6</v>
       </c>
       <c r="I50" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="J50" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2636,11 +2636,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1467</v>
+        <v>1295</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Merrimack</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -2660,16 +2660,16 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>11.6</v>
+        <v>12.1</v>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="I51" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2680,11 +2680,11 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1250</v>
+        <v>1474</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Lehigh</t>
+          <t>Queens NC</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2694,23 +2694,23 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>34.2</v>
+        <v>100</v>
       </c>
       <c r="G52" t="n">
-        <v>0.5</v>
+        <v>5.9</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2724,11 +2724,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1126</v>
+        <v>1254</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Bethune-Cookman</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2738,23 +2738,23 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>65.8</v>
+        <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="H53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I53" t="n">
         <v>0.1</v>
-      </c>
-      <c r="I53" t="n">
-        <v>0</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>95.09999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="H54" t="n">
-        <v>74.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I54" t="n">
-        <v>54.2</v>
+        <v>57.6</v>
       </c>
       <c r="J54" t="n">
-        <v>37</v>
+        <v>39.4</v>
       </c>
       <c r="K54" t="n">
-        <v>23.9</v>
+        <v>25.6</v>
       </c>
       <c r="L54" t="n">
-        <v>15.6</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="55">
@@ -2839,28 +2839,28 @@
         <v>88.7</v>
       </c>
       <c r="H55" t="n">
-        <v>67.90000000000001</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="I55" t="n">
-        <v>42.3</v>
+        <v>40.2</v>
       </c>
       <c r="J55" t="n">
-        <v>20</v>
+        <v>19.8</v>
       </c>
       <c r="K55" t="n">
-        <v>10.4</v>
+        <v>10.1</v>
       </c>
       <c r="L55" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1104</v>
+        <v>1211</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2880,31 +2880,31 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>82</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>55.8</v>
+        <v>57.6</v>
       </c>
       <c r="I56" t="n">
-        <v>30.5</v>
+        <v>32.7</v>
       </c>
       <c r="J56" t="n">
-        <v>13.7</v>
+        <v>15.6</v>
       </c>
       <c r="K56" t="n">
-        <v>6.3</v>
+        <v>7.7</v>
       </c>
       <c r="L56" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1211</v>
+        <v>1438</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2924,31 +2924,31 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>87.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H57" t="n">
-        <v>53.3</v>
+        <v>42.8</v>
       </c>
       <c r="I57" t="n">
-        <v>21.9</v>
+        <v>13.4</v>
       </c>
       <c r="J57" t="n">
-        <v>11.8</v>
+        <v>5.6</v>
       </c>
       <c r="K57" t="n">
-        <v>6.1</v>
+        <v>2</v>
       </c>
       <c r="L57" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1397</v>
+        <v>1116</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2968,22 +2968,22 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>82.40000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="H58" t="n">
-        <v>39.8</v>
+        <v>44.5</v>
       </c>
       <c r="I58" t="n">
-        <v>13.5</v>
+        <v>15.1</v>
       </c>
       <c r="J58" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="K58" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="59">
@@ -3012,19 +3012,19 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>73.3</v>
+        <v>75.2</v>
       </c>
       <c r="H59" t="n">
-        <v>31.1</v>
+        <v>33.8</v>
       </c>
       <c r="I59" t="n">
-        <v>12.9</v>
+        <v>13.6</v>
       </c>
       <c r="J59" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="K59" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="L59" t="n">
         <v>0.5</v>
@@ -3032,11 +3032,11 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1274</v>
+        <v>1246</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3056,22 +3056,22 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>51.1</v>
+        <v>55.3</v>
       </c>
       <c r="H60" t="n">
-        <v>15.5</v>
+        <v>18.8</v>
       </c>
       <c r="I60" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="J60" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="K60" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L60" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="61">
@@ -3106,13 +3106,13 @@
         <v>14.5</v>
       </c>
       <c r="I61" t="n">
-        <v>5.2</v>
+        <v>6.8</v>
       </c>
       <c r="J61" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="K61" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="L61" t="n">
         <v>0.2</v>
@@ -3147,16 +3147,16 @@
         <v>46.8</v>
       </c>
       <c r="H62" t="n">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="I62" t="n">
-        <v>3.8</v>
+        <v>4.7</v>
       </c>
       <c r="J62" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="K62" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L62" t="n">
         <v>0.1</v>
@@ -3164,11 +3164,11 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1400</v>
+        <v>1387</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3188,19 +3188,19 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>48.9</v>
+        <v>44.7</v>
       </c>
       <c r="H63" t="n">
-        <v>15.2</v>
+        <v>14.9</v>
       </c>
       <c r="I63" t="n">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="J63" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="K63" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L63" t="n">
         <v>0.1</v>
@@ -3208,11 +3208,11 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1416</v>
+        <v>1275</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3232,19 +3232,19 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>26.7</v>
+        <v>24.8</v>
       </c>
       <c r="H64" t="n">
-        <v>9.300000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="I64" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="K64" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -3252,11 +3252,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1320</v>
+        <v>1463</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>17.6</v>
+        <v>25.3</v>
       </c>
       <c r="H65" t="n">
-        <v>4</v>
+        <v>7.7</v>
       </c>
       <c r="I65" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="J65" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3296,11 +3296,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1430</v>
+        <v>1372</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Utah Valley</t>
+          <t>SF Austin</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3320,13 +3320,13 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>12.1</v>
+        <v>16.6</v>
       </c>
       <c r="H66" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="I66" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="J66" t="n">
         <v>0.2</v>
@@ -3340,11 +3340,11 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1407</v>
+        <v>1414</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>UC Irvine</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3364,16 +3364,16 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>18</v>
+        <v>11.9</v>
       </c>
       <c r="H67" t="n">
         <v>3.8</v>
       </c>
       <c r="I67" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3411,7 +3411,7 @@
         <v>11.3</v>
       </c>
       <c r="H68" t="n">
-        <v>1.4</v>
+        <v>1.9</v>
       </c>
       <c r="I68" t="n">
         <v>0.2</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1254</v>
+        <v>1373</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Siena</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>4.9</v>
+        <v>5.2</v>
       </c>
       <c r="H69" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-12)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,19 +504,19 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>98.3</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>85.2</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>69.7</v>
+        <v>68.3</v>
       </c>
       <c r="J2" t="n">
-        <v>51.1</v>
+        <v>50.4</v>
       </c>
       <c r="K2" t="n">
-        <v>35.4</v>
+        <v>35.2</v>
       </c>
       <c r="L2" t="n">
         <v>22.4</v>
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>88.09999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="H3" t="n">
-        <v>63.5</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>37.6</v>
+        <v>38.8</v>
       </c>
       <c r="J3" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="K3" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="L3" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>82.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="I4" t="n">
         <v>33</v>
       </c>
       <c r="J4" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="K4" t="n">
         <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="5">
@@ -636,16 +636,16 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>75.09999999999999</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>38.1</v>
+        <v>39.1</v>
       </c>
       <c r="I5" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="J5" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="K5" t="n">
         <v>1.4</v>
@@ -656,11 +656,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1435</v>
+        <v>1397</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>75.3</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>47.7</v>
+        <v>51.3</v>
       </c>
       <c r="I6" t="n">
-        <v>12.4</v>
+        <v>13.7</v>
       </c>
       <c r="J6" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="K6" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="L6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -724,22 +724,22 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>63.1</v>
+        <v>72.7</v>
       </c>
       <c r="H7" t="n">
-        <v>26.6</v>
+        <v>30.7</v>
       </c>
       <c r="I7" t="n">
-        <v>10.7</v>
+        <v>12.9</v>
       </c>
       <c r="J7" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8">
@@ -768,31 +768,31 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>50</v>
+        <v>59.8</v>
       </c>
       <c r="H8" t="n">
-        <v>18</v>
+        <v>20.7</v>
       </c>
       <c r="I8" t="n">
-        <v>6.8</v>
+        <v>8.4</v>
       </c>
       <c r="J8" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1429</v>
+        <v>1274</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Utah St</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -812,22 +812,22 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>47</v>
+        <v>42.2</v>
       </c>
       <c r="H9" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="I9" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
       <c r="J9" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="K9" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -856,31 +856,31 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>53</v>
+        <v>57.8</v>
       </c>
       <c r="H10" t="n">
-        <v>8.6</v>
+        <v>11</v>
       </c>
       <c r="I10" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1365</v>
+        <v>1416</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -900,31 +900,31 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>50</v>
+        <v>40.2</v>
       </c>
       <c r="H11" t="n">
-        <v>17.2</v>
+        <v>12</v>
       </c>
       <c r="I11" t="n">
-        <v>7.2</v>
+        <v>4</v>
       </c>
       <c r="J11" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="K11" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1416</v>
+        <v>1275</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -934,26 +934,26 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>44.2</v>
+        <v>100</v>
       </c>
       <c r="G12" t="n">
-        <v>15.9</v>
+        <v>27.3</v>
       </c>
       <c r="H12" t="n">
-        <v>5.6</v>
+        <v>8.4</v>
       </c>
       <c r="I12" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K12" t="n">
         <v>0.1</v>
@@ -964,11 +964,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1231</v>
+        <v>1320</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Indiana</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -978,29 +978,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>55.8</v>
+        <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>20.9</v>
+        <v>18.6</v>
       </c>
       <c r="H13" t="n">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="I13" t="n">
-        <v>2.4</v>
+        <v>0.9</v>
       </c>
       <c r="J13" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1008,11 +1008,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1219</v>
+        <v>1358</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>Sam Houston St</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1032,19 +1032,19 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>24.7</v>
+        <v>23.1</v>
       </c>
       <c r="H14" t="n">
-        <v>8.300000000000001</v>
+        <v>2.9</v>
       </c>
       <c r="I14" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1052,11 +1052,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1220</v>
+        <v>1407</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hofstra</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1076,16 +1076,16 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>24.9</v>
+        <v>17.6</v>
       </c>
       <c r="H15" t="n">
-        <v>5.9</v>
+        <v>4.1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="J15" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1096,11 +1096,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1407</v>
+        <v>1474</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Queens NC</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1120,16 +1120,16 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>17.4</v>
+        <v>11.8</v>
       </c>
       <c r="H16" t="n">
-        <v>3.6</v>
+        <v>1.7</v>
       </c>
       <c r="I16" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1140,11 +1140,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1420</v>
+        <v>1373</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Siena</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -1164,13 +1164,13 @@
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>11.8</v>
+        <v>2.1</v>
       </c>
       <c r="H17" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1184,99 +1184,99 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1224</v>
+        <v>1196</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>53.5</v>
+        <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>1.7</v>
+        <v>97.8</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1</v>
+        <v>77.7</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>49.7</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>31.6</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1285</v>
+        <v>1222</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Montana</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>46.5</v>
+        <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>96.3</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>72.5</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>27.5</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>13.2</v>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1196</v>
+        <v>1304</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1296,31 +1296,31 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>98.5</v>
+        <v>88.3</v>
       </c>
       <c r="H20" t="n">
-        <v>80.90000000000001</v>
+        <v>49.5</v>
       </c>
       <c r="I20" t="n">
-        <v>51.9</v>
+        <v>20.3</v>
       </c>
       <c r="J20" t="n">
-        <v>33.9</v>
+        <v>7.2</v>
       </c>
       <c r="K20" t="n">
-        <v>16.8</v>
+        <v>2.4</v>
       </c>
       <c r="L20" t="n">
-        <v>8.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1222</v>
+        <v>1345</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -1340,31 +1340,31 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>96.2</v>
+        <v>90</v>
       </c>
       <c r="H21" t="n">
-        <v>71.2</v>
+        <v>61.6</v>
       </c>
       <c r="I21" t="n">
-        <v>48</v>
+        <v>31.1</v>
       </c>
       <c r="J21" t="n">
-        <v>25</v>
+        <v>17.3</v>
       </c>
       <c r="K21" t="n">
-        <v>11.7</v>
+        <v>7.5</v>
       </c>
       <c r="L21" t="n">
-        <v>6.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1304</v>
+        <v>1385</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1384,31 +1384,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>88.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="H22" t="n">
-        <v>47</v>
+        <v>27.1</v>
       </c>
       <c r="I22" t="n">
-        <v>19.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>7</v>
+        <v>3.7</v>
       </c>
       <c r="K22" t="n">
-        <v>2.5</v>
+        <v>1.1</v>
       </c>
       <c r="L22" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1345</v>
+        <v>1140</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>BYU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1428,31 +1428,31 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>89.8</v>
+        <v>61.9</v>
       </c>
       <c r="H23" t="n">
-        <v>61.4</v>
+        <v>33.8</v>
       </c>
       <c r="I23" t="n">
-        <v>30.3</v>
+        <v>12</v>
       </c>
       <c r="J23" t="n">
-        <v>16.8</v>
+        <v>4.4</v>
       </c>
       <c r="K23" t="n">
-        <v>7.2</v>
+        <v>1.6</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1385</v>
+        <v>1388</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1472,31 +1472,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>68.7</v>
+        <v>63.9</v>
       </c>
       <c r="H24" t="n">
-        <v>27.1</v>
+        <v>19.2</v>
       </c>
       <c r="I24" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="J24" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="K24" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="L24" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1257</v>
+        <v>1395</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -1516,31 +1516,31 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>71.2</v>
+        <v>44.3</v>
       </c>
       <c r="H25" t="n">
-        <v>41.4</v>
+        <v>8.5</v>
       </c>
       <c r="I25" t="n">
-        <v>17.5</v>
+        <v>2.8</v>
       </c>
       <c r="J25" t="n">
-        <v>6.8</v>
+        <v>0.8</v>
       </c>
       <c r="K25" t="n">
-        <v>2.2</v>
+        <v>0.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1388</v>
+        <v>1326</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>Ohio St</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E26" t="b">
@@ -1560,31 +1560,31 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>66.5</v>
+        <v>55.7</v>
       </c>
       <c r="H26" t="n">
-        <v>19.9</v>
+        <v>13.6</v>
       </c>
       <c r="I26" t="n">
-        <v>9.300000000000001</v>
+        <v>4.8</v>
       </c>
       <c r="J26" t="n">
-        <v>3.3</v>
+        <v>1.7</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1274</v>
+        <v>1301</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -1604,19 +1604,19 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>51</v>
+        <v>36.1</v>
       </c>
       <c r="H27" t="n">
-        <v>9.5</v>
+        <v>8</v>
       </c>
       <c r="I27" t="n">
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="K27" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1395</v>
+        <v>1374</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1638,29 +1638,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>100</v>
+        <v>44.2</v>
       </c>
       <c r="G28" t="n">
-        <v>49</v>
+        <v>14.3</v>
       </c>
       <c r="H28" t="n">
-        <v>9.5</v>
+        <v>4.7</v>
       </c>
       <c r="I28" t="n">
-        <v>3</v>
+        <v>1.1</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1400</v>
+        <v>1120</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Texas</t>
+          <t>Auburn</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1682,29 +1682,29 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>100</v>
+        <v>55.8</v>
       </c>
       <c r="G29" t="n">
-        <v>33.5</v>
+        <v>23.8</v>
       </c>
       <c r="H29" t="n">
-        <v>8.699999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I29" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="J29" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="K29" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L29" t="n">
         <v>0.1</v>
@@ -1712,11 +1712,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1281</v>
+        <v>1378</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E30" t="b">
@@ -1736,16 +1736,16 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>28.8</v>
+        <v>30.8</v>
       </c>
       <c r="H30" t="n">
-        <v>9.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I30" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="J30" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="K30" t="n">
         <v>0.1</v>
@@ -1756,11 +1756,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1378</v>
+        <v>1220</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>Hofstra</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E31" t="b">
@@ -1780,19 +1780,19 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>31.3</v>
+        <v>10</v>
       </c>
       <c r="H31" t="n">
-        <v>9.699999999999999</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>2.1</v>
+        <v>0.3</v>
       </c>
       <c r="J31" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -1800,11 +1800,11 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1251</v>
+        <v>1460</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Liberty</t>
+          <t>Wright St</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E32" t="b">
@@ -1824,13 +1824,13 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>10.2</v>
+        <v>11.7</v>
       </c>
       <c r="H32" t="n">
-        <v>1.8</v>
+        <v>2.2</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1460</v>
+        <v>1202</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Wright St</t>
+          <t>Furman</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="b">
@@ -1868,13 +1868,13 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>11.6</v>
+        <v>3.7</v>
       </c>
       <c r="H33" t="n">
-        <v>1.7</v>
+        <v>0.3</v>
       </c>
       <c r="I33" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1888,11 +1888,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1202</v>
+        <v>1380</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Furman</t>
+          <t>Southern Univ</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1902,20 +1902,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>100</v>
+        <v>56.6</v>
       </c>
       <c r="G34" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="H34" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1126</v>
+        <v>1250</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bethune-Cookman</t>
+          <t>Lehigh</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1946,17 +1946,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E35" t="b">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>67</v>
+        <v>43.4</v>
       </c>
       <c r="G35" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1976,55 +1976,55 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1250</v>
+        <v>1276</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Lehigh</t>
+          <t>Michigan</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>MW</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>0.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>56.6</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>37.5</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>21.8</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1276</v>
+        <v>1163</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Michigan</t>
+          <t>Connecticut</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E37" t="b">
@@ -2044,31 +2044,31 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>96.2</v>
+        <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>78.3</v>
+        <v>60.6</v>
       </c>
       <c r="I37" t="n">
-        <v>57.8</v>
+        <v>27.8</v>
       </c>
       <c r="J37" t="n">
-        <v>39.1</v>
+        <v>11.4</v>
       </c>
       <c r="K37" t="n">
-        <v>22.9</v>
+        <v>4.4</v>
       </c>
       <c r="L37" t="n">
-        <v>13.1</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1163</v>
+        <v>1235</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Connecticut</t>
+          <t>Iowa St</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E38" t="b">
@@ -2088,31 +2088,31 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>94</v>
+        <v>88.3</v>
       </c>
       <c r="H38" t="n">
-        <v>64.8</v>
+        <v>62.1</v>
       </c>
       <c r="I38" t="n">
-        <v>33</v>
+        <v>42.4</v>
       </c>
       <c r="J38" t="n">
-        <v>13.2</v>
+        <v>22.3</v>
       </c>
       <c r="K38" t="n">
-        <v>5.2</v>
+        <v>10.9</v>
       </c>
       <c r="L38" t="n">
-        <v>1.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1235</v>
+        <v>1403</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Iowa St</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E39" t="b">
@@ -2132,31 +2132,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>87.90000000000001</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>60.7</v>
+        <v>44.6</v>
       </c>
       <c r="I39" t="n">
-        <v>38.5</v>
+        <v>16.6</v>
       </c>
       <c r="J39" t="n">
-        <v>19.1</v>
+        <v>8.5</v>
       </c>
       <c r="K39" t="n">
-        <v>9.1</v>
+        <v>3.5</v>
       </c>
       <c r="L39" t="n">
-        <v>3.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1403</v>
+        <v>1435</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E40" t="b">
@@ -2176,31 +2176,31 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>74.40000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="H40" t="n">
-        <v>41.7</v>
+        <v>42.8</v>
       </c>
       <c r="I40" t="n">
-        <v>15.1</v>
+        <v>15.8</v>
       </c>
       <c r="J40" t="n">
-        <v>8.300000000000001</v>
+        <v>7</v>
       </c>
       <c r="K40" t="n">
-        <v>3.3</v>
+        <v>2.7</v>
       </c>
       <c r="L40" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1397</v>
+        <v>1257</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E41" t="b">
@@ -2220,31 +2220,31 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>81.3</v>
+        <v>72.5</v>
       </c>
       <c r="H41" t="n">
-        <v>48</v>
+        <v>28.7</v>
       </c>
       <c r="I41" t="n">
-        <v>16.9</v>
+        <v>14.7</v>
       </c>
       <c r="J41" t="n">
-        <v>8.4</v>
+        <v>5.9</v>
       </c>
       <c r="K41" t="n">
-        <v>3.1</v>
+        <v>2.2</v>
       </c>
       <c r="L41" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1458</v>
+        <v>1208</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E42" t="b">
@@ -2264,31 +2264,31 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>67.7</v>
+        <v>55.9</v>
       </c>
       <c r="H42" t="n">
-        <v>27.5</v>
+        <v>22.6</v>
       </c>
       <c r="I42" t="n">
-        <v>13.6</v>
+        <v>7.9</v>
       </c>
       <c r="J42" t="n">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
       <c r="K42" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="L42" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1208</v>
+        <v>1429</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Utah St</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E43" t="b">
@@ -2308,31 +2308,31 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>66</v>
+        <v>53.5</v>
       </c>
       <c r="H43" t="n">
-        <v>24.2</v>
+        <v>13.9</v>
       </c>
       <c r="I43" t="n">
-        <v>8.699999999999999</v>
+        <v>5.6</v>
       </c>
       <c r="J43" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="K43" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="L43" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1326</v>
+        <v>1155</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ohio St</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E44" t="b">
@@ -2352,31 +2352,31 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>62.9</v>
+        <v>46.5</v>
       </c>
       <c r="H44" t="n">
-        <v>15.1</v>
+        <v>8.9</v>
       </c>
       <c r="I44" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
       <c r="K44" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="L44" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1155</v>
+        <v>1365</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E45" t="b">
@@ -2396,31 +2396,31 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>37.1</v>
+        <v>44.1</v>
       </c>
       <c r="H45" t="n">
-        <v>6.2</v>
+        <v>15.4</v>
       </c>
       <c r="I45" t="n">
-        <v>2.1</v>
+        <v>4.7</v>
       </c>
       <c r="J45" t="n">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="K45" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1301</v>
+        <v>1281</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2430,29 +2430,29 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>100</v>
+        <v>53.3</v>
       </c>
       <c r="G46" t="n">
-        <v>34</v>
+        <v>14.7</v>
       </c>
       <c r="H46" t="n">
-        <v>10.2</v>
+        <v>3.5</v>
       </c>
       <c r="I46" t="n">
-        <v>2.9</v>
+        <v>0.9</v>
       </c>
       <c r="J46" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="K46" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2460,11 +2460,11 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1374</v>
+        <v>1433</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2474,26 +2474,26 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E47" t="b">
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>55.6</v>
+        <v>46.7</v>
       </c>
       <c r="G47" t="n">
-        <v>18.8</v>
+        <v>12.8</v>
       </c>
       <c r="H47" t="n">
-        <v>5.8</v>
+        <v>3.3</v>
       </c>
       <c r="I47" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="J47" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2504,11 +2504,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1433</v>
+        <v>1219</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VCU</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2518,23 +2518,23 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>44.4</v>
+        <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>13.5</v>
+        <v>24.3</v>
       </c>
       <c r="H48" t="n">
-        <v>3.9</v>
+        <v>6.7</v>
       </c>
       <c r="I48" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="J48" t="n">
         <v>0.2</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1320</v>
+        <v>1430</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>Utah Valley</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -2572,13 +2572,13 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>18.7</v>
+        <v>25.6</v>
       </c>
       <c r="H49" t="n">
-        <v>4.7</v>
+        <v>5.9</v>
       </c>
       <c r="I49" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="J49" t="n">
         <v>0.2</v>
@@ -2592,11 +2592,11 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1430</v>
+        <v>1295</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Utah Valley</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -2616,16 +2616,16 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>25.6</v>
+        <v>11.7</v>
       </c>
       <c r="H50" t="n">
-        <v>5.6</v>
+        <v>2.3</v>
       </c>
       <c r="I50" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="J50" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2636,11 +2636,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1295</v>
+        <v>1420</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E51" t="b">
@@ -2660,16 +2660,16 @@
         <v>100</v>
       </c>
       <c r="G51" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
       <c r="H51" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="I51" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
@@ -2680,11 +2680,11 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1474</v>
+        <v>1224</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Queens NC</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2694,23 +2694,23 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E52" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>100</v>
+        <v>40.8</v>
       </c>
       <c r="G52" t="n">
-        <v>5.9</v>
+        <v>1.9</v>
       </c>
       <c r="H52" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -2724,11 +2724,11 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1254</v>
+        <v>1225</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2738,23 +2738,23 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>100</v>
+        <v>59.2</v>
       </c>
       <c r="G53" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="H53" t="n">
         <v>0.3</v>
       </c>
       <c r="I53" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>94.8</v>
+        <v>95.2</v>
       </c>
       <c r="H54" t="n">
-        <v>74.09999999999999</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>57.6</v>
+        <v>57.5</v>
       </c>
       <c r="J54" t="n">
-        <v>39.4</v>
+        <v>39.8</v>
       </c>
       <c r="K54" t="n">
-        <v>25.6</v>
+        <v>25.8</v>
       </c>
       <c r="L54" t="n">
-        <v>16.5</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="55">
@@ -2836,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>88.7</v>
+        <v>88.5</v>
       </c>
       <c r="H55" t="n">
-        <v>64.40000000000001</v>
+        <v>64.7</v>
       </c>
       <c r="I55" t="n">
-        <v>40.2</v>
+        <v>40.8</v>
       </c>
       <c r="J55" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="K55" t="n">
-        <v>10.1</v>
+        <v>10.6</v>
       </c>
       <c r="L55" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="56">
@@ -2883,19 +2883,19 @@
         <v>88.09999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>57.6</v>
+        <v>56.3</v>
       </c>
       <c r="I56" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="J56" t="n">
-        <v>15.6</v>
+        <v>14.3</v>
       </c>
       <c r="K56" t="n">
-        <v>7.7</v>
+        <v>7</v>
       </c>
       <c r="L56" t="n">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>83.40000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="H57" t="n">
-        <v>42.8</v>
+        <v>38.7</v>
       </c>
       <c r="I57" t="n">
-        <v>13.4</v>
+        <v>12.5</v>
       </c>
       <c r="J57" t="n">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="K57" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="L57" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="58">
@@ -2968,31 +2968,31 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>74.7</v>
+        <v>74.3</v>
       </c>
       <c r="H58" t="n">
-        <v>44.5</v>
+        <v>43.8</v>
       </c>
       <c r="I58" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="J58" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="K58" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="L58" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1140</v>
+        <v>1458</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>BYU</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3012,16 +3012,16 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>75.2</v>
+        <v>64</v>
       </c>
       <c r="H59" t="n">
-        <v>33.8</v>
+        <v>30.3</v>
       </c>
       <c r="I59" t="n">
-        <v>13.6</v>
+        <v>12.6</v>
       </c>
       <c r="J59" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="K59" t="n">
         <v>1.7</v>
@@ -3056,16 +3056,16 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
       <c r="H60" t="n">
         <v>18.8</v>
       </c>
       <c r="I60" t="n">
-        <v>7</v>
+        <v>7.6</v>
       </c>
       <c r="J60" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="K60" t="n">
         <v>0.8</v>
@@ -3100,10 +3100,10 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>53.2</v>
+        <v>53.7</v>
       </c>
       <c r="H61" t="n">
-        <v>14.5</v>
+        <v>14.1</v>
       </c>
       <c r="I61" t="n">
         <v>6.8</v>
@@ -3144,19 +3144,19 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>46.8</v>
+        <v>46.3</v>
       </c>
       <c r="H62" t="n">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="I62" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="J62" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="K62" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L62" t="n">
         <v>0.1</v>
@@ -3188,13 +3188,13 @@
         <v>100</v>
       </c>
       <c r="G63" t="n">
-        <v>44.7</v>
+        <v>44.4</v>
       </c>
       <c r="H63" t="n">
-        <v>14.9</v>
+        <v>14.6</v>
       </c>
       <c r="I63" t="n">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="J63" t="n">
         <v>1.1</v>
@@ -3208,11 +3208,11 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>1275</v>
+        <v>1400</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>Texas</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3232,19 +3232,19 @@
         <v>100</v>
       </c>
       <c r="G64" t="n">
-        <v>24.8</v>
+        <v>36</v>
       </c>
       <c r="H64" t="n">
-        <v>4.9</v>
+        <v>11</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>3.6</v>
       </c>
       <c r="J64" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K64" t="n">
         <v>0.2</v>
-      </c>
-      <c r="K64" t="n">
-        <v>0</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -3276,13 +3276,13 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>25.3</v>
+        <v>25.7</v>
       </c>
       <c r="H65" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
       <c r="I65" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="J65" t="n">
         <v>0.3</v>
@@ -3296,11 +3296,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1372</v>
+        <v>1270</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SF Austin</t>
+          <t>McNeese St</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3320,19 +3320,19 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>16.6</v>
+        <v>26.2</v>
       </c>
       <c r="H66" t="n">
-        <v>5</v>
+        <v>10.1</v>
       </c>
       <c r="I66" t="n">
-        <v>0.9</v>
+        <v>2.2</v>
       </c>
       <c r="J66" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3367,13 +3367,13 @@
         <v>11.9</v>
       </c>
       <c r="H67" t="n">
-        <v>3.8</v>
+        <v>2.5</v>
       </c>
       <c r="I67" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="J67" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
@@ -3408,13 +3408,13 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>11.3</v>
+        <v>11.5</v>
       </c>
       <c r="H68" t="n">
         <v>1.9</v>
       </c>
       <c r="I68" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1373</v>
+        <v>1254</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Siena</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3452,7 +3452,7 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
       <c r="H69" t="n">
         <v>0.4</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-13)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,62 +429,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TeamID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>TeamName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Is_FirstFour</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pct_R64</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pct_R32</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pct_S16</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pct_E8</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pct_F4</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pct_Finals</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pct_Champion</t>
         </is>
@@ -504,31 +516,31 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>97.90000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="H2" t="n">
-        <v>83.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>68.3</v>
+        <v>58.6</v>
       </c>
       <c r="J2" t="n">
-        <v>50.4</v>
+        <v>41.2</v>
       </c>
       <c r="K2" t="n">
-        <v>35.2</v>
+        <v>29.4</v>
       </c>
       <c r="L2" t="n">
-        <v>22.4</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1277</v>
+        <v>1235</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Michigan St</t>
+          <t>Iowa St</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -548,31 +560,31 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>88.2</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>65.59999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>38.8</v>
+        <v>45.2</v>
       </c>
       <c r="J3" t="n">
-        <v>14.9</v>
+        <v>20.3</v>
       </c>
       <c r="K3" t="n">
-        <v>7.5</v>
+        <v>11.1</v>
       </c>
       <c r="L3" t="n">
-        <v>3.4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1104</v>
+        <v>1228</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Illinois</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -595,28 +607,28 @@
         <v>82.40000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>56.8</v>
+        <v>57.7</v>
       </c>
       <c r="I4" t="n">
-        <v>33</v>
+        <v>31.1</v>
       </c>
       <c r="J4" t="n">
-        <v>14.5</v>
+        <v>13.8</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="L4" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1242</v>
+        <v>1345</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kansas</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -636,31 +648,31 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>76.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="H5" t="n">
-        <v>39.1</v>
+        <v>56.2</v>
       </c>
       <c r="I5" t="n">
-        <v>9.6</v>
+        <v>22.3</v>
       </c>
       <c r="J5" t="n">
-        <v>4</v>
+        <v>11.4</v>
       </c>
       <c r="K5" t="n">
-        <v>1.4</v>
+        <v>5.8</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1397</v>
+        <v>1116</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,31 +692,31 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>81.40000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="H6" t="n">
-        <v>51.3</v>
+        <v>34.1</v>
       </c>
       <c r="I6" t="n">
-        <v>13.7</v>
+        <v>11.7</v>
       </c>
       <c r="J6" t="n">
-        <v>7</v>
+        <v>4.8</v>
       </c>
       <c r="K6" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1314</v>
+        <v>1257</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -724,31 +736,31 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>72.7</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
         <v>30.7</v>
       </c>
       <c r="I7" t="n">
-        <v>12.9</v>
+        <v>11.4</v>
       </c>
       <c r="J7" t="n">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="L7" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1437</v>
+        <v>1246</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -768,19 +780,19 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>59.8</v>
+        <v>56</v>
       </c>
       <c r="H8" t="n">
-        <v>20.7</v>
+        <v>16</v>
       </c>
       <c r="I8" t="n">
-        <v>8.4</v>
+        <v>5.9</v>
       </c>
       <c r="J8" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L8" t="n">
         <v>0.1</v>
@@ -788,11 +800,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1274</v>
+        <v>1208</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -812,31 +824,31 @@
         <v>100</v>
       </c>
       <c r="G9" t="n">
-        <v>42.2</v>
+        <v>55.6</v>
       </c>
       <c r="H9" t="n">
-        <v>5.7</v>
+        <v>10.8</v>
       </c>
       <c r="I9" t="n">
-        <v>2.2</v>
+        <v>3.9</v>
       </c>
       <c r="J9" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1234</v>
+        <v>1395</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -856,31 +868,31 @@
         <v>100</v>
       </c>
       <c r="G10" t="n">
-        <v>57.8</v>
+        <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>11</v>
+        <v>6.3</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>2.1</v>
       </c>
       <c r="J10" t="n">
-        <v>2.1</v>
+        <v>0.6</v>
       </c>
       <c r="K10" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1416</v>
+        <v>1365</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>Santa Clara</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -900,31 +912,31 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>40.2</v>
+        <v>44</v>
       </c>
       <c r="H11" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="I11" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="K11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L11" t="n">
         <v>0.1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1275</v>
+        <v>1281</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>Missouri</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -934,29 +946,29 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>51.1</v>
       </c>
       <c r="G12" t="n">
-        <v>27.3</v>
+        <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>8.4</v>
+        <v>3.8</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>0.9</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -964,11 +976,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1320</v>
+        <v>1433</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -978,29 +990,29 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>100</v>
+        <v>48.9</v>
       </c>
       <c r="G13" t="n">
-        <v>18.6</v>
+        <v>13.6</v>
       </c>
       <c r="H13" t="n">
-        <v>6.7</v>
+        <v>4.4</v>
       </c>
       <c r="I13" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="J13" t="n">
         <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1008,11 +1020,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1358</v>
+        <v>1463</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sam Houston St</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1022,7 +1034,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -1032,16 +1044,16 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>23.1</v>
+        <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>2.9</v>
+        <v>6.6</v>
       </c>
       <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
         <v>0.2</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -1052,11 +1064,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1407</v>
+        <v>1320</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1066,7 +1078,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E15" t="b">
@@ -1076,16 +1088,16 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>17.6</v>
+        <v>10</v>
       </c>
       <c r="H15" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1096,11 +1108,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1474</v>
+        <v>1295</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Queens NC</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1110,7 +1122,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E16" t="b">
@@ -1120,13 +1132,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>11.8</v>
+        <v>17.6</v>
       </c>
       <c r="H16" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1140,11 +1152,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1373</v>
+        <v>1398</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Siena</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1154,7 +1166,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E17" t="b">
@@ -1164,13 +1176,13 @@
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>2.1</v>
+        <v>5.1</v>
       </c>
       <c r="H17" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1184,21 +1196,21 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1196</v>
+        <v>1373</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>Siena</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E18" t="b">
@@ -1208,31 +1220,31 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>97.8</v>
+        <v>2.8</v>
       </c>
       <c r="H18" t="n">
-        <v>77.7</v>
+        <v>0.3</v>
       </c>
       <c r="I18" t="n">
-        <v>49.7</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>31.6</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1222</v>
+        <v>1196</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Houston</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1242,7 +1254,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E19" t="b">
@@ -1252,31 +1264,31 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>96.3</v>
+        <v>97.8</v>
       </c>
       <c r="H19" t="n">
-        <v>72.5</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>51</v>
+        <v>57.9</v>
       </c>
       <c r="J19" t="n">
-        <v>27.5</v>
+        <v>37.1</v>
       </c>
       <c r="K19" t="n">
-        <v>13.2</v>
+        <v>18.1</v>
       </c>
       <c r="L19" t="n">
-        <v>6.9</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1304</v>
+        <v>1222</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1286,7 +1298,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E20" t="b">
@@ -1296,31 +1308,31 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>88.3</v>
+        <v>96.3</v>
       </c>
       <c r="H20" t="n">
-        <v>49.5</v>
+        <v>72.5</v>
       </c>
       <c r="I20" t="n">
-        <v>20.3</v>
+        <v>51.4</v>
       </c>
       <c r="J20" t="n">
-        <v>7.2</v>
+        <v>29.4</v>
       </c>
       <c r="K20" t="n">
-        <v>2.4</v>
+        <v>14.3</v>
       </c>
       <c r="L20" t="n">
-        <v>0.8</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1345</v>
+        <v>1304</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1330,7 +1342,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E21" t="b">
@@ -1340,31 +1352,31 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>90</v>
+        <v>88.3</v>
       </c>
       <c r="H21" t="n">
-        <v>61.6</v>
+        <v>54.4</v>
       </c>
       <c r="I21" t="n">
-        <v>31.1</v>
+        <v>22.2</v>
       </c>
       <c r="J21" t="n">
-        <v>17.3</v>
+        <v>8.4</v>
       </c>
       <c r="K21" t="n">
-        <v>7.5</v>
+        <v>2.5</v>
       </c>
       <c r="L21" t="n">
-        <v>3.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1385</v>
+        <v>1403</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1374,7 +1386,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E22" t="b">
@@ -1384,31 +1396,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>69.2</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>27.1</v>
+        <v>43.1</v>
       </c>
       <c r="I22" t="n">
-        <v>9.199999999999999</v>
+        <v>15.6</v>
       </c>
       <c r="J22" t="n">
-        <v>3.7</v>
+        <v>7</v>
       </c>
       <c r="K22" t="n">
-        <v>1.1</v>
+        <v>2.3</v>
       </c>
       <c r="L22" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1140</v>
+        <v>1385</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BYU</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1418,7 +1430,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E23" t="b">
@@ -1428,31 +1440,31 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>61.9</v>
+        <v>72.7</v>
       </c>
       <c r="H23" t="n">
-        <v>33.8</v>
+        <v>40.3</v>
       </c>
       <c r="I23" t="n">
-        <v>12</v>
+        <v>13.7</v>
       </c>
       <c r="J23" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="K23" t="n">
         <v>1.6</v>
       </c>
       <c r="L23" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1388</v>
+        <v>1314</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1462,7 +1474,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E24" t="b">
@@ -1472,31 +1484,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>63.9</v>
+        <v>67.7</v>
       </c>
       <c r="H24" t="n">
-        <v>19.2</v>
+        <v>32.9</v>
       </c>
       <c r="I24" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="J24" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="K24" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1395</v>
+        <v>1388</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1506,7 +1518,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E25" t="b">
@@ -1516,22 +1528,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>44.3</v>
+        <v>63.9</v>
       </c>
       <c r="H25" t="n">
-        <v>8.5</v>
+        <v>19.2</v>
       </c>
       <c r="I25" t="n">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="J25" t="n">
-        <v>0.8</v>
+        <v>3.7</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2</v>
+        <v>1.1</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="26">
@@ -1550,7 +1562,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E26" t="b">
@@ -1560,31 +1572,31 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>55.7</v>
+        <v>59.2</v>
       </c>
       <c r="H26" t="n">
-        <v>13.6</v>
+        <v>14.5</v>
       </c>
       <c r="I26" t="n">
-        <v>4.8</v>
+        <v>6.4</v>
       </c>
       <c r="J26" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
       <c r="K26" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L26" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1301</v>
+        <v>1155</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1594,7 +1606,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E27" t="b">
@@ -1604,19 +1616,19 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>36.1</v>
+        <v>40.8</v>
       </c>
       <c r="H27" t="n">
-        <v>8</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I27" t="n">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
       <c r="J27" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -1624,11 +1636,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1374</v>
+        <v>1387</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SMU</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1638,29 +1650,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>44.2</v>
+        <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>14.3</v>
+        <v>36.1</v>
       </c>
       <c r="H28" t="n">
-        <v>4.7</v>
+        <v>8</v>
       </c>
       <c r="I28" t="n">
-        <v>1.1</v>
+        <v>3.3</v>
       </c>
       <c r="J28" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K28" t="n">
         <v>0.2</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1668,11 +1680,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1120</v>
+        <v>1378</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Auburn</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1682,41 +1694,41 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>55.8</v>
+        <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>23.8</v>
+        <v>32.3</v>
       </c>
       <c r="H29" t="n">
-        <v>9.699999999999999</v>
+        <v>10.5</v>
       </c>
       <c r="I29" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="J29" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="K29" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="L29" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1378</v>
+        <v>1270</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>McNeese St</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1736,13 +1748,13 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>30.8</v>
+        <v>27.3</v>
       </c>
       <c r="H30" t="n">
-        <v>9.300000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="I30" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="J30" t="n">
         <v>0.5</v>
@@ -1756,11 +1768,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1220</v>
+        <v>1430</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hofstra</t>
+          <t>Utah Valley</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1780,16 +1792,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>10</v>
+        <v>26.9</v>
       </c>
       <c r="H31" t="n">
-        <v>2</v>
+        <v>6.4</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1830,7 +1842,7 @@
         <v>2.2</v>
       </c>
       <c r="I32" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1959,7 +1971,7 @@
         <v>0.9</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2003,19 +2015,19 @@
         <v>95.40000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>76.59999999999999</v>
+        <v>75.8</v>
       </c>
       <c r="I36" t="n">
-        <v>56.6</v>
+        <v>57</v>
       </c>
       <c r="J36" t="n">
-        <v>37.5</v>
+        <v>39.7</v>
       </c>
       <c r="K36" t="n">
-        <v>21.8</v>
+        <v>23.4</v>
       </c>
       <c r="L36" t="n">
-        <v>12.4</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="37">
@@ -2047,28 +2059,28 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>60.6</v>
+        <v>66.8</v>
       </c>
       <c r="I37" t="n">
-        <v>27.8</v>
+        <v>37.4</v>
       </c>
       <c r="J37" t="n">
-        <v>11.4</v>
+        <v>17.2</v>
       </c>
       <c r="K37" t="n">
-        <v>4.4</v>
+        <v>7.4</v>
       </c>
       <c r="L37" t="n">
-        <v>1.7</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1235</v>
+        <v>1104</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Iowa St</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2088,31 +2100,31 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>88.3</v>
+        <v>82.7</v>
       </c>
       <c r="H38" t="n">
-        <v>62.1</v>
+        <v>57</v>
       </c>
       <c r="I38" t="n">
-        <v>42.4</v>
+        <v>33.2</v>
       </c>
       <c r="J38" t="n">
-        <v>22.3</v>
+        <v>15.1</v>
       </c>
       <c r="K38" t="n">
-        <v>10.9</v>
+        <v>6.7</v>
       </c>
       <c r="L38" t="n">
-        <v>4.7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1403</v>
+        <v>1242</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Kansas</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2132,31 +2144,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>74.40000000000001</v>
+        <v>77</v>
       </c>
       <c r="H39" t="n">
-        <v>44.6</v>
+        <v>37.6</v>
       </c>
       <c r="I39" t="n">
-        <v>16.6</v>
+        <v>12</v>
       </c>
       <c r="J39" t="n">
-        <v>8.5</v>
+        <v>5.3</v>
       </c>
       <c r="K39" t="n">
-        <v>3.5</v>
+        <v>1.7</v>
       </c>
       <c r="L39" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1435</v>
+        <v>1397</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2176,31 +2188,31 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>75.7</v>
+        <v>72.8</v>
       </c>
       <c r="H40" t="n">
-        <v>42.8</v>
+        <v>47.4</v>
       </c>
       <c r="I40" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
       <c r="J40" t="n">
-        <v>7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K40" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="L40" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1257</v>
+        <v>1458</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2220,31 +2232,31 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>72.5</v>
+        <v>72.8</v>
       </c>
       <c r="H41" t="n">
-        <v>28.7</v>
+        <v>31.4</v>
       </c>
       <c r="I41" t="n">
-        <v>14.7</v>
+        <v>15.5</v>
       </c>
       <c r="J41" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="K41" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="L41" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1208</v>
+        <v>1274</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2267,19 +2279,19 @@
         <v>55.9</v>
       </c>
       <c r="H42" t="n">
-        <v>22.6</v>
+        <v>17.2</v>
       </c>
       <c r="I42" t="n">
-        <v>7.9</v>
+        <v>6.7</v>
       </c>
       <c r="J42" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="K42" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="L42" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="43">
@@ -2308,19 +2320,19 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>53.5</v>
+        <v>46.4</v>
       </c>
       <c r="H43" t="n">
-        <v>13.9</v>
+        <v>12.1</v>
       </c>
       <c r="I43" t="n">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="J43" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="K43" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2328,11 +2340,11 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1155</v>
+        <v>1234</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2352,31 +2364,31 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>46.5</v>
+        <v>53.6</v>
       </c>
       <c r="H44" t="n">
-        <v>8.9</v>
+        <v>11.8</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>5.3</v>
       </c>
       <c r="J44" t="n">
-        <v>0.8</v>
+        <v>2.1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1365</v>
+        <v>1416</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2399,28 +2411,28 @@
         <v>44.1</v>
       </c>
       <c r="H45" t="n">
-        <v>15.4</v>
+        <v>14.1</v>
       </c>
       <c r="I45" t="n">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
       <c r="J45" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="K45" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L45" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1281</v>
+        <v>1275</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Missouri</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2430,26 +2442,26 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>11a</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>53.3</v>
+        <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>14.7</v>
+        <v>27.2</v>
       </c>
       <c r="H46" t="n">
-        <v>3.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I46" t="n">
-        <v>0.9</v>
+        <v>2</v>
       </c>
       <c r="J46" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K46" t="n">
         <v>0</v>
@@ -2460,11 +2472,11 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1433</v>
+        <v>1103</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>VCU</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2474,29 +2486,29 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>11b</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>46.7</v>
+        <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>12.8</v>
+        <v>27.2</v>
       </c>
       <c r="H47" t="n">
-        <v>3.3</v>
+        <v>12.2</v>
       </c>
       <c r="I47" t="n">
-        <v>1.1</v>
+        <v>2.8</v>
       </c>
       <c r="J47" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="K47" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
@@ -2504,11 +2516,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1219</v>
+        <v>1358</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>Sam Houston St</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2518,7 +2530,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E48" t="b">
@@ -2528,16 +2540,16 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>24.3</v>
+        <v>23</v>
       </c>
       <c r="H48" t="n">
-        <v>6.7</v>
+        <v>2.7</v>
       </c>
       <c r="I48" t="n">
-        <v>1.3</v>
+        <v>0.4</v>
       </c>
       <c r="J48" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K48" t="n">
         <v>0</v>
@@ -2548,11 +2560,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1430</v>
+        <v>1407</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Utah Valley</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2562,7 +2574,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E49" t="b">
@@ -2572,16 +2584,16 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>25.6</v>
+        <v>17.3</v>
       </c>
       <c r="H49" t="n">
-        <v>5.9</v>
+        <v>3.4</v>
       </c>
       <c r="I49" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J49" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2592,11 +2604,11 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1295</v>
+        <v>1420</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2606,7 +2618,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E50" t="b">
@@ -2619,13 +2631,13 @@
         <v>11.7</v>
       </c>
       <c r="H50" t="n">
-        <v>2.3</v>
+        <v>1.9</v>
       </c>
       <c r="I50" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="J50" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
         <v>0</v>
@@ -2636,11 +2648,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1420</v>
+        <v>1224</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2650,23 +2662,23 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16a</t>
         </is>
       </c>
       <c r="E51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="G51" t="n">
-        <v>11.7</v>
+        <v>1.9</v>
       </c>
       <c r="H51" t="n">
-        <v>1.3</v>
+        <v>0.1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2680,11 +2692,11 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2694,17 +2706,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16a</t>
+          <t>16b</t>
         </is>
       </c>
       <c r="E52" t="b">
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>40.8</v>
+        <v>59</v>
       </c>
       <c r="G52" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2724,55 +2736,55 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1225</v>
+        <v>1112</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>Arizona</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>MW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16b</t>
+          <t>01</t>
         </is>
       </c>
       <c r="E53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>59.2</v>
+        <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>2.7</v>
+        <v>95.2</v>
       </c>
       <c r="H53" t="n">
-        <v>0.3</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>59.1</v>
       </c>
       <c r="J53" t="n">
-        <v>0</v>
+        <v>42.8</v>
       </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>28.2</v>
       </c>
       <c r="L53" t="n">
-        <v>0</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1112</v>
+        <v>1277</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>Michigan St</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2782,7 +2794,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E54" t="b">
@@ -2792,31 +2804,31 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>95.2</v>
+        <v>88.5</v>
       </c>
       <c r="H54" t="n">
-        <v>74.90000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="I54" t="n">
-        <v>57.5</v>
+        <v>38.1</v>
       </c>
       <c r="J54" t="n">
-        <v>39.8</v>
+        <v>16.4</v>
       </c>
       <c r="K54" t="n">
-        <v>25.8</v>
+        <v>7.9</v>
       </c>
       <c r="L54" t="n">
-        <v>15.9</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1228</v>
+        <v>1211</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Illinois</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2826,7 +2838,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="E55" t="b">
@@ -2836,31 +2848,31 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>88.5</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>64.7</v>
+        <v>56.6</v>
       </c>
       <c r="I55" t="n">
-        <v>40.8</v>
+        <v>34</v>
       </c>
       <c r="J55" t="n">
-        <v>19.9</v>
+        <v>15.2</v>
       </c>
       <c r="K55" t="n">
-        <v>10.6</v>
+        <v>7.9</v>
       </c>
       <c r="L55" t="n">
-        <v>4.6</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1211</v>
+        <v>1438</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2870,7 +2882,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="E56" t="b">
@@ -2880,31 +2892,31 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>88.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="H56" t="n">
-        <v>56.3</v>
+        <v>44.5</v>
       </c>
       <c r="I56" t="n">
-        <v>30.6</v>
+        <v>13.1</v>
       </c>
       <c r="J56" t="n">
-        <v>14.3</v>
+        <v>6</v>
       </c>
       <c r="K56" t="n">
-        <v>7</v>
+        <v>2.2</v>
       </c>
       <c r="L56" t="n">
-        <v>2.9</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1438</v>
+        <v>1435</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2914,7 +2926,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="E57" t="b">
@@ -2924,31 +2936,31 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>73.8</v>
+        <v>75.7</v>
       </c>
       <c r="H57" t="n">
-        <v>38.7</v>
+        <v>45.7</v>
       </c>
       <c r="I57" t="n">
-        <v>12.5</v>
+        <v>16</v>
       </c>
       <c r="J57" t="n">
-        <v>5.1</v>
+        <v>7.8</v>
       </c>
       <c r="K57" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="L57" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>1116</v>
+        <v>1140</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>BYU</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2958,7 +2970,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="E58" t="b">
@@ -2968,31 +2980,31 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>74.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>43.8</v>
+        <v>30.1</v>
       </c>
       <c r="I58" t="n">
-        <v>15.3</v>
+        <v>14</v>
       </c>
       <c r="J58" t="n">
-        <v>6.9</v>
+        <v>4.8</v>
       </c>
       <c r="K58" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="L58" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1458</v>
+        <v>1437</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3002,7 +3014,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="E59" t="b">
@@ -3012,31 +3024,31 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>64</v>
+        <v>53.9</v>
       </c>
       <c r="H59" t="n">
-        <v>30.3</v>
+        <v>17.8</v>
       </c>
       <c r="I59" t="n">
-        <v>12.6</v>
+        <v>5.6</v>
       </c>
       <c r="J59" t="n">
-        <v>4.6</v>
+        <v>1.5</v>
       </c>
       <c r="K59" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
       <c r="L59" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1246</v>
+        <v>1417</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Kentucky</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3046,7 +3058,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>08</t>
         </is>
       </c>
       <c r="E60" t="b">
@@ -3056,13 +3068,13 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>55.6</v>
+        <v>56.5</v>
       </c>
       <c r="H60" t="n">
-        <v>18.8</v>
+        <v>14.9</v>
       </c>
       <c r="I60" t="n">
-        <v>7.6</v>
+        <v>6.7</v>
       </c>
       <c r="J60" t="n">
         <v>2.5</v>
@@ -3076,11 +3088,11 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1417</v>
+        <v>1401</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3090,7 +3102,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>09</t>
         </is>
       </c>
       <c r="E61" t="b">
@@ -3100,31 +3112,31 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>53.7</v>
+        <v>43.5</v>
       </c>
       <c r="H61" t="n">
-        <v>14.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I61" t="n">
-        <v>6.8</v>
+        <v>3.3</v>
       </c>
       <c r="J61" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="K61" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="L61" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1401</v>
+        <v>1301</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3134,7 +3146,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E62" t="b">
@@ -3144,31 +3156,31 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>46.3</v>
+        <v>46.1</v>
       </c>
       <c r="H62" t="n">
-        <v>10.6</v>
+        <v>13.8</v>
       </c>
       <c r="I62" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="J62" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="K62" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L62" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>1387</v>
+        <v>1374</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>SMU</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3178,32 +3190,32 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11a</t>
         </is>
       </c>
       <c r="E63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>100</v>
+        <v>43.2</v>
       </c>
       <c r="G63" t="n">
-        <v>44.4</v>
+        <v>14.5</v>
       </c>
       <c r="H63" t="n">
-        <v>14.6</v>
+        <v>4.5</v>
       </c>
       <c r="I63" t="n">
-        <v>4.1</v>
+        <v>1.5</v>
       </c>
       <c r="J63" t="n">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="K63" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="L63" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -3222,29 +3234,29 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>11b</t>
         </is>
       </c>
       <c r="E64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>100</v>
+        <v>56.8</v>
       </c>
       <c r="G64" t="n">
-        <v>36</v>
+        <v>18.1</v>
       </c>
       <c r="H64" t="n">
-        <v>11</v>
+        <v>5.6</v>
       </c>
       <c r="I64" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
       <c r="J64" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="K64" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -3252,11 +3264,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1463</v>
+        <v>1219</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3276,13 +3288,13 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>25.7</v>
+        <v>24.3</v>
       </c>
       <c r="H65" t="n">
-        <v>7.3</v>
+        <v>6</v>
       </c>
       <c r="I65" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="J65" t="n">
         <v>0.3</v>
@@ -3296,11 +3308,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1270</v>
+        <v>1220</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>McNeese St</t>
+          <t>Hofstra</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3320,19 +3332,19 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>26.2</v>
+        <v>16.2</v>
       </c>
       <c r="H66" t="n">
-        <v>10.1</v>
+        <v>3.8</v>
       </c>
       <c r="I66" t="n">
-        <v>2.2</v>
+        <v>0.5</v>
       </c>
       <c r="J66" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="K66" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -3367,10 +3379,10 @@
         <v>11.9</v>
       </c>
       <c r="H67" t="n">
-        <v>2.5</v>
+        <v>3.3</v>
       </c>
       <c r="I67" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J67" t="n">
         <v>0.1</v>
@@ -3384,11 +3396,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1398</v>
+        <v>1474</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>Queens NC</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3411,10 +3423,10 @@
         <v>11.5</v>
       </c>
       <c r="H68" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-14)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>97.2</v>
+        <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>82.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="I2" t="n">
-        <v>58.6</v>
+        <v>60.9</v>
       </c>
       <c r="J2" t="n">
-        <v>41.2</v>
+        <v>39.1</v>
       </c>
       <c r="K2" t="n">
-        <v>29.4</v>
+        <v>24.2</v>
       </c>
       <c r="L2" t="n">
-        <v>18.2</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>94.90000000000001</v>
+        <v>96.3</v>
       </c>
       <c r="H3" t="n">
-        <v>71.59999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>45.2</v>
+        <v>47.5</v>
       </c>
       <c r="J3" t="n">
-        <v>20.3</v>
+        <v>25.7</v>
       </c>
       <c r="K3" t="n">
-        <v>11.1</v>
+        <v>13.7</v>
       </c>
       <c r="L3" t="n">
-        <v>5.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -592,31 +592,31 @@
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>82.40000000000001</v>
+        <v>88</v>
       </c>
       <c r="H4" t="n">
-        <v>57.7</v>
+        <v>60.8</v>
       </c>
       <c r="I4" t="n">
-        <v>31.1</v>
+        <v>30.7</v>
       </c>
       <c r="J4" t="n">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
       <c r="K4" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
       <c r="L4" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1345</v>
+        <v>1435</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Purdue</t>
+          <t>Vanderbilt</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -639,28 +639,28 @@
         <v>90</v>
       </c>
       <c r="H5" t="n">
-        <v>56.2</v>
+        <v>55.4</v>
       </c>
       <c r="I5" t="n">
-        <v>22.3</v>
+        <v>19.3</v>
       </c>
       <c r="J5" t="n">
-        <v>11.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>5.8</v>
+        <v>3.1</v>
       </c>
       <c r="L5" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1116</v>
+        <v>1458</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arkansas</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>74.2</v>
+        <v>72.7</v>
       </c>
       <c r="H6" t="n">
-        <v>34.1</v>
+        <v>35.2</v>
       </c>
       <c r="I6" t="n">
-        <v>11.7</v>
+        <v>10.8</v>
       </c>
       <c r="J6" t="n">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7">
@@ -727,16 +727,16 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>30.7</v>
+        <v>29.3</v>
       </c>
       <c r="I7" t="n">
-        <v>11.4</v>
+        <v>10.6</v>
       </c>
       <c r="J7" t="n">
-        <v>3.3</v>
+        <v>3.8</v>
       </c>
       <c r="K7" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="L7" t="n">
         <v>0.5</v>
@@ -768,13 +768,13 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>56</v>
+        <v>53.7</v>
       </c>
       <c r="H8" t="n">
-        <v>16</v>
+        <v>13.8</v>
       </c>
       <c r="I8" t="n">
-        <v>5.9</v>
+        <v>5.3</v>
       </c>
       <c r="J8" t="n">
         <v>1.6</v>
@@ -815,16 +815,16 @@
         <v>55.6</v>
       </c>
       <c r="H9" t="n">
-        <v>10.8</v>
+        <v>12.5</v>
       </c>
       <c r="I9" t="n">
-        <v>3.9</v>
+        <v>5.1</v>
       </c>
       <c r="J9" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="K9" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L9" t="n">
         <v>0.1</v>
@@ -859,10 +859,10 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>6.3</v>
+        <v>6.7</v>
       </c>
       <c r="I10" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="J10" t="n">
         <v>0.6</v>
@@ -900,19 +900,19 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>44</v>
+        <v>46.3</v>
       </c>
       <c r="H11" t="n">
-        <v>11.5</v>
+        <v>11.8</v>
       </c>
       <c r="I11" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="J11" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L11" t="n">
         <v>0.1</v>
@@ -947,10 +947,10 @@
         <v>14</v>
       </c>
       <c r="H12" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="I12" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="J12" t="n">
         <v>0.2</v>
@@ -991,10 +991,10 @@
         <v>13.6</v>
       </c>
       <c r="H13" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="I13" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>0.2</v>
@@ -1008,11 +1008,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1463</v>
+        <v>1219</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1032,13 +1032,13 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>25.8</v>
+        <v>27.3</v>
       </c>
       <c r="H14" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="J14" t="n">
         <v>0.2</v>
@@ -1052,11 +1052,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1320</v>
+        <v>1295</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1079,13 +1079,13 @@
         <v>10</v>
       </c>
       <c r="H15" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1096,11 +1096,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1295</v>
+        <v>1460</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>Wright St</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1120,13 +1120,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>17.6</v>
+        <v>12</v>
       </c>
       <c r="H16" t="n">
-        <v>3.5</v>
+        <v>1.8</v>
       </c>
       <c r="I16" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1140,11 +1140,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1398</v>
+        <v>1202</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>Furman</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1164,13 +1164,13 @@
         <v>100</v>
       </c>
       <c r="G17" t="n">
-        <v>5.1</v>
+        <v>3.7</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1184,11 +1184,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1373</v>
+        <v>1420</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Siena</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1208,13 +1208,13 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="H18" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>97.8</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>77.09999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>57.9</v>
+        <v>53.7</v>
       </c>
       <c r="J19" t="n">
-        <v>37.1</v>
+        <v>28.9</v>
       </c>
       <c r="K19" t="n">
-        <v>18.1</v>
+        <v>15.4</v>
       </c>
       <c r="L19" t="n">
-        <v>9.300000000000001</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="20">
@@ -1296,31 +1296,31 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>96.3</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>72.5</v>
+        <v>75.5</v>
       </c>
       <c r="I20" t="n">
-        <v>51.4</v>
+        <v>49.5</v>
       </c>
       <c r="J20" t="n">
-        <v>29.4</v>
+        <v>31.1</v>
       </c>
       <c r="K20" t="n">
-        <v>14.3</v>
+        <v>17.6</v>
       </c>
       <c r="L20" t="n">
-        <v>7.6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1304</v>
+        <v>1345</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nebraska</t>
+          <t>Purdue</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1343,28 +1343,28 @@
         <v>88.3</v>
       </c>
       <c r="H21" t="n">
-        <v>54.4</v>
+        <v>54.7</v>
       </c>
       <c r="I21" t="n">
-        <v>22.2</v>
+        <v>27.5</v>
       </c>
       <c r="J21" t="n">
-        <v>8.4</v>
+        <v>15.5</v>
       </c>
       <c r="K21" t="n">
-        <v>2.5</v>
+        <v>7.6</v>
       </c>
       <c r="L21" t="n">
-        <v>0.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1403</v>
+        <v>1438</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Texas Tech</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1384,31 +1384,31 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>73.09999999999999</v>
+        <v>86</v>
       </c>
       <c r="H22" t="n">
-        <v>43.1</v>
+        <v>48.2</v>
       </c>
       <c r="I22" t="n">
-        <v>15.6</v>
+        <v>17.4</v>
       </c>
       <c r="J22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K22" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="L22" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1385</v>
+        <v>1403</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>Texas Tech</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1428,31 +1428,31 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>72.7</v>
+        <v>74.3</v>
       </c>
       <c r="H23" t="n">
-        <v>40.3</v>
+        <v>40.4</v>
       </c>
       <c r="I23" t="n">
-        <v>13.7</v>
+        <v>16.4</v>
       </c>
       <c r="J23" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="K23" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="L23" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1314</v>
+        <v>1397</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>Tennessee</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1472,31 +1472,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>67.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>32.9</v>
+        <v>37.4</v>
       </c>
       <c r="I24" t="n">
-        <v>10.4</v>
+        <v>14</v>
       </c>
       <c r="J24" t="n">
-        <v>3.3</v>
+        <v>6.4</v>
       </c>
       <c r="K24" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L24" t="n">
         <v>0.8</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1388</v>
+        <v>1417</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>63.9</v>
+        <v>59.2</v>
       </c>
       <c r="H25" t="n">
-        <v>19.2</v>
+        <v>16.4</v>
       </c>
       <c r="I25" t="n">
-        <v>10</v>
+        <v>5.6</v>
       </c>
       <c r="J25" t="n">
-        <v>3.7</v>
+        <v>2.1</v>
       </c>
       <c r="K25" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26">
@@ -1560,16 +1560,16 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>59.2</v>
+        <v>55.6</v>
       </c>
       <c r="H26" t="n">
-        <v>14.5</v>
+        <v>16.5</v>
       </c>
       <c r="I26" t="n">
-        <v>6.4</v>
+        <v>6.9</v>
       </c>
       <c r="J26" t="n">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="K26" t="n">
         <v>0.6</v>
@@ -1580,11 +1580,11 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1155</v>
+        <v>1437</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Villanova</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1604,16 +1604,16 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>40.8</v>
+        <v>44.4</v>
       </c>
       <c r="H27" t="n">
-        <v>8.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="I27" t="n">
-        <v>3.3</v>
+        <v>3.5</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K27" t="n">
         <v>0.2</v>
@@ -1624,11 +1624,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1387</v>
+        <v>1401</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>St Louis</t>
+          <t>Texas A&amp;M</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1648,19 +1648,19 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>36.1</v>
+        <v>40.8</v>
       </c>
       <c r="H28" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="I28" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="J28" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1378</v>
+        <v>1275</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>South Florida</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1692,19 +1692,19 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>32.3</v>
+        <v>24.4</v>
       </c>
       <c r="H29" t="n">
-        <v>10.5</v>
+        <v>5.9</v>
       </c>
       <c r="I29" t="n">
-        <v>2.4</v>
+        <v>0.9</v>
       </c>
       <c r="J29" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -1712,11 +1712,11 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1270</v>
+        <v>1463</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>McNeese St</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1736,19 +1736,19 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>27.3</v>
+        <v>25.7</v>
       </c>
       <c r="H30" t="n">
-        <v>10.1</v>
+        <v>7.1</v>
       </c>
       <c r="I30" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="J30" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
@@ -1780,16 +1780,16 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>26.9</v>
+        <v>14</v>
       </c>
       <c r="H31" t="n">
-        <v>6.4</v>
+        <v>4.3</v>
       </c>
       <c r="I31" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1800,11 +1800,11 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1460</v>
+        <v>1407</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wright St</t>
+          <t>Troy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1827,10 +1827,10 @@
         <v>11.7</v>
       </c>
       <c r="H32" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1202</v>
+        <v>1254</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Furman</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1868,10 +1868,10 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="H33" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -1909,10 +1909,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>56.6</v>
+        <v>25.5</v>
       </c>
       <c r="G34" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1250</v>
+        <v>1256</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Lehigh</t>
+          <t>Louisiana Tech</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>43.4</v>
+        <v>74.5</v>
       </c>
       <c r="G35" t="n">
-        <v>0.9</v>
+        <v>3.6</v>
       </c>
       <c r="H35" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2000,22 +2000,22 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>95.40000000000001</v>
+        <v>96.2</v>
       </c>
       <c r="H36" t="n">
-        <v>75.8</v>
+        <v>79.3</v>
       </c>
       <c r="I36" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="J36" t="n">
-        <v>39.7</v>
+        <v>42.1</v>
       </c>
       <c r="K36" t="n">
-        <v>23.4</v>
+        <v>24.7</v>
       </c>
       <c r="L36" t="n">
-        <v>13.1</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="37">
@@ -2044,31 +2044,31 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>88.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>66.8</v>
+        <v>65.3</v>
       </c>
       <c r="I37" t="n">
-        <v>37.4</v>
+        <v>44.7</v>
       </c>
       <c r="J37" t="n">
-        <v>17.2</v>
+        <v>21</v>
       </c>
       <c r="K37" t="n">
-        <v>7.4</v>
+        <v>9</v>
       </c>
       <c r="L37" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1104</v>
+        <v>1304</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alabama</t>
+          <t>Nebraska</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>82.7</v>
+        <v>88.3</v>
       </c>
       <c r="H38" t="n">
-        <v>57</v>
+        <v>52.5</v>
       </c>
       <c r="I38" t="n">
-        <v>33.2</v>
+        <v>22</v>
       </c>
       <c r="J38" t="n">
-        <v>15.1</v>
+        <v>8.1</v>
       </c>
       <c r="K38" t="n">
-        <v>6.7</v>
+        <v>2.6</v>
       </c>
       <c r="L38" t="n">
-        <v>3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="39">
@@ -2132,31 +2132,31 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>77</v>
+        <v>72.5</v>
       </c>
       <c r="H39" t="n">
-        <v>37.6</v>
+        <v>36</v>
       </c>
       <c r="I39" t="n">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="J39" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="K39" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="L39" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1397</v>
+        <v>1116</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Tennessee</t>
+          <t>Arkansas</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2179,28 +2179,28 @@
         <v>72.8</v>
       </c>
       <c r="H40" t="n">
-        <v>47.4</v>
+        <v>44</v>
       </c>
       <c r="I40" t="n">
-        <v>17.2</v>
+        <v>15.6</v>
       </c>
       <c r="J40" t="n">
-        <v>8.800000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="K40" t="n">
-        <v>3.5</v>
+        <v>3.2</v>
       </c>
       <c r="L40" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1458</v>
+        <v>1314</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>North Carolina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2220,31 +2220,31 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>72.8</v>
+        <v>68</v>
       </c>
       <c r="H41" t="n">
-        <v>31.4</v>
+        <v>34.7</v>
       </c>
       <c r="I41" t="n">
-        <v>15.5</v>
+        <v>13</v>
       </c>
       <c r="J41" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
       <c r="K41" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="L41" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1274</v>
+        <v>1388</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Miami FL</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2264,31 +2264,31 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>55.9</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H42" t="n">
-        <v>17.2</v>
+        <v>23.8</v>
       </c>
       <c r="I42" t="n">
-        <v>6.7</v>
+        <v>12.7</v>
       </c>
       <c r="J42" t="n">
-        <v>1.8</v>
+        <v>5</v>
       </c>
       <c r="K42" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L42" t="n">
         <v>0.5</v>
-      </c>
-      <c r="L42" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1429</v>
+        <v>1155</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Utah St</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2308,19 +2308,19 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>46.4</v>
+        <v>53</v>
       </c>
       <c r="H43" t="n">
-        <v>12.1</v>
+        <v>9.9</v>
       </c>
       <c r="I43" t="n">
-        <v>5.3</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="K43" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2328,11 +2328,11 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>1234</v>
+        <v>1387</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>St Louis</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>53.6</v>
+        <v>47</v>
       </c>
       <c r="H44" t="n">
-        <v>11.8</v>
+        <v>10.3</v>
       </c>
       <c r="I44" t="n">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="J44" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="K44" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2372,11 +2372,11 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1416</v>
+        <v>1301</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>UCF</t>
+          <t>NC State</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2396,31 +2396,31 @@
         <v>100</v>
       </c>
       <c r="G45" t="n">
-        <v>44.1</v>
+        <v>35.9</v>
       </c>
       <c r="H45" t="n">
-        <v>14.1</v>
+        <v>10.4</v>
       </c>
       <c r="I45" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="J45" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="K45" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1275</v>
+        <v>1378</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2440,19 +2440,19 @@
         <v>100</v>
       </c>
       <c r="G46" t="n">
-        <v>27.2</v>
+        <v>32</v>
       </c>
       <c r="H46" t="n">
-        <v>8.199999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="I46" t="n">
-        <v>2</v>
+        <v>2.9</v>
       </c>
       <c r="J46" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2487,13 +2487,13 @@
         <v>27.2</v>
       </c>
       <c r="H47" t="n">
-        <v>12.2</v>
+        <v>11.3</v>
       </c>
       <c r="I47" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="J47" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="K47" t="n">
         <v>0.2</v>
@@ -2504,11 +2504,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1358</v>
+        <v>1320</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Sam Houston St</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>23</v>
+        <v>27.5</v>
       </c>
       <c r="H48" t="n">
-        <v>2.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I48" t="n">
-        <v>0.4</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K48" t="n">
         <v>0.1</v>
-      </c>
-      <c r="K48" t="n">
-        <v>0</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1407</v>
+        <v>1398</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Troy</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2572,16 +2572,16 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>17.3</v>
+        <v>11.7</v>
       </c>
       <c r="H49" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
       <c r="I49" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
@@ -2592,11 +2592,11 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1420</v>
+        <v>1474</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>Queens NC</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>11.7</v>
+        <v>5.1</v>
       </c>
       <c r="H50" t="n">
-        <v>1.9</v>
+        <v>0.5</v>
       </c>
       <c r="I50" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2636,11 +2636,11 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1224</v>
+        <v>1250</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Howard</t>
+          <t>Lehigh</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2657,13 +2657,13 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>41</v>
+        <v>25.7</v>
       </c>
       <c r="G51" t="n">
-        <v>1.9</v>
+        <v>0.3</v>
       </c>
       <c r="H51" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>59</v>
+        <v>74.3</v>
       </c>
       <c r="G52" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2748,22 +2748,22 @@
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>95.2</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>75.59999999999999</v>
+        <v>73.8</v>
       </c>
       <c r="I53" t="n">
-        <v>59.1</v>
+        <v>55.8</v>
       </c>
       <c r="J53" t="n">
-        <v>42.8</v>
+        <v>40.4</v>
       </c>
       <c r="K53" t="n">
-        <v>28.2</v>
+        <v>27.3</v>
       </c>
       <c r="L53" t="n">
-        <v>17.7</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="54">
@@ -2795,16 +2795,16 @@
         <v>88.5</v>
       </c>
       <c r="H54" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>38.1</v>
+        <v>37.3</v>
       </c>
       <c r="J54" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="K54" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="L54" t="n">
         <v>3.3</v>
@@ -2842,25 +2842,25 @@
         <v>56.6</v>
       </c>
       <c r="I55" t="n">
-        <v>34</v>
+        <v>34.5</v>
       </c>
       <c r="J55" t="n">
-        <v>15.2</v>
+        <v>16</v>
       </c>
       <c r="K55" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="L55" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1438</v>
+        <v>1104</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Alabama</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2880,31 +2880,31 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>83.8</v>
+        <v>76.8</v>
       </c>
       <c r="H56" t="n">
-        <v>44.5</v>
+        <v>46.2</v>
       </c>
       <c r="I56" t="n">
-        <v>13.1</v>
+        <v>17.1</v>
       </c>
       <c r="J56" t="n">
-        <v>6</v>
+        <v>8.6</v>
       </c>
       <c r="K56" t="n">
-        <v>2.2</v>
+        <v>4.1</v>
       </c>
       <c r="L56" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1435</v>
+        <v>1385</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Vanderbilt</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>75.7</v>
+        <v>72.8</v>
       </c>
       <c r="H57" t="n">
-        <v>45.7</v>
+        <v>38.9</v>
       </c>
       <c r="I57" t="n">
-        <v>16</v>
+        <v>12.9</v>
       </c>
       <c r="J57" t="n">
-        <v>7.8</v>
+        <v>6.2</v>
       </c>
       <c r="K57" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="L57" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="58">
@@ -2974,13 +2974,13 @@
         <v>30.1</v>
       </c>
       <c r="I58" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="J58" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="K58" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="L58" t="n">
         <v>0.6</v>
@@ -2988,11 +2988,11 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>1437</v>
+        <v>1274</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Villanova</t>
+          <t>Miami FL</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3012,16 +3012,16 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>53.9</v>
+        <v>55.6</v>
       </c>
       <c r="H59" t="n">
-        <v>17.8</v>
+        <v>19.4</v>
       </c>
       <c r="I59" t="n">
-        <v>5.6</v>
+        <v>6.1</v>
       </c>
       <c r="J59" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="K59" t="n">
         <v>0.4</v>
@@ -3032,11 +3032,11 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>1417</v>
+        <v>1429</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>Utah St</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3056,19 +3056,19 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>56.5</v>
+        <v>46.4</v>
       </c>
       <c r="H60" t="n">
-        <v>14.9</v>
+        <v>11.1</v>
       </c>
       <c r="I60" t="n">
-        <v>6.7</v>
+        <v>4.9</v>
       </c>
       <c r="J60" t="n">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="K60" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L60" t="n">
         <v>0.2</v>
@@ -3076,11 +3076,11 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>1401</v>
+        <v>1234</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Texas A&amp;M</t>
+          <t>Iowa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3100,31 +3100,31 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>43.5</v>
+        <v>53.6</v>
       </c>
       <c r="H61" t="n">
-        <v>9.199999999999999</v>
+        <v>14.7</v>
       </c>
       <c r="I61" t="n">
-        <v>3.3</v>
+        <v>6.3</v>
       </c>
       <c r="J61" t="n">
-        <v>1</v>
+        <v>2.3</v>
       </c>
       <c r="K61" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L61" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>1301</v>
+        <v>1416</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NC State</t>
+          <t>UCF</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3144,16 +3144,16 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>46.1</v>
+        <v>44.4</v>
       </c>
       <c r="H62" t="n">
         <v>13.8</v>
       </c>
       <c r="I62" t="n">
-        <v>3.9</v>
+        <v>3.6</v>
       </c>
       <c r="J62" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="K62" t="n">
         <v>0.2</v>
@@ -3197,7 +3197,7 @@
         <v>1.5</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K63" t="n">
         <v>0.1</v>
@@ -3235,7 +3235,7 @@
         <v>18.1</v>
       </c>
       <c r="H64" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="I64" t="n">
         <v>1.9</v>
@@ -3252,11 +3252,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1219</v>
+        <v>1270</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>McNeese St</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>24.3</v>
+        <v>27.2</v>
       </c>
       <c r="H65" t="n">
-        <v>6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I65" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="J65" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3320,13 +3320,13 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>16.2</v>
+        <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>3.8</v>
+        <v>5.1</v>
       </c>
       <c r="I66" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="J66" t="n">
         <v>0.1</v>
@@ -3370,7 +3370,7 @@
         <v>3.3</v>
       </c>
       <c r="I67" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="J67" t="n">
         <v>0.1</v>
@@ -3384,11 +3384,11 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>1474</v>
+        <v>1373</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Queens NC</t>
+          <t>Siena</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3411,10 +3411,10 @@
         <v>11.5</v>
       </c>
       <c r="H68" t="n">
-        <v>1.7</v>
+        <v>1.4</v>
       </c>
       <c r="I68" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3428,11 +3428,11 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1254</v>
+        <v>1224</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>Howard</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3452,13 +3452,13 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>4.8</v>
+        <v>5.9</v>
       </c>
       <c r="H69" t="n">
         <v>0.4</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-15)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -504,22 +504,22 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>95.2</v>
+        <v>97.2</v>
       </c>
       <c r="H2" t="n">
-        <v>80</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>60.9</v>
+        <v>59.2</v>
       </c>
       <c r="J2" t="n">
-        <v>39.1</v>
+        <v>38.3</v>
       </c>
       <c r="K2" t="n">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L2" t="n">
-        <v>14.7</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="3">
@@ -557,13 +557,13 @@
         <v>47.5</v>
       </c>
       <c r="J3" t="n">
-        <v>25.7</v>
+        <v>24.5</v>
       </c>
       <c r="K3" t="n">
-        <v>13.7</v>
+        <v>13.1</v>
       </c>
       <c r="L3" t="n">
-        <v>7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="4">
@@ -595,19 +595,19 @@
         <v>88</v>
       </c>
       <c r="H4" t="n">
-        <v>60.8</v>
+        <v>61.4</v>
       </c>
       <c r="I4" t="n">
-        <v>30.7</v>
+        <v>31</v>
       </c>
       <c r="J4" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="K4" t="n">
-        <v>6.3</v>
+        <v>6.9</v>
       </c>
       <c r="L4" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="5">
@@ -636,31 +636,31 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>90</v>
+        <v>83.8</v>
       </c>
       <c r="H5" t="n">
-        <v>55.4</v>
+        <v>50.7</v>
       </c>
       <c r="I5" t="n">
-        <v>19.3</v>
+        <v>18.6</v>
       </c>
       <c r="J5" t="n">
-        <v>8.199999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="L5" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1458</v>
+        <v>1385</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Wisconsin</t>
+          <t>St John's</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -680,22 +680,22 @@
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>72.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>35.2</v>
+        <v>37.8</v>
       </c>
       <c r="I6" t="n">
-        <v>10.8</v>
+        <v>12.6</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="K6" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
@@ -724,16 +724,16 @@
         <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>72.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="H7" t="n">
-        <v>29.3</v>
+        <v>29.6</v>
       </c>
       <c r="I7" t="n">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="J7" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="K7" t="n">
         <v>1.4</v>
@@ -788,11 +788,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1208</v>
+        <v>1326</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Ohio St</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -815,19 +815,19 @@
         <v>55.6</v>
       </c>
       <c r="H9" t="n">
-        <v>12.5</v>
+        <v>13.9</v>
       </c>
       <c r="I9" t="n">
-        <v>5.1</v>
+        <v>5.5</v>
       </c>
       <c r="J9" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="K9" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="10">
@@ -859,10 +859,10 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>6.7</v>
+        <v>6.3</v>
       </c>
       <c r="I10" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="J10" t="n">
         <v>0.6</v>
@@ -941,16 +941,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>51.1</v>
+        <v>63.9</v>
       </c>
       <c r="G12" t="n">
-        <v>14</v>
+        <v>17.6</v>
       </c>
       <c r="H12" t="n">
-        <v>3.7</v>
+        <v>4.7</v>
       </c>
       <c r="I12" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J12" t="n">
         <v>0.2</v>
@@ -964,11 +964,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1433</v>
+        <v>1275</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VCU</t>
+          <t>Miami OH</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -985,22 +985,22 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>48.9</v>
+        <v>36.1</v>
       </c>
       <c r="G13" t="n">
-        <v>13.6</v>
+        <v>9.4</v>
       </c>
       <c r="H13" t="n">
-        <v>4.3</v>
+        <v>2.5</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1008,11 +1008,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1219</v>
+        <v>1103</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>High Point</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1032,19 +1032,19 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>27.3</v>
+        <v>24.4</v>
       </c>
       <c r="H14" t="n">
-        <v>7.4</v>
+        <v>7.8</v>
       </c>
       <c r="I14" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1052,11 +1052,11 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1295</v>
+        <v>1320</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>N Dakota St</t>
+          <t>Northern Iowa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1076,16 +1076,16 @@
         <v>100</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>16.2</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1184,11 +1184,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1420</v>
+        <v>1254</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>UMBC</t>
+          <t>LIU Brooklyn</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1208,13 +1208,13 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>4.8</v>
+        <v>2.8</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>95.90000000000001</v>
+        <v>94.7</v>
       </c>
       <c r="H19" t="n">
-        <v>74.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="I19" t="n">
-        <v>53.7</v>
+        <v>47</v>
       </c>
       <c r="J19" t="n">
-        <v>28.9</v>
+        <v>25.6</v>
       </c>
       <c r="K19" t="n">
-        <v>15.4</v>
+        <v>13.6</v>
       </c>
       <c r="L19" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>97.09999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>75.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>49.5</v>
+        <v>44.2</v>
       </c>
       <c r="J20" t="n">
-        <v>31.1</v>
+        <v>26.1</v>
       </c>
       <c r="K20" t="n">
-        <v>17.6</v>
+        <v>14.3</v>
       </c>
       <c r="L20" t="n">
-        <v>10</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="21">
@@ -1343,28 +1343,28 @@
         <v>88.3</v>
       </c>
       <c r="H21" t="n">
-        <v>54.7</v>
+        <v>54</v>
       </c>
       <c r="I21" t="n">
-        <v>27.5</v>
+        <v>27.9</v>
       </c>
       <c r="J21" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="K21" t="n">
-        <v>7.6</v>
+        <v>7.9</v>
       </c>
       <c r="L21" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1438</v>
+        <v>1211</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Virginia</t>
+          <t>Gonzaga</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1384,22 +1384,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>86</v>
+        <v>88.3</v>
       </c>
       <c r="H22" t="n">
-        <v>48.2</v>
+        <v>62</v>
       </c>
       <c r="I22" t="n">
-        <v>17.4</v>
+        <v>31.8</v>
       </c>
       <c r="J22" t="n">
-        <v>6</v>
+        <v>15.5</v>
       </c>
       <c r="K22" t="n">
-        <v>1.8</v>
+        <v>6.6</v>
       </c>
       <c r="L22" t="n">
-        <v>0.6</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="23">
@@ -1431,19 +1431,19 @@
         <v>74.3</v>
       </c>
       <c r="H23" t="n">
-        <v>40.4</v>
+        <v>29.6</v>
       </c>
       <c r="I23" t="n">
-        <v>16.4</v>
+        <v>12.3</v>
       </c>
       <c r="J23" t="n">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="K23" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="L23" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="24">
@@ -1472,31 +1472,31 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>75.59999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="H24" t="n">
-        <v>37.4</v>
+        <v>36.7</v>
       </c>
       <c r="I24" t="n">
-        <v>14</v>
+        <v>15.3</v>
       </c>
       <c r="J24" t="n">
-        <v>6.4</v>
+        <v>6.7</v>
       </c>
       <c r="K24" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="L24" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1417</v>
+        <v>1388</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>UCLA</t>
+          <t>St Mary's CA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1516,31 +1516,31 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>59.2</v>
+        <v>66</v>
       </c>
       <c r="H25" t="n">
-        <v>16.4</v>
+        <v>20.6</v>
       </c>
       <c r="I25" t="n">
-        <v>5.6</v>
+        <v>8.4</v>
       </c>
       <c r="J25" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1326</v>
+        <v>1155</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ohio St</t>
+          <t>Clemson</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1560,22 +1560,22 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>55.6</v>
+        <v>53.3</v>
       </c>
       <c r="H26" t="n">
-        <v>16.5</v>
+        <v>11.8</v>
       </c>
       <c r="I26" t="n">
-        <v>6.9</v>
+        <v>3.9</v>
       </c>
       <c r="J26" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
       <c r="K26" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1604,13 +1604,13 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>44.4</v>
+        <v>46.7</v>
       </c>
       <c r="H27" t="n">
-        <v>9</v>
+        <v>10.7</v>
       </c>
       <c r="I27" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="J27" t="n">
         <v>0.8</v>
@@ -1648,16 +1648,16 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>40.8</v>
+        <v>34</v>
       </c>
       <c r="H28" t="n">
-        <v>7.9</v>
+        <v>7.2</v>
       </c>
       <c r="I28" t="n">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="J28" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K28" t="n">
         <v>0.1</v>
@@ -1668,11 +1668,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1275</v>
+        <v>1433</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Miami OH</t>
+          <t>VCU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1692,19 +1692,19 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>24.4</v>
+        <v>25.8</v>
       </c>
       <c r="H29" t="n">
-        <v>5.9</v>
+        <v>7.7</v>
       </c>
       <c r="I29" t="n">
-        <v>0.9</v>
+        <v>1.9</v>
       </c>
       <c r="J29" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -1739,13 +1739,13 @@
         <v>25.7</v>
       </c>
       <c r="H30" t="n">
-        <v>7.1</v>
+        <v>5.5</v>
       </c>
       <c r="I30" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J30" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1756,11 +1756,11 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1430</v>
+        <v>1220</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Utah Valley</t>
+          <t>Hofstra</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1780,13 +1780,13 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>14</v>
+        <v>11.7</v>
       </c>
       <c r="H31" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="I31" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J31" t="n">
         <v>0.1</v>
@@ -1827,10 +1827,10 @@
         <v>11.7</v>
       </c>
       <c r="H32" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
@@ -1844,11 +1844,11 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1254</v>
+        <v>1420</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LIU Brooklyn</t>
+          <t>UMBC</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1868,13 +1868,13 @@
         <v>100</v>
       </c>
       <c r="G33" t="n">
-        <v>2.9</v>
+        <v>5.9</v>
       </c>
       <c r="H33" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -1888,11 +1888,11 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1380</v>
+        <v>1244</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Southern Univ</t>
+          <t>Kennesaw</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1909,13 +1909,13 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>25.5</v>
+        <v>80.2</v>
       </c>
       <c r="G34" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H34" t="n">
         <v>0.6</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.1</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -1932,11 +1932,11 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1256</v>
+        <v>1341</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Louisiana Tech</t>
+          <t>Prairie View</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>74.5</v>
+        <v>19.8</v>
       </c>
       <c r="G35" t="n">
-        <v>3.6</v>
+        <v>0.5</v>
       </c>
       <c r="H35" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
@@ -2000,22 +2000,22 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>96.2</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>79.3</v>
+        <v>77.5</v>
       </c>
       <c r="I36" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J36" t="n">
-        <v>42.1</v>
+        <v>43.2</v>
       </c>
       <c r="K36" t="n">
-        <v>24.7</v>
+        <v>26.1</v>
       </c>
       <c r="L36" t="n">
-        <v>13.8</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="37">
@@ -2044,22 +2044,22 @@
         <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>94.90000000000001</v>
+        <v>94</v>
       </c>
       <c r="H37" t="n">
-        <v>65.3</v>
+        <v>59.4</v>
       </c>
       <c r="I37" t="n">
-        <v>44.7</v>
+        <v>35.3</v>
       </c>
       <c r="J37" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="K37" t="n">
-        <v>9</v>
+        <v>6.3</v>
       </c>
       <c r="L37" t="n">
-        <v>3.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="38">
@@ -2088,22 +2088,22 @@
         <v>100</v>
       </c>
       <c r="G38" t="n">
-        <v>88.3</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="H38" t="n">
-        <v>52.5</v>
+        <v>53.4</v>
       </c>
       <c r="I38" t="n">
-        <v>22</v>
+        <v>26.3</v>
       </c>
       <c r="J38" t="n">
-        <v>8.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K38" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="L38" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>72.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>36</v>
+        <v>39.7</v>
       </c>
       <c r="I39" t="n">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
       <c r="J39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K39" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="40">
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>72.8</v>
+        <v>68</v>
       </c>
       <c r="H40" t="n">
-        <v>44</v>
+        <v>41.2</v>
       </c>
       <c r="I40" t="n">
-        <v>15.6</v>
+        <v>14.9</v>
       </c>
       <c r="J40" t="n">
-        <v>8.4</v>
+        <v>8.1</v>
       </c>
       <c r="K40" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="L40" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
@@ -2223,28 +2223,28 @@
         <v>68</v>
       </c>
       <c r="H41" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="I41" t="n">
-        <v>13</v>
+        <v>16.2</v>
       </c>
       <c r="J41" t="n">
-        <v>4.6</v>
+        <v>5.9</v>
       </c>
       <c r="K41" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="L41" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1388</v>
+        <v>1417</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>St Mary's CA</t>
+          <t>UCLA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2267,13 +2267,13 @@
         <v>64.09999999999999</v>
       </c>
       <c r="H42" t="n">
-        <v>23.8</v>
+        <v>28.8</v>
       </c>
       <c r="I42" t="n">
-        <v>12.7</v>
+        <v>14.3</v>
       </c>
       <c r="J42" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="K42" t="n">
         <v>1.7</v>
@@ -2284,11 +2284,11 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1155</v>
+        <v>1208</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Clemson</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2308,22 +2308,22 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>53</v>
+        <v>55.2</v>
       </c>
       <c r="H43" t="n">
-        <v>9.9</v>
+        <v>11.8</v>
       </c>
       <c r="I43" t="n">
-        <v>4</v>
+        <v>5.4</v>
       </c>
       <c r="J43" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="K43" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="L43" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="44">
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>47</v>
+        <v>44.8</v>
       </c>
       <c r="H44" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="I44" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="J44" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="K44" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2399,10 +2399,10 @@
         <v>35.9</v>
       </c>
       <c r="H45" t="n">
-        <v>10.4</v>
+        <v>11</v>
       </c>
       <c r="I45" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="J45" t="n">
         <v>1.2</v>
@@ -2443,16 +2443,16 @@
         <v>32</v>
       </c>
       <c r="H46" t="n">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="I46" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="J46" t="n">
         <v>0.8</v>
       </c>
       <c r="K46" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2460,11 +2460,11 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1103</v>
+        <v>1270</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Akron</t>
+          <t>McNeese St</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2484,16 +2484,16 @@
         <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>27.2</v>
+        <v>32</v>
       </c>
       <c r="H47" t="n">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="I47" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="J47" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K47" t="n">
         <v>0.2</v>
@@ -2504,11 +2504,11 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1320</v>
+        <v>1465</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Northern Iowa</t>
+          <t>Cal Baptist</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2528,16 +2528,16 @@
         <v>100</v>
       </c>
       <c r="G48" t="n">
-        <v>27.5</v>
+        <v>25.6</v>
       </c>
       <c r="H48" t="n">
-        <v>8.699999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="J48" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="K48" t="n">
         <v>0.1</v>
@@ -2548,11 +2548,11 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1398</v>
+        <v>1218</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Tennessee St</t>
+          <t>Hawaii</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2572,10 +2572,10 @@
         <v>100</v>
       </c>
       <c r="G49" t="n">
-        <v>11.7</v>
+        <v>10.1</v>
       </c>
       <c r="H49" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="I49" t="n">
         <v>0.2</v>
@@ -2616,10 +2616,10 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>5.1</v>
+        <v>6</v>
       </c>
       <c r="H50" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I50" t="n">
         <v>0.1</v>
@@ -2660,10 +2660,10 @@
         <v>25.7</v>
       </c>
       <c r="G51" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -2707,7 +2707,7 @@
         <v>3.5</v>
       </c>
       <c r="H52" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2751,19 +2751,19 @@
         <v>94.09999999999999</v>
       </c>
       <c r="H53" t="n">
-        <v>73.8</v>
+        <v>72.3</v>
       </c>
       <c r="I53" t="n">
-        <v>55.8</v>
+        <v>53.9</v>
       </c>
       <c r="J53" t="n">
-        <v>40.4</v>
+        <v>41.1</v>
       </c>
       <c r="K53" t="n">
-        <v>27.3</v>
+        <v>27.7</v>
       </c>
       <c r="L53" t="n">
-        <v>17.2</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="54">
@@ -2798,25 +2798,25 @@
         <v>65.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>37.3</v>
+        <v>40.6</v>
       </c>
       <c r="J54" t="n">
-        <v>15.7</v>
+        <v>17.7</v>
       </c>
       <c r="K54" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
       <c r="L54" t="n">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>1211</v>
+        <v>1438</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Gonzaga</t>
+          <t>Virginia</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2836,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>88.09999999999999</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>56.6</v>
+        <v>54.6</v>
       </c>
       <c r="I55" t="n">
-        <v>34.5</v>
+        <v>27.9</v>
       </c>
       <c r="J55" t="n">
-        <v>16</v>
+        <v>10.3</v>
       </c>
       <c r="K55" t="n">
-        <v>8.300000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="L55" t="n">
-        <v>3.6</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="56">
@@ -2880,31 +2880,31 @@
         <v>100</v>
       </c>
       <c r="G56" t="n">
-        <v>76.8</v>
+        <v>80.3</v>
       </c>
       <c r="H56" t="n">
-        <v>46.2</v>
+        <v>49.9</v>
       </c>
       <c r="I56" t="n">
-        <v>17.1</v>
+        <v>18.7</v>
       </c>
       <c r="J56" t="n">
-        <v>8.6</v>
+        <v>10.1</v>
       </c>
       <c r="K56" t="n">
-        <v>4.1</v>
+        <v>4.9</v>
       </c>
       <c r="L56" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>1385</v>
+        <v>1458</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>St John's</t>
+          <t>Wisconsin</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2927,19 +2927,19 @@
         <v>72.8</v>
       </c>
       <c r="H57" t="n">
-        <v>38.9</v>
+        <v>36.4</v>
       </c>
       <c r="I57" t="n">
-        <v>12.9</v>
+        <v>12.3</v>
       </c>
       <c r="J57" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="K57" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="L57" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="58">
@@ -2971,19 +2971,19 @@
         <v>67.40000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>30.1</v>
+        <v>32.8</v>
       </c>
       <c r="I58" t="n">
-        <v>14.1</v>
+        <v>15.4</v>
       </c>
       <c r="J58" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="K58" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="L58" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="59">
@@ -3018,13 +3018,13 @@
         <v>19.4</v>
       </c>
       <c r="I59" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="J59" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="L59" t="n">
         <v>0.1</v>
@@ -3059,19 +3059,19 @@
         <v>46.4</v>
       </c>
       <c r="H60" t="n">
-        <v>11.1</v>
+        <v>12.6</v>
       </c>
       <c r="I60" t="n">
-        <v>4.9</v>
+        <v>6.1</v>
       </c>
       <c r="J60" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="K60" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="L60" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="61">
@@ -3106,16 +3106,16 @@
         <v>14.7</v>
       </c>
       <c r="I61" t="n">
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="J61" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="K61" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="62">
@@ -3150,10 +3150,10 @@
         <v>13.8</v>
       </c>
       <c r="I62" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="J62" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="K62" t="n">
         <v>0.2</v>
@@ -3194,7 +3194,7 @@
         <v>4.5</v>
       </c>
       <c r="I63" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="J63" t="n">
         <v>0.4</v>
@@ -3235,16 +3235,16 @@
         <v>18.1</v>
       </c>
       <c r="H64" t="n">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="I64" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="J64" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K64" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -3252,11 +3252,11 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>1270</v>
+        <v>1219</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>McNeese St</t>
+          <t>High Point</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3279,13 +3279,13 @@
         <v>27.2</v>
       </c>
       <c r="H65" t="n">
-        <v>9.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I65" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3296,11 +3296,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>1220</v>
+        <v>1295</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Hofstra</t>
+          <t>N Dakota St</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3320,13 +3320,13 @@
         <v>100</v>
       </c>
       <c r="G66" t="n">
-        <v>23.2</v>
+        <v>19.7</v>
       </c>
       <c r="H66" t="n">
-        <v>5.1</v>
+        <v>4.4</v>
       </c>
       <c r="I66" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="J66" t="n">
         <v>0.1</v>
@@ -3340,11 +3340,11 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>1414</v>
+        <v>1398</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>UC Irvine</t>
+          <t>Tennessee St</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3364,16 +3364,16 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>11.9</v>
+        <v>7.9</v>
       </c>
       <c r="H67" t="n">
-        <v>3.3</v>
+        <v>1.2</v>
       </c>
       <c r="I67" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="J67" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-16)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,62 +429,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TeamID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>TeamName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Is_FirstFour</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pct_R64</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pct_R32</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pct_S16</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pct_E8</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pct_F4</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pct_Finals</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pct_Champion</t>
         </is>
@@ -507,19 +519,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>78</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>60.6</v>
+        <v>60</v>
       </c>
       <c r="J2" t="n">
-        <v>44.1</v>
+        <v>44.6</v>
       </c>
       <c r="K2" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="L2" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="3">
@@ -548,16 +560,16 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>94.09999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="H3" t="n">
-        <v>58.7</v>
+        <v>57</v>
       </c>
       <c r="I3" t="n">
-        <v>30.4</v>
+        <v>29.5</v>
       </c>
       <c r="J3" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="K3" t="n">
         <v>4.7</v>
@@ -598,16 +610,16 @@
         <v>51.7</v>
       </c>
       <c r="I4" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="J4" t="n">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
       <c r="K4" t="n">
-        <v>7.1</v>
+        <v>6.6</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="5">
@@ -639,10 +651,10 @@
         <v>74.2</v>
       </c>
       <c r="H5" t="n">
-        <v>35.5</v>
+        <v>35.2</v>
       </c>
       <c r="I5" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="J5" t="n">
         <v>4.5</v>
@@ -683,19 +695,19 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>52.8</v>
+        <v>53.3</v>
       </c>
       <c r="I6" t="n">
-        <v>18.1</v>
+        <v>18.8</v>
       </c>
       <c r="J6" t="n">
-        <v>8.9</v>
+        <v>9.6</v>
       </c>
       <c r="K6" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="L6" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -727,19 +739,19 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>35.7</v>
       </c>
       <c r="I7" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="J7" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="K7" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8">
@@ -771,13 +783,13 @@
         <v>69.5</v>
       </c>
       <c r="H8" t="n">
-        <v>31.3</v>
+        <v>32.3</v>
       </c>
       <c r="I8" t="n">
-        <v>12.6</v>
+        <v>13.3</v>
       </c>
       <c r="J8" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="K8" t="n">
         <v>1.4</v>
@@ -818,10 +830,10 @@
         <v>14.4</v>
       </c>
       <c r="I9" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="J9" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="K9" t="n">
         <v>0.9</v>
@@ -859,16 +871,16 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -903,13 +915,13 @@
         <v>30.5</v>
       </c>
       <c r="H11" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="I11" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K11" t="n">
         <v>0.1</v>
@@ -947,7 +959,7 @@
         <v>27.6</v>
       </c>
       <c r="H12" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I12" t="n">
         <v>2.7</v>
@@ -1000,7 +1012,7 @@
         <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1035,7 +1047,7 @@
         <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="I14" t="n">
         <v>0.9</v>
@@ -1079,7 +1091,7 @@
         <v>17.6</v>
       </c>
       <c r="H15" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="I15" t="n">
         <v>0.6</v>
@@ -1120,13 +1132,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>5.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1211,19 +1223,19 @@
         <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>75</v>
+        <v>73.3</v>
       </c>
       <c r="I18" t="n">
-        <v>52.6</v>
+        <v>51.3</v>
       </c>
       <c r="J18" t="n">
-        <v>29.5</v>
+        <v>28.2</v>
       </c>
       <c r="K18" t="n">
-        <v>16.3</v>
+        <v>15.5</v>
       </c>
       <c r="L18" t="n">
-        <v>7.9</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="19">
@@ -1258,16 +1270,16 @@
         <v>71.40000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>45.6</v>
+        <v>46.4</v>
       </c>
       <c r="J19" t="n">
-        <v>28.3</v>
+        <v>29.6</v>
       </c>
       <c r="K19" t="n">
-        <v>16.4</v>
+        <v>17.5</v>
       </c>
       <c r="L19" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1302,16 +1314,16 @@
         <v>61.9</v>
       </c>
       <c r="I20" t="n">
-        <v>31.8</v>
+        <v>31</v>
       </c>
       <c r="J20" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="K20" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="L20" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1352,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>85.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>41.4</v>
+        <v>36.9</v>
       </c>
       <c r="I21" t="n">
-        <v>14.6</v>
+        <v>12.7</v>
       </c>
       <c r="J21" t="n">
-        <v>5.3</v>
+        <v>4.6</v>
       </c>
       <c r="K21" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22">
@@ -1384,22 +1396,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>75.7</v>
+        <v>77</v>
       </c>
       <c r="H22" t="n">
-        <v>48.6</v>
+        <v>53.1</v>
       </c>
       <c r="I22" t="n">
-        <v>20.5</v>
+        <v>22.8</v>
       </c>
       <c r="J22" t="n">
-        <v>9.199999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="K22" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="L22" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="23">
@@ -1431,7 +1443,7 @@
         <v>65.7</v>
       </c>
       <c r="H23" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="I23" t="n">
         <v>8</v>
@@ -1481,10 +1493,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J24" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="K24" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="L24" t="n">
         <v>0.4</v>
@@ -1519,19 +1531,19 @@
         <v>41</v>
       </c>
       <c r="H25" t="n">
-        <v>8.5</v>
+        <v>10.2</v>
       </c>
       <c r="I25" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="J25" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -1566,10 +1578,10 @@
         <v>16.3</v>
       </c>
       <c r="I26" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="J26" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="K26" t="n">
         <v>0.8</v>
@@ -1651,13 +1663,13 @@
         <v>34.3</v>
       </c>
       <c r="H28" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="I28" t="n">
         <v>2.7</v>
       </c>
       <c r="J28" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="K28" t="n">
         <v>0.2</v>
@@ -1692,10 +1704,10 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>24.3</v>
+        <v>23</v>
       </c>
       <c r="H29" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="I29" t="n">
         <v>1.9</v>
@@ -1736,10 +1748,10 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>14.7</v>
+        <v>17.4</v>
       </c>
       <c r="H30" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="I30" t="n">
         <v>0.3</v>
@@ -1783,7 +1795,7 @@
         <v>11.7</v>
       </c>
       <c r="H31" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="I31" t="n">
         <v>0.1</v>
@@ -1865,7 +1877,7 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>44.2</v>
+        <v>46.6</v>
       </c>
       <c r="G33" t="n">
         <v>1.3</v>
@@ -1909,10 +1921,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>55.8</v>
+        <v>53.4</v>
       </c>
       <c r="G34" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1956,22 +1968,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>94.7</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>76.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="I35" t="n">
-        <v>54.3</v>
+        <v>53.2</v>
       </c>
       <c r="J35" t="n">
-        <v>35.4</v>
+        <v>34</v>
       </c>
       <c r="K35" t="n">
-        <v>20.1</v>
+        <v>18.8</v>
       </c>
       <c r="L35" t="n">
-        <v>11.7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
@@ -2006,16 +2018,16 @@
         <v>73</v>
       </c>
       <c r="I36" t="n">
-        <v>50.1</v>
+        <v>50.2</v>
       </c>
       <c r="J36" t="n">
-        <v>26.9</v>
+        <v>28.1</v>
       </c>
       <c r="K36" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="L36" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="37">
@@ -2047,19 +2059,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>45.7</v>
+        <v>46</v>
       </c>
       <c r="I37" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="J37" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="K37" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="L37" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2091,19 +2103,19 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>46.8</v>
+        <v>45.5</v>
       </c>
       <c r="I38" t="n">
-        <v>20.2</v>
+        <v>19.2</v>
       </c>
       <c r="J38" t="n">
-        <v>10.1</v>
+        <v>9.5</v>
       </c>
       <c r="K38" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="L38" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="39">
@@ -2135,19 +2147,19 @@
         <v>69.2</v>
       </c>
       <c r="H39" t="n">
-        <v>36.8</v>
+        <v>38.1</v>
       </c>
       <c r="I39" t="n">
-        <v>13</v>
+        <v>14.1</v>
       </c>
       <c r="J39" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="K39" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="40">
@@ -2176,13 +2188,13 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>74.59999999999999</v>
+        <v>74.3</v>
       </c>
       <c r="H40" t="n">
-        <v>44.6</v>
+        <v>44.4</v>
       </c>
       <c r="I40" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="J40" t="n">
         <v>7.6</v>
@@ -2267,10 +2279,10 @@
         <v>55.2</v>
       </c>
       <c r="H42" t="n">
-        <v>12.2</v>
+        <v>13.4</v>
       </c>
       <c r="I42" t="n">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="J42" t="n">
         <v>1.7</v>
@@ -2311,16 +2323,16 @@
         <v>44.8</v>
       </c>
       <c r="H43" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="I43" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="J43" t="n">
         <v>1.1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2393,19 +2405,19 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>36</v>
+        <v>30.7</v>
       </c>
       <c r="G45" t="n">
-        <v>8.9</v>
+        <v>7.6</v>
       </c>
       <c r="H45" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="I45" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2437,19 +2449,19 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>64</v>
+        <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>16.6</v>
+        <v>18.1</v>
       </c>
       <c r="H46" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I46" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="J46" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K46" t="n">
         <v>0.1</v>
@@ -2487,13 +2499,13 @@
         <v>30.8</v>
       </c>
       <c r="H47" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="I47" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="J47" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2531,7 +2543,7 @@
         <v>23</v>
       </c>
       <c r="H48" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="I48" t="n">
         <v>0.7</v>
@@ -2657,16 +2669,16 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>56.7</v>
+        <v>59.4</v>
       </c>
       <c r="G51" t="n">
-        <v>3.3</v>
+        <v>7</v>
       </c>
       <c r="H51" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2701,10 +2713,10 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>43.3</v>
+        <v>40.6</v>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2751,19 +2763,19 @@
         <v>95.2</v>
       </c>
       <c r="H53" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="I53" t="n">
-        <v>57.3</v>
+        <v>56.2</v>
       </c>
       <c r="J53" t="n">
-        <v>39.6</v>
+        <v>38.7</v>
       </c>
       <c r="K53" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="L53" t="n">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="54">
@@ -2795,19 +2807,19 @@
         <v>94.3</v>
       </c>
       <c r="H54" t="n">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="I54" t="n">
-        <v>45.2</v>
+        <v>47.1</v>
       </c>
       <c r="J54" t="n">
-        <v>22.2</v>
+        <v>23.2</v>
       </c>
       <c r="K54" t="n">
-        <v>11.6</v>
+        <v>12.9</v>
       </c>
       <c r="L54" t="n">
-        <v>5.9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -2836,22 +2848,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>95.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H55" t="n">
-        <v>60.7</v>
+        <v>60.9</v>
       </c>
       <c r="I55" t="n">
-        <v>32</v>
+        <v>31.7</v>
       </c>
       <c r="J55" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="K55" t="n">
         <v>7.4</v>
       </c>
       <c r="L55" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="56">
@@ -2886,16 +2898,16 @@
         <v>46.2</v>
       </c>
       <c r="I56" t="n">
-        <v>15.7</v>
+        <v>16.4</v>
       </c>
       <c r="J56" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="K56" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="57">
@@ -2930,13 +2942,13 @@
         <v>39.9</v>
       </c>
       <c r="I57" t="n">
-        <v>13.5</v>
+        <v>12.9</v>
       </c>
       <c r="J57" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="K57" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="L57" t="n">
         <v>0.6</v>
@@ -2968,22 +2980,22 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>70.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>30.1</v>
+        <v>29.1</v>
       </c>
       <c r="I58" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="J58" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="K58" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="L58" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="59">
@@ -3015,10 +3027,10 @@
         <v>55.6</v>
       </c>
       <c r="H59" t="n">
-        <v>16.5</v>
+        <v>15.6</v>
       </c>
       <c r="I59" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="J59" t="n">
         <v>1.3</v>
@@ -3056,22 +3068,22 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>44.1</v>
+        <v>33.8</v>
       </c>
       <c r="H60" t="n">
-        <v>9.199999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="I60" t="n">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="K60" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L60" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -3100,22 +3112,22 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>55.9</v>
+        <v>66.2</v>
       </c>
       <c r="H61" t="n">
-        <v>14.8</v>
+        <v>17.5</v>
       </c>
       <c r="I61" t="n">
-        <v>7.2</v>
+        <v>9.1</v>
       </c>
       <c r="J61" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="K61" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="L61" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="62">
@@ -3147,10 +3159,10 @@
         <v>44.4</v>
       </c>
       <c r="H62" t="n">
-        <v>9.9</v>
+        <v>8.9</v>
       </c>
       <c r="I62" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="J62" t="n">
         <v>0.6</v>
@@ -3185,16 +3197,16 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>45.9</v>
+        <v>51</v>
       </c>
       <c r="G63" t="n">
-        <v>12.5</v>
+        <v>16.2</v>
       </c>
       <c r="H63" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="J63" t="n">
         <v>0.3</v>
@@ -3229,19 +3241,19 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>54.1</v>
+        <v>49</v>
       </c>
       <c r="G64" t="n">
-        <v>17.3</v>
+        <v>15.7</v>
       </c>
       <c r="H64" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I64" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K64" t="n">
         <v>0.1</v>
@@ -3279,10 +3291,10 @@
         <v>27.2</v>
       </c>
       <c r="H65" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="I65" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="J65" t="n">
         <v>0.4</v>
@@ -3323,7 +3335,7 @@
         <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="I66" t="n">
         <v>0.4</v>
@@ -3364,10 +3376,10 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="H67" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I67" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Revert "Update bracket sim outputs (2026-03-16)"
This reverts commit b6dc8acbc1d949d9b3ef0b66804f5e87d39653c0.
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,62 +417,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>TeamID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>TeamName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Is_FirstFour</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>pct_R64</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>pct_R32</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pct_S16</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>pct_E8</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pct_F4</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pct_Finals</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pct_Champion</t>
         </is>
@@ -519,19 +507,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>77.09999999999999</v>
+        <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>60</v>
+        <v>60.6</v>
       </c>
       <c r="J2" t="n">
-        <v>44.6</v>
+        <v>44.1</v>
       </c>
       <c r="K2" t="n">
-        <v>28.2</v>
+        <v>28.1</v>
       </c>
       <c r="L2" t="n">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="3">
@@ -560,16 +548,16 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>91.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>57</v>
+        <v>58.7</v>
       </c>
       <c r="I3" t="n">
-        <v>29.5</v>
+        <v>30.4</v>
       </c>
       <c r="J3" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="K3" t="n">
         <v>4.7</v>
@@ -610,16 +598,16 @@
         <v>51.7</v>
       </c>
       <c r="I4" t="n">
-        <v>32.7</v>
+        <v>32.5</v>
       </c>
       <c r="J4" t="n">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="K4" t="n">
-        <v>6.6</v>
+        <v>7.1</v>
       </c>
       <c r="L4" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -651,10 +639,10 @@
         <v>74.2</v>
       </c>
       <c r="H5" t="n">
-        <v>35.2</v>
+        <v>35.5</v>
       </c>
       <c r="I5" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="J5" t="n">
         <v>4.5</v>
@@ -695,19 +683,19 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>53.3</v>
+        <v>52.8</v>
       </c>
       <c r="I6" t="n">
-        <v>18.8</v>
+        <v>18.1</v>
       </c>
       <c r="J6" t="n">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="K6" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="7">
@@ -739,19 +727,19 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>35.7</v>
+        <v>36</v>
       </c>
       <c r="I7" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="J7" t="n">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="K7" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8">
@@ -783,13 +771,13 @@
         <v>69.5</v>
       </c>
       <c r="H8" t="n">
-        <v>32.3</v>
+        <v>31.3</v>
       </c>
       <c r="I8" t="n">
-        <v>13.3</v>
+        <v>12.6</v>
       </c>
       <c r="J8" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="K8" t="n">
         <v>1.4</v>
@@ -830,10 +818,10 @@
         <v>14.4</v>
       </c>
       <c r="I9" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
       <c r="J9" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="K9" t="n">
         <v>0.9</v>
@@ -871,16 +859,16 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="J10" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -915,13 +903,13 @@
         <v>30.5</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>9.5</v>
       </c>
       <c r="I11" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K11" t="n">
         <v>0.1</v>
@@ -959,7 +947,7 @@
         <v>27.6</v>
       </c>
       <c r="H12" t="n">
-        <v>9.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="I12" t="n">
         <v>2.7</v>
@@ -1012,7 +1000,7 @@
         <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1047,7 +1035,7 @@
         <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="I14" t="n">
         <v>0.9</v>
@@ -1091,7 +1079,7 @@
         <v>17.6</v>
       </c>
       <c r="H15" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="I15" t="n">
         <v>0.6</v>
@@ -1132,13 +1120,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>8.699999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="H16" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1223,19 +1211,19 @@
         <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>73.3</v>
+        <v>75</v>
       </c>
       <c r="I18" t="n">
-        <v>51.3</v>
+        <v>52.6</v>
       </c>
       <c r="J18" t="n">
-        <v>28.2</v>
+        <v>29.5</v>
       </c>
       <c r="K18" t="n">
-        <v>15.5</v>
+        <v>16.3</v>
       </c>
       <c r="L18" t="n">
-        <v>7.4</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="19">
@@ -1270,16 +1258,16 @@
         <v>71.40000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>46.4</v>
+        <v>45.6</v>
       </c>
       <c r="J19" t="n">
-        <v>29.6</v>
+        <v>28.3</v>
       </c>
       <c r="K19" t="n">
-        <v>17.5</v>
+        <v>16.4</v>
       </c>
       <c r="L19" t="n">
-        <v>9.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1314,16 +1302,16 @@
         <v>61.9</v>
       </c>
       <c r="I20" t="n">
-        <v>31</v>
+        <v>31.8</v>
       </c>
       <c r="J20" t="n">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="K20" t="n">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="L20" t="n">
-        <v>3.3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="21">
@@ -1352,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>82.59999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="H21" t="n">
-        <v>36.9</v>
+        <v>41.4</v>
       </c>
       <c r="I21" t="n">
-        <v>12.7</v>
+        <v>14.6</v>
       </c>
       <c r="J21" t="n">
-        <v>4.6</v>
+        <v>5.3</v>
       </c>
       <c r="K21" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22">
@@ -1396,22 +1384,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>77</v>
+        <v>75.7</v>
       </c>
       <c r="H22" t="n">
-        <v>53.1</v>
+        <v>48.6</v>
       </c>
       <c r="I22" t="n">
-        <v>22.8</v>
+        <v>20.5</v>
       </c>
       <c r="J22" t="n">
-        <v>10.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K22" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="L22" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="23">
@@ -1443,7 +1431,7 @@
         <v>65.7</v>
       </c>
       <c r="H23" t="n">
-        <v>25</v>
+        <v>24.8</v>
       </c>
       <c r="I23" t="n">
         <v>8</v>
@@ -1493,10 +1481,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J24" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="K24" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="L24" t="n">
         <v>0.4</v>
@@ -1531,19 +1519,19 @@
         <v>41</v>
       </c>
       <c r="H25" t="n">
-        <v>10.2</v>
+        <v>8.5</v>
       </c>
       <c r="I25" t="n">
-        <v>3.7</v>
+        <v>3</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1578,10 +1566,10 @@
         <v>16.3</v>
       </c>
       <c r="I26" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="J26" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="K26" t="n">
         <v>0.8</v>
@@ -1663,13 +1651,13 @@
         <v>34.3</v>
       </c>
       <c r="H28" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="I28" t="n">
         <v>2.7</v>
       </c>
       <c r="J28" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="K28" t="n">
         <v>0.2</v>
@@ -1704,10 +1692,10 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>23</v>
+        <v>24.3</v>
       </c>
       <c r="H29" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="I29" t="n">
         <v>1.9</v>
@@ -1748,10 +1736,10 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>17.4</v>
+        <v>14.7</v>
       </c>
       <c r="H30" t="n">
-        <v>2.1</v>
+        <v>1.8</v>
       </c>
       <c r="I30" t="n">
         <v>0.3</v>
@@ -1795,7 +1783,7 @@
         <v>11.7</v>
       </c>
       <c r="H31" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="I31" t="n">
         <v>0.1</v>
@@ -1877,7 +1865,7 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>46.6</v>
+        <v>44.2</v>
       </c>
       <c r="G33" t="n">
         <v>1.3</v>
@@ -1921,10 +1909,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>53.4</v>
+        <v>55.8</v>
       </c>
       <c r="G34" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1968,22 +1956,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>91.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="H35" t="n">
-        <v>73.90000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="I35" t="n">
-        <v>53.2</v>
+        <v>54.3</v>
       </c>
       <c r="J35" t="n">
-        <v>34</v>
+        <v>35.4</v>
       </c>
       <c r="K35" t="n">
-        <v>18.8</v>
+        <v>20.1</v>
       </c>
       <c r="L35" t="n">
-        <v>11</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="36">
@@ -2018,16 +2006,16 @@
         <v>73</v>
       </c>
       <c r="I36" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="J36" t="n">
-        <v>28.1</v>
+        <v>26.9</v>
       </c>
       <c r="K36" t="n">
-        <v>13.7</v>
+        <v>13.5</v>
       </c>
       <c r="L36" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="37">
@@ -2059,19 +2047,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>46</v>
+        <v>45.7</v>
       </c>
       <c r="I37" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="J37" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="K37" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="38">
@@ -2103,19 +2091,19 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>45.5</v>
+        <v>46.8</v>
       </c>
       <c r="I38" t="n">
-        <v>19.2</v>
+        <v>20.2</v>
       </c>
       <c r="J38" t="n">
-        <v>9.5</v>
+        <v>10.1</v>
       </c>
       <c r="K38" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="L38" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="39">
@@ -2147,19 +2135,19 @@
         <v>69.2</v>
       </c>
       <c r="H39" t="n">
-        <v>38.1</v>
+        <v>36.8</v>
       </c>
       <c r="I39" t="n">
-        <v>14.1</v>
+        <v>13</v>
       </c>
       <c r="J39" t="n">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="K39" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="L39" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="40">
@@ -2188,13 +2176,13 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>74.3</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="H40" t="n">
-        <v>44.4</v>
+        <v>44.6</v>
       </c>
       <c r="I40" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="J40" t="n">
         <v>7.6</v>
@@ -2279,10 +2267,10 @@
         <v>55.2</v>
       </c>
       <c r="H42" t="n">
-        <v>13.4</v>
+        <v>12.2</v>
       </c>
       <c r="I42" t="n">
-        <v>5.8</v>
+        <v>5.3</v>
       </c>
       <c r="J42" t="n">
         <v>1.7</v>
@@ -2323,16 +2311,16 @@
         <v>44.8</v>
       </c>
       <c r="H43" t="n">
-        <v>11.5</v>
+        <v>10.4</v>
       </c>
       <c r="I43" t="n">
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
       <c r="J43" t="n">
         <v>1.1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2405,19 +2393,19 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>30.7</v>
+        <v>36</v>
       </c>
       <c r="G45" t="n">
-        <v>7.6</v>
+        <v>8.9</v>
       </c>
       <c r="H45" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
       <c r="I45" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2449,19 +2437,19 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>69.3</v>
+        <v>64</v>
       </c>
       <c r="G46" t="n">
-        <v>18.1</v>
+        <v>16.6</v>
       </c>
       <c r="H46" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="I46" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="J46" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K46" t="n">
         <v>0.1</v>
@@ -2499,13 +2487,13 @@
         <v>30.8</v>
       </c>
       <c r="H47" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="I47" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="J47" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2543,7 +2531,7 @@
         <v>23</v>
       </c>
       <c r="H48" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="I48" t="n">
         <v>0.7</v>
@@ -2669,16 +2657,16 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>59.4</v>
+        <v>56.7</v>
       </c>
       <c r="G51" t="n">
-        <v>7</v>
+        <v>3.3</v>
       </c>
       <c r="H51" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="I51" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2713,10 +2701,10 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>40.6</v>
+        <v>43.3</v>
       </c>
       <c r="G52" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2763,19 +2751,19 @@
         <v>95.2</v>
       </c>
       <c r="H53" t="n">
-        <v>75</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="I53" t="n">
-        <v>56.2</v>
+        <v>57.3</v>
       </c>
       <c r="J53" t="n">
-        <v>38.7</v>
+        <v>39.6</v>
       </c>
       <c r="K53" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="L53" t="n">
-        <v>16.5</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="54">
@@ -2807,19 +2795,19 @@
         <v>94.3</v>
       </c>
       <c r="H54" t="n">
-        <v>74.7</v>
+        <v>72.7</v>
       </c>
       <c r="I54" t="n">
-        <v>47.1</v>
+        <v>45.2</v>
       </c>
       <c r="J54" t="n">
-        <v>23.2</v>
+        <v>22.2</v>
       </c>
       <c r="K54" t="n">
-        <v>12.9</v>
+        <v>11.6</v>
       </c>
       <c r="L54" t="n">
-        <v>7</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="55">
@@ -2848,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>94.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>60.9</v>
+        <v>60.7</v>
       </c>
       <c r="I55" t="n">
-        <v>31.7</v>
+        <v>32</v>
       </c>
       <c r="J55" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="K55" t="n">
         <v>7.4</v>
       </c>
       <c r="L55" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="56">
@@ -2898,16 +2886,16 @@
         <v>46.2</v>
       </c>
       <c r="I56" t="n">
-        <v>16.4</v>
+        <v>15.7</v>
       </c>
       <c r="J56" t="n">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="K56" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="L56" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -2942,13 +2930,13 @@
         <v>39.9</v>
       </c>
       <c r="I57" t="n">
-        <v>12.9</v>
+        <v>13.5</v>
       </c>
       <c r="J57" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="K57" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="L57" t="n">
         <v>0.6</v>
@@ -2980,22 +2968,22 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>68.09999999999999</v>
+        <v>70.2</v>
       </c>
       <c r="H58" t="n">
-        <v>29.1</v>
+        <v>30.1</v>
       </c>
       <c r="I58" t="n">
-        <v>11.5</v>
+        <v>12.6</v>
       </c>
       <c r="J58" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="K58" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="L58" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="59">
@@ -3027,10 +3015,10 @@
         <v>55.6</v>
       </c>
       <c r="H59" t="n">
-        <v>15.6</v>
+        <v>16.5</v>
       </c>
       <c r="I59" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="J59" t="n">
         <v>1.3</v>
@@ -3068,22 +3056,22 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>33.8</v>
+        <v>44.1</v>
       </c>
       <c r="H60" t="n">
-        <v>7.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I60" t="n">
-        <v>2.7</v>
+        <v>3.6</v>
       </c>
       <c r="J60" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="K60" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L60" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="61">
@@ -3112,22 +3100,22 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>66.2</v>
+        <v>55.9</v>
       </c>
       <c r="H61" t="n">
-        <v>17.5</v>
+        <v>14.8</v>
       </c>
       <c r="I61" t="n">
-        <v>9.1</v>
+        <v>7.2</v>
       </c>
       <c r="J61" t="n">
-        <v>3.5</v>
+        <v>2.7</v>
       </c>
       <c r="K61" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="L61" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="62">
@@ -3159,10 +3147,10 @@
         <v>44.4</v>
       </c>
       <c r="H62" t="n">
-        <v>8.9</v>
+        <v>9.9</v>
       </c>
       <c r="I62" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="J62" t="n">
         <v>0.6</v>
@@ -3197,16 +3185,16 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>51</v>
+        <v>45.9</v>
       </c>
       <c r="G63" t="n">
-        <v>16.2</v>
+        <v>12.5</v>
       </c>
       <c r="H63" t="n">
-        <v>4.6</v>
+        <v>3.5</v>
       </c>
       <c r="I63" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
         <v>0.3</v>
@@ -3241,19 +3229,19 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>49</v>
+        <v>54.1</v>
       </c>
       <c r="G64" t="n">
-        <v>15.7</v>
+        <v>17.3</v>
       </c>
       <c r="H64" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="I64" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="J64" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K64" t="n">
         <v>0.1</v>
@@ -3291,10 +3279,10 @@
         <v>27.2</v>
       </c>
       <c r="H65" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="I65" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="J65" t="n">
         <v>0.4</v>
@@ -3335,7 +3323,7 @@
         <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="I66" t="n">
         <v>0.4</v>
@@ -3376,10 +3364,10 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="H67" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="I67" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Reapply "Update bracket sim outputs (2026-03-16)"
This reverts commit 83d1e4110bb7670065c91499991ffbe721311947.
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,62 +429,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TeamID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>TeamName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Is_FirstFour</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pct_R64</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>pct_R32</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pct_S16</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>pct_E8</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pct_F4</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pct_Finals</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pct_Champion</t>
         </is>
@@ -507,19 +519,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>78</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>60.6</v>
+        <v>60</v>
       </c>
       <c r="J2" t="n">
-        <v>44.1</v>
+        <v>44.6</v>
       </c>
       <c r="K2" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="L2" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="3">
@@ -548,16 +560,16 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>94.09999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="H3" t="n">
-        <v>58.7</v>
+        <v>57</v>
       </c>
       <c r="I3" t="n">
-        <v>30.4</v>
+        <v>29.5</v>
       </c>
       <c r="J3" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="K3" t="n">
         <v>4.7</v>
@@ -598,16 +610,16 @@
         <v>51.7</v>
       </c>
       <c r="I4" t="n">
-        <v>32.5</v>
+        <v>32.7</v>
       </c>
       <c r="J4" t="n">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
       <c r="K4" t="n">
-        <v>7.1</v>
+        <v>6.6</v>
       </c>
       <c r="L4" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="5">
@@ -639,10 +651,10 @@
         <v>74.2</v>
       </c>
       <c r="H5" t="n">
-        <v>35.5</v>
+        <v>35.2</v>
       </c>
       <c r="I5" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="J5" t="n">
         <v>4.5</v>
@@ -683,19 +695,19 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>52.8</v>
+        <v>53.3</v>
       </c>
       <c r="I6" t="n">
-        <v>18.1</v>
+        <v>18.8</v>
       </c>
       <c r="J6" t="n">
-        <v>8.9</v>
+        <v>9.6</v>
       </c>
       <c r="K6" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="L6" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -727,19 +739,19 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>35.7</v>
       </c>
       <c r="I7" t="n">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="J7" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="K7" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8">
@@ -771,13 +783,13 @@
         <v>69.5</v>
       </c>
       <c r="H8" t="n">
-        <v>31.3</v>
+        <v>32.3</v>
       </c>
       <c r="I8" t="n">
-        <v>12.6</v>
+        <v>13.3</v>
       </c>
       <c r="J8" t="n">
-        <v>4.2</v>
+        <v>4.4</v>
       </c>
       <c r="K8" t="n">
         <v>1.4</v>
@@ -818,10 +830,10 @@
         <v>14.4</v>
       </c>
       <c r="I9" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="J9" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="K9" t="n">
         <v>0.9</v>
@@ -859,16 +871,16 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -903,13 +915,13 @@
         <v>30.5</v>
       </c>
       <c r="H11" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
       <c r="I11" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K11" t="n">
         <v>0.1</v>
@@ -947,7 +959,7 @@
         <v>27.6</v>
       </c>
       <c r="H12" t="n">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I12" t="n">
         <v>2.7</v>
@@ -1000,7 +1012,7 @@
         <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1035,7 +1047,7 @@
         <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="I14" t="n">
         <v>0.9</v>
@@ -1079,7 +1091,7 @@
         <v>17.6</v>
       </c>
       <c r="H15" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="I15" t="n">
         <v>0.6</v>
@@ -1120,13 +1132,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>5.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1211,19 +1223,19 @@
         <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>75</v>
+        <v>73.3</v>
       </c>
       <c r="I18" t="n">
-        <v>52.6</v>
+        <v>51.3</v>
       </c>
       <c r="J18" t="n">
-        <v>29.5</v>
+        <v>28.2</v>
       </c>
       <c r="K18" t="n">
-        <v>16.3</v>
+        <v>15.5</v>
       </c>
       <c r="L18" t="n">
-        <v>7.9</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="19">
@@ -1258,16 +1270,16 @@
         <v>71.40000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>45.6</v>
+        <v>46.4</v>
       </c>
       <c r="J19" t="n">
-        <v>28.3</v>
+        <v>29.6</v>
       </c>
       <c r="K19" t="n">
-        <v>16.4</v>
+        <v>17.5</v>
       </c>
       <c r="L19" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1302,16 +1314,16 @@
         <v>61.9</v>
       </c>
       <c r="I20" t="n">
-        <v>31.8</v>
+        <v>31</v>
       </c>
       <c r="J20" t="n">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="K20" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="L20" t="n">
-        <v>3.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1352,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>85.3</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>41.4</v>
+        <v>36.9</v>
       </c>
       <c r="I21" t="n">
-        <v>14.6</v>
+        <v>12.7</v>
       </c>
       <c r="J21" t="n">
-        <v>5.3</v>
+        <v>4.6</v>
       </c>
       <c r="K21" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22">
@@ -1384,22 +1396,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>75.7</v>
+        <v>77</v>
       </c>
       <c r="H22" t="n">
-        <v>48.6</v>
+        <v>53.1</v>
       </c>
       <c r="I22" t="n">
-        <v>20.5</v>
+        <v>22.8</v>
       </c>
       <c r="J22" t="n">
-        <v>9.199999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="K22" t="n">
-        <v>3.9</v>
+        <v>4.4</v>
       </c>
       <c r="L22" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="23">
@@ -1431,7 +1443,7 @@
         <v>65.7</v>
       </c>
       <c r="H23" t="n">
-        <v>24.8</v>
+        <v>25</v>
       </c>
       <c r="I23" t="n">
         <v>8</v>
@@ -1481,10 +1493,10 @@
         <v>9.199999999999999</v>
       </c>
       <c r="J24" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="K24" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="L24" t="n">
         <v>0.4</v>
@@ -1519,19 +1531,19 @@
         <v>41</v>
       </c>
       <c r="H25" t="n">
-        <v>8.5</v>
+        <v>10.2</v>
       </c>
       <c r="I25" t="n">
-        <v>3</v>
+        <v>3.7</v>
       </c>
       <c r="J25" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26">
@@ -1566,10 +1578,10 @@
         <v>16.3</v>
       </c>
       <c r="I26" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="J26" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="K26" t="n">
         <v>0.8</v>
@@ -1651,13 +1663,13 @@
         <v>34.3</v>
       </c>
       <c r="H28" t="n">
-        <v>11.4</v>
+        <v>11.2</v>
       </c>
       <c r="I28" t="n">
         <v>2.7</v>
       </c>
       <c r="J28" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="K28" t="n">
         <v>0.2</v>
@@ -1692,10 +1704,10 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>24.3</v>
+        <v>23</v>
       </c>
       <c r="H29" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="I29" t="n">
         <v>1.9</v>
@@ -1736,10 +1748,10 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>14.7</v>
+        <v>17.4</v>
       </c>
       <c r="H30" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="I30" t="n">
         <v>0.3</v>
@@ -1783,7 +1795,7 @@
         <v>11.7</v>
       </c>
       <c r="H31" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="I31" t="n">
         <v>0.1</v>
@@ -1865,7 +1877,7 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>44.2</v>
+        <v>46.6</v>
       </c>
       <c r="G33" t="n">
         <v>1.3</v>
@@ -1909,10 +1921,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>55.8</v>
+        <v>53.4</v>
       </c>
       <c r="G34" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1956,22 +1968,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>94.7</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>76.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="I35" t="n">
-        <v>54.3</v>
+        <v>53.2</v>
       </c>
       <c r="J35" t="n">
-        <v>35.4</v>
+        <v>34</v>
       </c>
       <c r="K35" t="n">
-        <v>20.1</v>
+        <v>18.8</v>
       </c>
       <c r="L35" t="n">
-        <v>11.7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36">
@@ -2006,16 +2018,16 @@
         <v>73</v>
       </c>
       <c r="I36" t="n">
-        <v>50.1</v>
+        <v>50.2</v>
       </c>
       <c r="J36" t="n">
-        <v>26.9</v>
+        <v>28.1</v>
       </c>
       <c r="K36" t="n">
-        <v>13.5</v>
+        <v>13.7</v>
       </c>
       <c r="L36" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="37">
@@ -2047,19 +2059,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>45.7</v>
+        <v>46</v>
       </c>
       <c r="I37" t="n">
-        <v>18.6</v>
+        <v>18.8</v>
       </c>
       <c r="J37" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="K37" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="L37" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2091,19 +2103,19 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>46.8</v>
+        <v>45.5</v>
       </c>
       <c r="I38" t="n">
-        <v>20.2</v>
+        <v>19.2</v>
       </c>
       <c r="J38" t="n">
-        <v>10.1</v>
+        <v>9.5</v>
       </c>
       <c r="K38" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="L38" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="39">
@@ -2135,19 +2147,19 @@
         <v>69.2</v>
       </c>
       <c r="H39" t="n">
-        <v>36.8</v>
+        <v>38.1</v>
       </c>
       <c r="I39" t="n">
-        <v>13</v>
+        <v>14.1</v>
       </c>
       <c r="J39" t="n">
-        <v>5.5</v>
+        <v>5.9</v>
       </c>
       <c r="K39" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="40">
@@ -2176,13 +2188,13 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>74.59999999999999</v>
+        <v>74.3</v>
       </c>
       <c r="H40" t="n">
-        <v>44.6</v>
+        <v>44.4</v>
       </c>
       <c r="I40" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="J40" t="n">
         <v>7.6</v>
@@ -2267,10 +2279,10 @@
         <v>55.2</v>
       </c>
       <c r="H42" t="n">
-        <v>12.2</v>
+        <v>13.4</v>
       </c>
       <c r="I42" t="n">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="J42" t="n">
         <v>1.7</v>
@@ -2311,16 +2323,16 @@
         <v>44.8</v>
       </c>
       <c r="H43" t="n">
-        <v>10.4</v>
+        <v>11.5</v>
       </c>
       <c r="I43" t="n">
-        <v>3.9</v>
+        <v>4.3</v>
       </c>
       <c r="J43" t="n">
         <v>1.1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2393,19 +2405,19 @@
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>36</v>
+        <v>30.7</v>
       </c>
       <c r="G45" t="n">
-        <v>8.9</v>
+        <v>7.6</v>
       </c>
       <c r="H45" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="I45" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2437,19 +2449,19 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>64</v>
+        <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>16.6</v>
+        <v>18.1</v>
       </c>
       <c r="H46" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I46" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="J46" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K46" t="n">
         <v>0.1</v>
@@ -2487,13 +2499,13 @@
         <v>30.8</v>
       </c>
       <c r="H47" t="n">
-        <v>11.2</v>
+        <v>11</v>
       </c>
       <c r="I47" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="J47" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2531,7 +2543,7 @@
         <v>23</v>
       </c>
       <c r="H48" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="I48" t="n">
         <v>0.7</v>
@@ -2657,16 +2669,16 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>56.7</v>
+        <v>59.4</v>
       </c>
       <c r="G51" t="n">
-        <v>3.3</v>
+        <v>7</v>
       </c>
       <c r="H51" t="n">
-        <v>0.4</v>
+        <v>1.1</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2701,10 +2713,10 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>43.3</v>
+        <v>40.6</v>
       </c>
       <c r="G52" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2751,19 +2763,19 @@
         <v>95.2</v>
       </c>
       <c r="H53" t="n">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
       <c r="I53" t="n">
-        <v>57.3</v>
+        <v>56.2</v>
       </c>
       <c r="J53" t="n">
-        <v>39.6</v>
+        <v>38.7</v>
       </c>
       <c r="K53" t="n">
-        <v>25.9</v>
+        <v>25.8</v>
       </c>
       <c r="L53" t="n">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="54">
@@ -2795,19 +2807,19 @@
         <v>94.3</v>
       </c>
       <c r="H54" t="n">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="I54" t="n">
-        <v>45.2</v>
+        <v>47.1</v>
       </c>
       <c r="J54" t="n">
-        <v>22.2</v>
+        <v>23.2</v>
       </c>
       <c r="K54" t="n">
-        <v>11.6</v>
+        <v>12.9</v>
       </c>
       <c r="L54" t="n">
-        <v>5.9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -2836,22 +2848,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>95.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H55" t="n">
-        <v>60.7</v>
+        <v>60.9</v>
       </c>
       <c r="I55" t="n">
-        <v>32</v>
+        <v>31.7</v>
       </c>
       <c r="J55" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="K55" t="n">
         <v>7.4</v>
       </c>
       <c r="L55" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="56">
@@ -2886,16 +2898,16 @@
         <v>46.2</v>
       </c>
       <c r="I56" t="n">
-        <v>15.7</v>
+        <v>16.4</v>
       </c>
       <c r="J56" t="n">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="K56" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="L56" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="57">
@@ -2930,13 +2942,13 @@
         <v>39.9</v>
       </c>
       <c r="I57" t="n">
-        <v>13.5</v>
+        <v>12.9</v>
       </c>
       <c r="J57" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="K57" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="L57" t="n">
         <v>0.6</v>
@@ -2968,22 +2980,22 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>70.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>30.1</v>
+        <v>29.1</v>
       </c>
       <c r="I58" t="n">
-        <v>12.6</v>
+        <v>11.5</v>
       </c>
       <c r="J58" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="K58" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="L58" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="59">
@@ -3015,10 +3027,10 @@
         <v>55.6</v>
       </c>
       <c r="H59" t="n">
-        <v>16.5</v>
+        <v>15.6</v>
       </c>
       <c r="I59" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="J59" t="n">
         <v>1.3</v>
@@ -3056,22 +3068,22 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>44.1</v>
+        <v>33.8</v>
       </c>
       <c r="H60" t="n">
-        <v>9.199999999999999</v>
+        <v>7.1</v>
       </c>
       <c r="I60" t="n">
-        <v>3.6</v>
+        <v>2.7</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="K60" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L60" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -3100,22 +3112,22 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>55.9</v>
+        <v>66.2</v>
       </c>
       <c r="H61" t="n">
-        <v>14.8</v>
+        <v>17.5</v>
       </c>
       <c r="I61" t="n">
-        <v>7.2</v>
+        <v>9.1</v>
       </c>
       <c r="J61" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="K61" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="L61" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="62">
@@ -3147,10 +3159,10 @@
         <v>44.4</v>
       </c>
       <c r="H62" t="n">
-        <v>9.9</v>
+        <v>8.9</v>
       </c>
       <c r="I62" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="J62" t="n">
         <v>0.6</v>
@@ -3185,16 +3197,16 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>45.9</v>
+        <v>51</v>
       </c>
       <c r="G63" t="n">
-        <v>12.5</v>
+        <v>16.2</v>
       </c>
       <c r="H63" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="J63" t="n">
         <v>0.3</v>
@@ -3229,19 +3241,19 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>54.1</v>
+        <v>49</v>
       </c>
       <c r="G64" t="n">
-        <v>17.3</v>
+        <v>15.7</v>
       </c>
       <c r="H64" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I64" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K64" t="n">
         <v>0.1</v>
@@ -3279,10 +3291,10 @@
         <v>27.2</v>
       </c>
       <c r="H65" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="I65" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="J65" t="n">
         <v>0.4</v>
@@ -3323,7 +3335,7 @@
         <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="I66" t="n">
         <v>0.4</v>
@@ -3364,10 +3376,10 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="H67" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I67" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-18)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -1956,22 +1956,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>91.09999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="H35" t="n">
-        <v>74.09999999999999</v>
+        <v>73.8</v>
       </c>
       <c r="I35" t="n">
-        <v>52.1</v>
+        <v>51.9</v>
       </c>
       <c r="J35" t="n">
-        <v>33.1</v>
+        <v>33</v>
       </c>
       <c r="K35" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="L35" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="36">
@@ -2094,7 +2094,7 @@
         <v>45.5</v>
       </c>
       <c r="I38" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="J38" t="n">
         <v>10</v>
@@ -2267,7 +2267,7 @@
         <v>55.2</v>
       </c>
       <c r="H42" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="I42" t="n">
         <v>5.8</v>
@@ -2311,7 +2311,7 @@
         <v>44.8</v>
       </c>
       <c r="H43" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="I43" t="n">
         <v>4.3</v>
@@ -2657,10 +2657,10 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>59.4</v>
+        <v>63.9</v>
       </c>
       <c r="G51" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="n">
         <v>1.1</v>
@@ -2701,10 +2701,10 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>40.6</v>
+        <v>36.1</v>
       </c>
       <c r="G52" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2760,7 +2760,7 @@
         <v>38.6</v>
       </c>
       <c r="K53" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="L53" t="n">
         <v>16.4</v>
@@ -2798,7 +2798,7 @@
         <v>74.7</v>
       </c>
       <c r="I54" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
       <c r="J54" t="n">
         <v>23.3</v>
@@ -2839,16 +2839,16 @@
         <v>94.90000000000001</v>
       </c>
       <c r="H55" t="n">
-        <v>60.6</v>
+        <v>61.1</v>
       </c>
       <c r="I55" t="n">
-        <v>31.3</v>
+        <v>31.5</v>
       </c>
       <c r="J55" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="K55" t="n">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="L55" t="n">
         <v>3.4</v>
@@ -2968,16 +2968,16 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>70.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="H58" t="n">
-        <v>30.1</v>
+        <v>29.6</v>
       </c>
       <c r="I58" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="J58" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="K58" t="n">
         <v>1.6</v>
@@ -3185,22 +3185,22 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>51</v>
+        <v>45.9</v>
       </c>
       <c r="G63" t="n">
-        <v>13.9</v>
+        <v>12.5</v>
       </c>
       <c r="H63" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="I63" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="J63" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K63" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
@@ -3229,19 +3229,19 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>49</v>
+        <v>54.1</v>
       </c>
       <c r="G64" t="n">
-        <v>15.7</v>
+        <v>18.3</v>
       </c>
       <c r="H64" t="n">
-        <v>4.5</v>
+        <v>5.2</v>
       </c>
       <c r="I64" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="J64" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K64" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-19)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -1865,13 +1865,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>46.6</v>
+        <v>48.8</v>
       </c>
       <c r="G33" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -1909,7 +1909,7 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>53.4</v>
+        <v>51.2</v>
       </c>
       <c r="G34" t="n">
         <v>1.5</v>
@@ -2006,7 +2006,7 @@
         <v>73</v>
       </c>
       <c r="I36" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="J36" t="n">
         <v>28.2</v>
@@ -2047,13 +2047,13 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>46</v>
+        <v>45.7</v>
       </c>
       <c r="I37" t="n">
-        <v>18.8</v>
+        <v>18.7</v>
       </c>
       <c r="J37" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
       <c r="K37" t="n">
         <v>2.8</v>
@@ -2176,19 +2176,19 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>74.3</v>
+        <v>75.5</v>
       </c>
       <c r="H40" t="n">
-        <v>44.4</v>
+        <v>45.2</v>
       </c>
       <c r="I40" t="n">
-        <v>18.6</v>
+        <v>18.9</v>
       </c>
       <c r="J40" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
       <c r="K40" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="L40" t="n">
         <v>1.2</v>
@@ -2226,13 +2226,13 @@
         <v>14</v>
       </c>
       <c r="I41" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
       <c r="J41" t="n">
         <v>2</v>
       </c>
       <c r="K41" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L41" t="n">
         <v>0.2</v>
@@ -2405,7 +2405,7 @@
         <v>0.3</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2440,13 +2440,13 @@
         <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>18.1</v>
+        <v>16.9</v>
       </c>
       <c r="H46" t="n">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="I46" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="J46" t="n">
         <v>0.4</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-20)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -507,19 +507,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>77.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>60</v>
+        <v>56.9</v>
       </c>
       <c r="J2" t="n">
-        <v>44.6</v>
+        <v>40.7</v>
       </c>
       <c r="K2" t="n">
-        <v>28.2</v>
+        <v>25.1</v>
       </c>
       <c r="L2" t="n">
-        <v>16.3</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="3">
@@ -554,13 +554,13 @@
         <v>57</v>
       </c>
       <c r="I3" t="n">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
       <c r="J3" t="n">
-        <v>11.7</v>
+        <v>12.2</v>
       </c>
       <c r="K3" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="L3" t="n">
         <v>1.9</v>
@@ -595,19 +595,19 @@
         <v>82.40000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>51.7</v>
+        <v>51.4</v>
       </c>
       <c r="I4" t="n">
-        <v>32.7</v>
+        <v>32.3</v>
       </c>
       <c r="J4" t="n">
-        <v>13.5</v>
+        <v>15</v>
       </c>
       <c r="K4" t="n">
-        <v>6.6</v>
+        <v>7.3</v>
       </c>
       <c r="L4" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5">
@@ -642,16 +642,16 @@
         <v>35.2</v>
       </c>
       <c r="I5" t="n">
-        <v>9.800000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="J5" t="n">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="K5" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">
@@ -686,16 +686,16 @@
         <v>53.3</v>
       </c>
       <c r="I6" t="n">
-        <v>18.8</v>
+        <v>19.9</v>
       </c>
       <c r="J6" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="K6" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="7">
@@ -727,19 +727,19 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>36.3</v>
       </c>
       <c r="I7" t="n">
-        <v>18.4</v>
+        <v>18.7</v>
       </c>
       <c r="J7" t="n">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8">
@@ -777,10 +777,10 @@
         <v>13.2</v>
       </c>
       <c r="J8" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="K8" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="L8" t="n">
         <v>0.4</v>
@@ -818,13 +818,13 @@
         <v>14.4</v>
       </c>
       <c r="I9" t="n">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="J9" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L9" t="n">
         <v>0.2</v>
@@ -859,13 +859,13 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7.8</v>
+        <v>9.4</v>
       </c>
       <c r="I10" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="J10" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="K10" t="n">
         <v>0.3</v>
@@ -950,7 +950,7 @@
         <v>8.9</v>
       </c>
       <c r="I12" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="J12" t="n">
         <v>0.7</v>
@@ -994,13 +994,13 @@
         <v>6</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1214,16 +1214,16 @@
         <v>73.3</v>
       </c>
       <c r="I18" t="n">
-        <v>51.3</v>
+        <v>48.2</v>
       </c>
       <c r="J18" t="n">
-        <v>28.9</v>
+        <v>25.8</v>
       </c>
       <c r="K18" t="n">
-        <v>15.9</v>
+        <v>14.7</v>
       </c>
       <c r="L18" t="n">
-        <v>7.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>94.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>71.40000000000001</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>46.5</v>
+        <v>46.8</v>
       </c>
       <c r="J19" t="n">
-        <v>29</v>
+        <v>30.1</v>
       </c>
       <c r="K19" t="n">
-        <v>17.1</v>
+        <v>18</v>
       </c>
       <c r="L19" t="n">
-        <v>9.1</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>88.3</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="H20" t="n">
-        <v>62.4</v>
+        <v>68</v>
       </c>
       <c r="I20" t="n">
-        <v>31.2</v>
+        <v>34.9</v>
       </c>
       <c r="J20" t="n">
-        <v>16.1</v>
+        <v>18.7</v>
       </c>
       <c r="K20" t="n">
-        <v>7.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L20" t="n">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>82.59999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="H21" t="n">
-        <v>37.2</v>
+        <v>40</v>
       </c>
       <c r="I21" t="n">
-        <v>12.9</v>
+        <v>14.3</v>
       </c>
       <c r="J21" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="K21" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="22">
@@ -1387,19 +1387,19 @@
         <v>75.7</v>
       </c>
       <c r="H22" t="n">
-        <v>52.2</v>
+        <v>51</v>
       </c>
       <c r="I22" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J22" t="n">
-        <v>9.9</v>
+        <v>11</v>
       </c>
       <c r="K22" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="L22" t="n">
-        <v>1.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="23">
@@ -1428,22 +1428,22 @@
         <v>100</v>
       </c>
       <c r="G23" t="n">
-        <v>57.7</v>
+        <v>55.5</v>
       </c>
       <c r="H23" t="n">
-        <v>21.9</v>
+        <v>16.9</v>
       </c>
       <c r="I23" t="n">
-        <v>7</v>
+        <v>5.1</v>
       </c>
       <c r="J23" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="K23" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="L23" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="24">
@@ -1472,22 +1472,22 @@
         <v>100</v>
       </c>
       <c r="G24" t="n">
-        <v>66</v>
+        <v>55.7</v>
       </c>
       <c r="H24" t="n">
-        <v>20.8</v>
+        <v>16.2</v>
       </c>
       <c r="I24" t="n">
-        <v>9.199999999999999</v>
+        <v>6.7</v>
       </c>
       <c r="J24" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="K24" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="25">
@@ -1522,13 +1522,13 @@
         <v>10.2</v>
       </c>
       <c r="I25" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
       <c r="J25" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L25" t="n">
         <v>0.1</v>
@@ -1566,13 +1566,13 @@
         <v>16.3</v>
       </c>
       <c r="I26" t="n">
-        <v>7.7</v>
+        <v>7</v>
       </c>
       <c r="J26" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L26" t="n">
         <v>0.2</v>
@@ -1604,22 +1604,22 @@
         <v>100</v>
       </c>
       <c r="G27" t="n">
-        <v>34</v>
+        <v>44.3</v>
       </c>
       <c r="H27" t="n">
-        <v>7.4</v>
+        <v>9.4</v>
       </c>
       <c r="I27" t="n">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
       <c r="J27" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="K27" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="28">
@@ -1648,19 +1648,19 @@
         <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>42.3</v>
+        <v>44.5</v>
       </c>
       <c r="H28" t="n">
-        <v>13.7</v>
+        <v>13.9</v>
       </c>
       <c r="I28" t="n">
         <v>3.3</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L28" t="n">
         <v>0.1</v>
@@ -1695,13 +1695,13 @@
         <v>24.3</v>
       </c>
       <c r="H29" t="n">
-        <v>8.4</v>
+        <v>7.6</v>
       </c>
       <c r="I29" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="J29" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K29" t="n">
         <v>0.1</v>
@@ -1736,13 +1736,13 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>17.4</v>
+        <v>11.7</v>
       </c>
       <c r="H30" t="n">
-        <v>2.2</v>
+        <v>1.5</v>
       </c>
       <c r="I30" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1780,10 +1780,10 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>11.7</v>
+        <v>8.6</v>
       </c>
       <c r="H31" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="I31" t="n">
         <v>0.1</v>
@@ -1824,7 +1824,7 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>5.9</v>
+        <v>5.1</v>
       </c>
       <c r="H32" t="n">
         <v>0.4</v>
@@ -1956,22 +1956,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>90.8</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>73.8</v>
+        <v>72.3</v>
       </c>
       <c r="I35" t="n">
-        <v>51.9</v>
+        <v>51</v>
       </c>
       <c r="J35" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K35" t="n">
-        <v>18.2</v>
+        <v>17.5</v>
       </c>
       <c r="L35" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="36">
@@ -2009,13 +2009,13 @@
         <v>50.1</v>
       </c>
       <c r="J36" t="n">
-        <v>28.2</v>
+        <v>28.3</v>
       </c>
       <c r="K36" t="n">
         <v>13.6</v>
       </c>
       <c r="L36" t="n">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="37">
@@ -2053,13 +2053,13 @@
         <v>18.7</v>
       </c>
       <c r="J37" t="n">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K37" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="38">
@@ -2094,13 +2094,13 @@
         <v>45.5</v>
       </c>
       <c r="I38" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="J38" t="n">
-        <v>10</v>
+        <v>10.1</v>
       </c>
       <c r="K38" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="L38" t="n">
         <v>1.7</v>
@@ -2138,7 +2138,7 @@
         <v>38.1</v>
       </c>
       <c r="I39" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="J39" t="n">
         <v>5.9</v>
@@ -2185,7 +2185,7 @@
         <v>18.9</v>
       </c>
       <c r="J40" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="K40" t="n">
         <v>3.1</v>
@@ -2229,7 +2229,7 @@
         <v>6.2</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="K41" t="n">
         <v>0.6</v>
@@ -2264,19 +2264,19 @@
         <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>55.2</v>
+        <v>53</v>
       </c>
       <c r="H42" t="n">
-        <v>13.5</v>
+        <v>12.8</v>
       </c>
       <c r="I42" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="J42" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="K42" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L42" t="n">
         <v>0.1</v>
@@ -2308,19 +2308,19 @@
         <v>100</v>
       </c>
       <c r="G43" t="n">
-        <v>44.8</v>
+        <v>47</v>
       </c>
       <c r="H43" t="n">
-        <v>11.4</v>
+        <v>13.6</v>
       </c>
       <c r="I43" t="n">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="J43" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="K43" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2405,7 +2405,7 @@
         <v>0.3</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -2490,7 +2490,7 @@
         <v>11</v>
       </c>
       <c r="I47" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="J47" t="n">
         <v>0.6</v>
@@ -2657,10 +2657,10 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>63.9</v>
+        <v>59.4</v>
       </c>
       <c r="G51" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="H51" t="n">
         <v>1.1</v>
@@ -2701,10 +2701,10 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>36.1</v>
+        <v>40.6</v>
       </c>
       <c r="G52" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="H52" t="n">
         <v>0.2</v>
@@ -2754,16 +2754,16 @@
         <v>75</v>
       </c>
       <c r="I53" t="n">
-        <v>56</v>
+        <v>56.8</v>
       </c>
       <c r="J53" t="n">
-        <v>38.6</v>
+        <v>39</v>
       </c>
       <c r="K53" t="n">
-        <v>25.7</v>
+        <v>26.1</v>
       </c>
       <c r="L53" t="n">
-        <v>16.4</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="54">
@@ -2798,16 +2798,16 @@
         <v>74.7</v>
       </c>
       <c r="I54" t="n">
-        <v>47.1</v>
+        <v>47.3</v>
       </c>
       <c r="J54" t="n">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="K54" t="n">
-        <v>13.1</v>
+        <v>13.3</v>
       </c>
       <c r="L54" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="55">
@@ -2839,16 +2839,16 @@
         <v>94.90000000000001</v>
       </c>
       <c r="H55" t="n">
-        <v>61.1</v>
+        <v>64.2</v>
       </c>
       <c r="I55" t="n">
-        <v>31.5</v>
+        <v>33.2</v>
       </c>
       <c r="J55" t="n">
-        <v>14.8</v>
+        <v>15.4</v>
       </c>
       <c r="K55" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="L55" t="n">
         <v>3.4</v>
@@ -2883,19 +2883,19 @@
         <v>76.8</v>
       </c>
       <c r="H56" t="n">
-        <v>46.2</v>
+        <v>52.2</v>
       </c>
       <c r="I56" t="n">
-        <v>16.4</v>
+        <v>18.5</v>
       </c>
       <c r="J56" t="n">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K56" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="L56" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="57">
@@ -2924,22 +2924,22 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>72.8</v>
+        <v>69.2</v>
       </c>
       <c r="H57" t="n">
-        <v>39.9</v>
+        <v>31.5</v>
       </c>
       <c r="I57" t="n">
-        <v>13.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J57" t="n">
-        <v>4.8</v>
+        <v>3.4</v>
       </c>
       <c r="K57" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="L57" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="58">
@@ -2968,22 +2968,22 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>69.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="H58" t="n">
-        <v>29.6</v>
+        <v>26.5</v>
       </c>
       <c r="I58" t="n">
-        <v>11.7</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J58" t="n">
-        <v>4.2</v>
+        <v>3.4</v>
       </c>
       <c r="K58" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="L58" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="59">
@@ -3018,7 +3018,7 @@
         <v>15.6</v>
       </c>
       <c r="I59" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="J59" t="n">
         <v>1.3</v>
@@ -3065,7 +3065,7 @@
         <v>2.7</v>
       </c>
       <c r="J60" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="K60" t="n">
         <v>0.2</v>
@@ -3106,7 +3106,7 @@
         <v>17.5</v>
       </c>
       <c r="I61" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J61" t="n">
         <v>3.5</v>
@@ -3150,7 +3150,7 @@
         <v>8.9</v>
       </c>
       <c r="I62" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="J62" t="n">
         <v>0.6</v>
@@ -3232,13 +3232,13 @@
         <v>54.1</v>
       </c>
       <c r="G64" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="H64" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="I64" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="J64" t="n">
         <v>0.4</v>
@@ -3276,16 +3276,16 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>27.2</v>
+        <v>30.8</v>
       </c>
       <c r="H65" t="n">
-        <v>10.3</v>
+        <v>11.6</v>
       </c>
       <c r="I65" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="J65" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3323,13 +3323,13 @@
         <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
       <c r="I66" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-21)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -510,16 +510,16 @@
         <v>75.59999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="J2" t="n">
-        <v>40.7</v>
+        <v>40.8</v>
       </c>
       <c r="K2" t="n">
-        <v>25.1</v>
+        <v>25</v>
       </c>
       <c r="L2" t="n">
-        <v>14.1</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>91.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>57</v>
+        <v>58.3</v>
       </c>
       <c r="I3" t="n">
-        <v>29.7</v>
+        <v>30.4</v>
       </c>
       <c r="J3" t="n">
         <v>12.2</v>
       </c>
       <c r="K3" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="L3" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="4">
@@ -598,16 +598,16 @@
         <v>51.4</v>
       </c>
       <c r="I4" t="n">
-        <v>32.3</v>
+        <v>31.9</v>
       </c>
       <c r="J4" t="n">
-        <v>15</v>
+        <v>14.8</v>
       </c>
       <c r="K4" t="n">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="5">
@@ -636,10 +636,10 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>74.2</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="I5" t="n">
         <v>11.2</v>
@@ -651,7 +651,7 @@
         <v>1.6</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -683,16 +683,16 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>53.3</v>
+        <v>54.3</v>
       </c>
       <c r="I6" t="n">
-        <v>19.9</v>
+        <v>20.5</v>
       </c>
       <c r="J6" t="n">
-        <v>10.1</v>
+        <v>10.6</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>4.3</v>
       </c>
       <c r="L6" t="n">
         <v>1.5</v>
@@ -730,16 +730,16 @@
         <v>36.3</v>
       </c>
       <c r="I7" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="K7" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="L7" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8">
@@ -768,13 +768,13 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>69.5</v>
+        <v>67.2</v>
       </c>
       <c r="H8" t="n">
-        <v>32.3</v>
+        <v>31.5</v>
       </c>
       <c r="I8" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="J8" t="n">
         <v>4.5</v>
@@ -862,16 +862,16 @@
         <v>9.4</v>
       </c>
       <c r="I10" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="J10" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="K10" t="n">
         <v>0.3</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -900,16 +900,16 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>30.5</v>
+        <v>32.8</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="J11" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K11" t="n">
         <v>0.1</v>
@@ -953,7 +953,7 @@
         <v>2.6</v>
       </c>
       <c r="J12" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K12" t="n">
         <v>0.2</v>
@@ -991,16 +991,16 @@
         <v>16.2</v>
       </c>
       <c r="H13" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="I13" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="J13" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1032,13 +1032,13 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>25.8</v>
+        <v>23.1</v>
       </c>
       <c r="H14" t="n">
-        <v>5.6</v>
+        <v>4.6</v>
       </c>
       <c r="I14" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="J14" t="n">
         <v>0.2</v>
@@ -1120,13 +1120,13 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>8.699999999999999</v>
+        <v>5.9</v>
       </c>
       <c r="H16" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1208,22 +1208,22 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>97.2</v>
+        <v>97.8</v>
       </c>
       <c r="H18" t="n">
-        <v>73.3</v>
+        <v>74.5</v>
       </c>
       <c r="I18" t="n">
-        <v>48.2</v>
+        <v>52.8</v>
       </c>
       <c r="J18" t="n">
-        <v>25.8</v>
+        <v>29.2</v>
       </c>
       <c r="K18" t="n">
-        <v>14.7</v>
+        <v>16.8</v>
       </c>
       <c r="L18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1261,13 +1261,13 @@
         <v>46.8</v>
       </c>
       <c r="J19" t="n">
-        <v>30.1</v>
+        <v>29.2</v>
       </c>
       <c r="K19" t="n">
-        <v>18</v>
+        <v>17.3</v>
       </c>
       <c r="L19" t="n">
-        <v>9.6</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="20">
@@ -1305,13 +1305,13 @@
         <v>34.9</v>
       </c>
       <c r="J20" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="K20" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L20" t="n">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="21">
@@ -1346,16 +1346,16 @@
         <v>40</v>
       </c>
       <c r="I21" t="n">
-        <v>14.3</v>
+        <v>13.2</v>
       </c>
       <c r="J21" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="K21" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="L21" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22">
@@ -1390,16 +1390,16 @@
         <v>51</v>
       </c>
       <c r="I22" t="n">
-        <v>25</v>
+        <v>21.2</v>
       </c>
       <c r="J22" t="n">
-        <v>11</v>
+        <v>9.4</v>
       </c>
       <c r="K22" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="L22" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="23">
@@ -1437,10 +1437,10 @@
         <v>5.1</v>
       </c>
       <c r="J23" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="K23" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L23" t="n">
         <v>0.1</v>
@@ -1481,13 +1481,13 @@
         <v>6.7</v>
       </c>
       <c r="J24" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="K24" t="n">
         <v>0.8</v>
       </c>
       <c r="L24" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="25">
@@ -1516,22 +1516,22 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>41</v>
+        <v>40.7</v>
       </c>
       <c r="H25" t="n">
-        <v>10.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="J25" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="K25" t="n">
         <v>0.2</v>
       </c>
       <c r="L25" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1560,22 +1560,22 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>59</v>
+        <v>59.3</v>
       </c>
       <c r="H26" t="n">
-        <v>16.3</v>
+        <v>17.2</v>
       </c>
       <c r="I26" t="n">
-        <v>7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
       <c r="K26" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
@@ -1613,10 +1613,10 @@
         <v>3.1</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K27" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L27" t="n">
         <v>0.1</v>
@@ -1657,13 +1657,13 @@
         <v>3.3</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K28" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L28" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1698,10 +1698,10 @@
         <v>7.6</v>
       </c>
       <c r="I29" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="J29" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K29" t="n">
         <v>0.1</v>
@@ -1742,7 +1742,7 @@
         <v>1.5</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1865,13 +1865,13 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>48.8</v>
+        <v>46.6</v>
       </c>
       <c r="G33" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -1909,10 +1909,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>51.2</v>
+        <v>53.4</v>
       </c>
       <c r="G34" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1962,16 +1962,16 @@
         <v>72.3</v>
       </c>
       <c r="I35" t="n">
-        <v>51</v>
+        <v>49.8</v>
       </c>
       <c r="J35" t="n">
-        <v>32</v>
+        <v>28.4</v>
       </c>
       <c r="K35" t="n">
-        <v>17.5</v>
+        <v>15.4</v>
       </c>
       <c r="L35" t="n">
-        <v>10.2</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="36">
@@ -2000,22 +2000,22 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>94.90000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>73</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="I36" t="n">
-        <v>50.1</v>
+        <v>58.5</v>
       </c>
       <c r="J36" t="n">
-        <v>28.3</v>
+        <v>35.8</v>
       </c>
       <c r="K36" t="n">
-        <v>13.6</v>
+        <v>17.8</v>
       </c>
       <c r="L36" t="n">
-        <v>7.3</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -2047,19 +2047,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>45.7</v>
+        <v>45.1</v>
       </c>
       <c r="I37" t="n">
-        <v>18.7</v>
+        <v>15.9</v>
       </c>
       <c r="J37" t="n">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="K37" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="L37" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="38">
@@ -2091,16 +2091,16 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>45.5</v>
+        <v>44.9</v>
       </c>
       <c r="I38" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="J38" t="n">
-        <v>10.1</v>
+        <v>9.6</v>
       </c>
       <c r="K38" t="n">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="L38" t="n">
         <v>1.7</v>
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>69.2</v>
+        <v>72.8</v>
       </c>
       <c r="H39" t="n">
-        <v>38.1</v>
+        <v>40.1</v>
       </c>
       <c r="I39" t="n">
-        <v>14.2</v>
+        <v>16.8</v>
       </c>
       <c r="J39" t="n">
-        <v>5.9</v>
+        <v>6.3</v>
       </c>
       <c r="K39" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="L39" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="40">
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>75.5</v>
+        <v>77.3</v>
       </c>
       <c r="H40" t="n">
-        <v>45.2</v>
+        <v>46.2</v>
       </c>
       <c r="I40" t="n">
-        <v>18.9</v>
+        <v>16.5</v>
       </c>
       <c r="J40" t="n">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="K40" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
       <c r="L40" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="41">
@@ -2220,22 +2220,22 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>53.6</v>
+        <v>55.9</v>
       </c>
       <c r="H41" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I41" t="n">
-        <v>6.2</v>
+        <v>5</v>
       </c>
       <c r="J41" t="n">
-        <v>2.1</v>
+        <v>1.7</v>
       </c>
       <c r="K41" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="L41" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="42">
@@ -2270,10 +2270,10 @@
         <v>12.8</v>
       </c>
       <c r="I42" t="n">
-        <v>5.4</v>
+        <v>5.2</v>
       </c>
       <c r="J42" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="K42" t="n">
         <v>0.4</v>
@@ -2314,13 +2314,13 @@
         <v>13.6</v>
       </c>
       <c r="I43" t="n">
-        <v>5.5</v>
+        <v>5.1</v>
       </c>
       <c r="J43" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="K43" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2352,19 +2352,19 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>46.4</v>
+        <v>44.1</v>
       </c>
       <c r="H44" t="n">
-        <v>12.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I44" t="n">
-        <v>4.2</v>
+        <v>2.9</v>
       </c>
       <c r="J44" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2396,13 +2396,13 @@
         <v>30.7</v>
       </c>
       <c r="G45" t="n">
-        <v>7.6</v>
+        <v>5.9</v>
       </c>
       <c r="H45" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="I45" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2440,16 +2440,16 @@
         <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="H46" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="I46" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="J46" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="K46" t="n">
         <v>0.1</v>
@@ -2484,16 +2484,16 @@
         <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>30.8</v>
+        <v>27.2</v>
       </c>
       <c r="H47" t="n">
-        <v>11</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>2.5</v>
+        <v>2.2</v>
       </c>
       <c r="J47" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2531,10 +2531,10 @@
         <v>23</v>
       </c>
       <c r="H48" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="I48" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="J48" t="n">
         <v>0.1</v>
@@ -2578,7 +2578,7 @@
         <v>1.7</v>
       </c>
       <c r="I49" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>5.1</v>
+        <v>2.9</v>
       </c>
       <c r="H50" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="I50" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2748,22 +2748,22 @@
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>95.2</v>
+        <v>97.2</v>
       </c>
       <c r="H53" t="n">
-        <v>75</v>
+        <v>77.3</v>
       </c>
       <c r="I53" t="n">
-        <v>56.8</v>
+        <v>58.6</v>
       </c>
       <c r="J53" t="n">
-        <v>39</v>
+        <v>40.2</v>
       </c>
       <c r="K53" t="n">
-        <v>26.1</v>
+        <v>26.9</v>
       </c>
       <c r="L53" t="n">
-        <v>16.7</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="54">
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>94.3</v>
+        <v>95.3</v>
       </c>
       <c r="H54" t="n">
-        <v>74.7</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="I54" t="n">
-        <v>47.3</v>
+        <v>50.8</v>
       </c>
       <c r="J54" t="n">
-        <v>23.2</v>
+        <v>24.8</v>
       </c>
       <c r="K54" t="n">
-        <v>13.3</v>
+        <v>13.6</v>
       </c>
       <c r="L54" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="55">
@@ -2842,16 +2842,16 @@
         <v>64.2</v>
       </c>
       <c r="I55" t="n">
-        <v>33.2</v>
+        <v>31.1</v>
       </c>
       <c r="J55" t="n">
-        <v>15.4</v>
+        <v>14.2</v>
       </c>
       <c r="K55" t="n">
-        <v>7.6</v>
+        <v>6.8</v>
       </c>
       <c r="L55" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56">
@@ -2886,16 +2886,16 @@
         <v>52.2</v>
       </c>
       <c r="I56" t="n">
-        <v>18.5</v>
+        <v>18.1</v>
       </c>
       <c r="J56" t="n">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="K56" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="L56" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="57">
@@ -2930,16 +2930,16 @@
         <v>31.5</v>
       </c>
       <c r="I57" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J57" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="K57" t="n">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
       <c r="L57" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="58">
@@ -2974,13 +2974,13 @@
         <v>26.5</v>
       </c>
       <c r="I58" t="n">
-        <v>9.699999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J58" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="K58" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="L58" t="n">
         <v>0.4</v>
@@ -3012,13 +3012,13 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>55.6</v>
+        <v>57.5</v>
       </c>
       <c r="H59" t="n">
-        <v>15.6</v>
+        <v>15.1</v>
       </c>
       <c r="I59" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="J59" t="n">
         <v>1.3</v>
@@ -3056,19 +3056,19 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>33.8</v>
+        <v>31.9</v>
       </c>
       <c r="H60" t="n">
-        <v>7.1</v>
+        <v>5.4</v>
       </c>
       <c r="I60" t="n">
-        <v>2.7</v>
+        <v>2</v>
       </c>
       <c r="J60" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="K60" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -3100,16 +3100,16 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>66.2</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H61" t="n">
-        <v>17.5</v>
+        <v>17.1</v>
       </c>
       <c r="I61" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="K61" t="n">
         <v>1.2</v>
@@ -3144,16 +3144,16 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>44.4</v>
+        <v>42.5</v>
       </c>
       <c r="H62" t="n">
-        <v>8.9</v>
+        <v>5.6</v>
       </c>
       <c r="I62" t="n">
-        <v>2.4</v>
+        <v>1.5</v>
       </c>
       <c r="J62" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="K62" t="n">
         <v>0.1</v>
@@ -3194,7 +3194,7 @@
         <v>3.2</v>
       </c>
       <c r="I63" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="J63" t="n">
         <v>0.2</v>
@@ -3238,7 +3238,7 @@
         <v>5.3</v>
       </c>
       <c r="I64" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="J64" t="n">
         <v>0.4</v>
@@ -3282,10 +3282,10 @@
         <v>11.6</v>
       </c>
       <c r="I65" t="n">
-        <v>2.6</v>
+        <v>2.3</v>
       </c>
       <c r="J65" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K65" t="n">
         <v>0.1</v>
@@ -3408,13 +3408,13 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="H68" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="I68" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>4.8</v>
+        <v>2.8</v>
       </c>
       <c r="H69" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-22)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -507,19 +507,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>75.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>57</v>
+        <v>59.6</v>
       </c>
       <c r="J2" t="n">
-        <v>40.8</v>
+        <v>43.1</v>
       </c>
       <c r="K2" t="n">
-        <v>25</v>
+        <v>26.4</v>
       </c>
       <c r="L2" t="n">
-        <v>13.8</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="3">
@@ -557,13 +557,13 @@
         <v>30.4</v>
       </c>
       <c r="J3" t="n">
-        <v>12.2</v>
+        <v>11.8</v>
       </c>
       <c r="K3" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="L3" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="4">
@@ -598,16 +598,16 @@
         <v>51.4</v>
       </c>
       <c r="I4" t="n">
-        <v>31.9</v>
+        <v>32.1</v>
       </c>
       <c r="J4" t="n">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="L4" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="5">
@@ -642,13 +642,13 @@
         <v>35.3</v>
       </c>
       <c r="I5" t="n">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="J5" t="n">
         <v>4.9</v>
       </c>
       <c r="K5" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="L5" t="n">
         <v>0.4</v>
@@ -686,16 +686,16 @@
         <v>54.3</v>
       </c>
       <c r="I6" t="n">
-        <v>20.5</v>
+        <v>19.2</v>
       </c>
       <c r="J6" t="n">
-        <v>10.6</v>
+        <v>10</v>
       </c>
       <c r="K6" t="n">
-        <v>4.3</v>
+        <v>3.6</v>
       </c>
       <c r="L6" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7">
@@ -727,19 +727,19 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36.3</v>
+        <v>36.1</v>
       </c>
       <c r="I7" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="J7" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="K7" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8">
@@ -774,16 +774,16 @@
         <v>31.5</v>
       </c>
       <c r="I8" t="n">
-        <v>13.3</v>
+        <v>13.1</v>
       </c>
       <c r="J8" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="K8" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="L8" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9">
@@ -821,10 +821,10 @@
         <v>6.1</v>
       </c>
       <c r="J9" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="K9" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="L9" t="n">
         <v>0.2</v>
@@ -859,16 +859,16 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>9.4</v>
+        <v>7</v>
       </c>
       <c r="I10" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="J10" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -956,7 +956,7 @@
         <v>0.6</v>
       </c>
       <c r="K12" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1079,10 +1079,10 @@
         <v>17.6</v>
       </c>
       <c r="H15" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="J15" t="n">
         <v>0.1</v>
@@ -1214,16 +1214,16 @@
         <v>74.5</v>
       </c>
       <c r="I18" t="n">
-        <v>52.8</v>
+        <v>52.4</v>
       </c>
       <c r="J18" t="n">
-        <v>29.2</v>
+        <v>27.5</v>
       </c>
       <c r="K18" t="n">
-        <v>16.8</v>
+        <v>15.6</v>
       </c>
       <c r="L18" t="n">
-        <v>8</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="19">
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>94.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H19" t="n">
-        <v>74.09999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>46.8</v>
+        <v>49</v>
       </c>
       <c r="J19" t="n">
-        <v>29.2</v>
+        <v>31.9</v>
       </c>
       <c r="K19" t="n">
-        <v>17.3</v>
+        <v>19.6</v>
       </c>
       <c r="L19" t="n">
-        <v>9.1</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="20">
@@ -1296,22 +1296,22 @@
         <v>100</v>
       </c>
       <c r="G20" t="n">
-        <v>91.40000000000001</v>
+        <v>94.2</v>
       </c>
       <c r="H20" t="n">
-        <v>68</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>34.9</v>
+        <v>37.9</v>
       </c>
       <c r="J20" t="n">
-        <v>18.4</v>
+        <v>21.4</v>
       </c>
       <c r="K20" t="n">
-        <v>9.199999999999999</v>
+        <v>11.1</v>
       </c>
       <c r="L20" t="n">
-        <v>4.1</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="21">
@@ -1343,13 +1343,13 @@
         <v>88.3</v>
       </c>
       <c r="H21" t="n">
-        <v>40</v>
+        <v>42.6</v>
       </c>
       <c r="I21" t="n">
-        <v>13.2</v>
+        <v>15</v>
       </c>
       <c r="J21" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="K21" t="n">
         <v>1.7</v>
@@ -1384,22 +1384,22 @@
         <v>100</v>
       </c>
       <c r="G22" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>51</v>
+        <v>48.4</v>
       </c>
       <c r="I22" t="n">
-        <v>21.2</v>
+        <v>20.1</v>
       </c>
       <c r="J22" t="n">
-        <v>9.4</v>
+        <v>7.2</v>
       </c>
       <c r="K22" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="L22" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="23">
@@ -1431,16 +1431,16 @@
         <v>55.5</v>
       </c>
       <c r="H23" t="n">
-        <v>16.9</v>
+        <v>14.6</v>
       </c>
       <c r="I23" t="n">
-        <v>5.1</v>
+        <v>3.8</v>
       </c>
       <c r="J23" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="K23" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L23" t="n">
         <v>0.1</v>
@@ -1475,16 +1475,16 @@
         <v>55.7</v>
       </c>
       <c r="H24" t="n">
-        <v>16.2</v>
+        <v>14.7</v>
       </c>
       <c r="I24" t="n">
-        <v>6.7</v>
+        <v>5.4</v>
       </c>
       <c r="J24" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="K24" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L24" t="n">
         <v>0.2</v>
@@ -1522,13 +1522,13 @@
         <v>8.199999999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="J25" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -1566,16 +1566,16 @@
         <v>17.2</v>
       </c>
       <c r="I26" t="n">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
       <c r="J26" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27">
@@ -1607,19 +1607,19 @@
         <v>44.3</v>
       </c>
       <c r="H27" t="n">
-        <v>9.4</v>
+        <v>6.9</v>
       </c>
       <c r="I27" t="n">
-        <v>3.1</v>
+        <v>1.9</v>
       </c>
       <c r="J27" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="K27" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L27" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1651,16 +1651,16 @@
         <v>44.5</v>
       </c>
       <c r="H28" t="n">
-        <v>13.9</v>
+        <v>10.2</v>
       </c>
       <c r="I28" t="n">
-        <v>3.3</v>
+        <v>2.1</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1692,7 +1692,7 @@
         <v>100</v>
       </c>
       <c r="G29" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="H29" t="n">
         <v>7.6</v>
@@ -1780,10 +1780,10 @@
         <v>100</v>
       </c>
       <c r="G31" t="n">
-        <v>8.6</v>
+        <v>5.8</v>
       </c>
       <c r="H31" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
         <v>0.1</v>
@@ -1824,10 +1824,10 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="H32" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -1959,19 +1959,19 @@
         <v>91.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>72.3</v>
+        <v>74</v>
       </c>
       <c r="I35" t="n">
-        <v>49.8</v>
+        <v>53.4</v>
       </c>
       <c r="J35" t="n">
-        <v>28.4</v>
+        <v>31.6</v>
       </c>
       <c r="K35" t="n">
-        <v>15.4</v>
+        <v>17.9</v>
       </c>
       <c r="L35" t="n">
-        <v>8.9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="36">
@@ -2009,13 +2009,13 @@
         <v>58.5</v>
       </c>
       <c r="J36" t="n">
-        <v>35.8</v>
+        <v>34.9</v>
       </c>
       <c r="K36" t="n">
-        <v>17.8</v>
+        <v>17.5</v>
       </c>
       <c r="L36" t="n">
-        <v>9.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="37">
@@ -2053,13 +2053,13 @@
         <v>15.9</v>
       </c>
       <c r="J37" t="n">
-        <v>6.8</v>
+        <v>6.3</v>
       </c>
       <c r="K37" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="L37" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="38">
@@ -2094,16 +2094,16 @@
         <v>44.9</v>
       </c>
       <c r="I38" t="n">
-        <v>20.1</v>
+        <v>19</v>
       </c>
       <c r="J38" t="n">
-        <v>9.6</v>
+        <v>9.1</v>
       </c>
       <c r="K38" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="L38" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="39">
@@ -2138,16 +2138,16 @@
         <v>40.1</v>
       </c>
       <c r="I39" t="n">
-        <v>16.8</v>
+        <v>14.9</v>
       </c>
       <c r="J39" t="n">
-        <v>6.3</v>
+        <v>5.6</v>
       </c>
       <c r="K39" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L39" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="40">
@@ -2185,13 +2185,13 @@
         <v>16.5</v>
       </c>
       <c r="J40" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="K40" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L40" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2311,16 +2311,16 @@
         <v>47</v>
       </c>
       <c r="H43" t="n">
-        <v>13.6</v>
+        <v>11.9</v>
       </c>
       <c r="I43" t="n">
-        <v>5.1</v>
+        <v>4.5</v>
       </c>
       <c r="J43" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L43" t="n">
         <v>0.1</v>
@@ -2361,7 +2361,7 @@
         <v>2.9</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K44" t="n">
         <v>0.2</v>
@@ -2490,7 +2490,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="I47" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="J47" t="n">
         <v>0.4</v>
@@ -2757,13 +2757,13 @@
         <v>58.6</v>
       </c>
       <c r="J53" t="n">
-        <v>40.2</v>
+        <v>41.3</v>
       </c>
       <c r="K53" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="L53" t="n">
-        <v>17.5</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="54">
@@ -2798,13 +2798,13 @@
         <v>78.59999999999999</v>
       </c>
       <c r="I54" t="n">
-        <v>50.8</v>
+        <v>54</v>
       </c>
       <c r="J54" t="n">
-        <v>24.8</v>
+        <v>26.4</v>
       </c>
       <c r="K54" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="L54" t="n">
         <v>7.6</v>
@@ -2836,22 +2836,22 @@
         <v>100</v>
       </c>
       <c r="G55" t="n">
-        <v>94.90000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="H55" t="n">
-        <v>64.2</v>
+        <v>56.8</v>
       </c>
       <c r="I55" t="n">
-        <v>31.1</v>
+        <v>25.1</v>
       </c>
       <c r="J55" t="n">
-        <v>14.2</v>
+        <v>10.2</v>
       </c>
       <c r="K55" t="n">
-        <v>6.8</v>
+        <v>4.3</v>
       </c>
       <c r="L55" t="n">
-        <v>3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="56">
@@ -2883,13 +2883,13 @@
         <v>76.8</v>
       </c>
       <c r="H56" t="n">
-        <v>52.2</v>
+        <v>52</v>
       </c>
       <c r="I56" t="n">
         <v>18.1</v>
       </c>
       <c r="J56" t="n">
-        <v>7.9</v>
+        <v>8.1</v>
       </c>
       <c r="K56" t="n">
         <v>3.2</v>
@@ -2924,19 +2924,19 @@
         <v>100</v>
       </c>
       <c r="G57" t="n">
-        <v>69.2</v>
+        <v>71.7</v>
       </c>
       <c r="H57" t="n">
-        <v>31.5</v>
+        <v>32.6</v>
       </c>
       <c r="I57" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="J57" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="K57" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
         <v>0.3</v>
@@ -2968,19 +2968,19 @@
         <v>100</v>
       </c>
       <c r="G58" t="n">
-        <v>69.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>26.5</v>
+        <v>30.6</v>
       </c>
       <c r="I58" t="n">
-        <v>9.300000000000001</v>
+        <v>10.7</v>
       </c>
       <c r="J58" t="n">
-        <v>3.2</v>
+        <v>3.7</v>
       </c>
       <c r="K58" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="L58" t="n">
         <v>0.4</v>
@@ -3018,10 +3018,10 @@
         <v>15.1</v>
       </c>
       <c r="I59" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="J59" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="K59" t="n">
         <v>0.3</v>
@@ -3109,7 +3109,7 @@
         <v>9.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="K61" t="n">
         <v>1.2</v>
@@ -3150,7 +3150,7 @@
         <v>5.6</v>
       </c>
       <c r="I62" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="J62" t="n">
         <v>0.3</v>
@@ -3185,16 +3185,16 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>45.9</v>
+        <v>43.2</v>
       </c>
       <c r="G63" t="n">
-        <v>12.5</v>
+        <v>11.8</v>
       </c>
       <c r="H63" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="I63" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J63" t="n">
         <v>0.2</v>
@@ -3229,19 +3229,19 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>54.1</v>
+        <v>56.8</v>
       </c>
       <c r="G64" t="n">
-        <v>18.4</v>
+        <v>19.3</v>
       </c>
       <c r="H64" t="n">
-        <v>5.3</v>
+        <v>7.4</v>
       </c>
       <c r="I64" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K64" t="n">
         <v>0.1</v>
@@ -3276,13 +3276,13 @@
         <v>100</v>
       </c>
       <c r="G65" t="n">
-        <v>30.8</v>
+        <v>28.3</v>
       </c>
       <c r="H65" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="I65" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="J65" t="n">
         <v>0.4</v>
@@ -3323,7 +3323,7 @@
         <v>23.2</v>
       </c>
       <c r="H66" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="I66" t="n">
         <v>0.5</v>
@@ -3364,10 +3364,10 @@
         <v>100</v>
       </c>
       <c r="G67" t="n">
-        <v>5.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H67" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="I67" t="n">
         <v>0.1</v>
@@ -3414,7 +3414,7 @@
         <v>0.7</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-23)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -510,16 +510,16 @@
         <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>59.6</v>
+        <v>58.9</v>
       </c>
       <c r="J2" t="n">
-        <v>43.1</v>
+        <v>42.2</v>
       </c>
       <c r="K2" t="n">
-        <v>26.4</v>
+        <v>27.1</v>
       </c>
       <c r="L2" t="n">
-        <v>14.7</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>94.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>58.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>30.4</v>
+        <v>37.2</v>
       </c>
       <c r="J3" t="n">
-        <v>11.8</v>
+        <v>15.6</v>
       </c>
       <c r="K3" t="n">
-        <v>4.4</v>
+        <v>6.2</v>
       </c>
       <c r="L3" t="n">
-        <v>1.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="4">
@@ -598,13 +598,13 @@
         <v>51.4</v>
       </c>
       <c r="I4" t="n">
-        <v>32.1</v>
+        <v>31.6</v>
       </c>
       <c r="J4" t="n">
-        <v>14.7</v>
+        <v>14.5</v>
       </c>
       <c r="K4" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="L4" t="n">
         <v>2.6</v>
@@ -636,22 +636,22 @@
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>76.90000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="H5" t="n">
-        <v>35.3</v>
+        <v>34</v>
       </c>
       <c r="I5" t="n">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="J5" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
       <c r="K5" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -683,19 +683,19 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>54.3</v>
+        <v>54.4</v>
       </c>
       <c r="I6" t="n">
-        <v>19.2</v>
+        <v>20</v>
       </c>
       <c r="J6" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="K6" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -730,13 +730,13 @@
         <v>36.1</v>
       </c>
       <c r="I7" t="n">
-        <v>18.3</v>
+        <v>15.6</v>
       </c>
       <c r="J7" t="n">
-        <v>6.3</v>
+        <v>5.5</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="L7" t="n">
         <v>0.6</v>
@@ -768,22 +768,22 @@
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>67.2</v>
+        <v>64.3</v>
       </c>
       <c r="H8" t="n">
-        <v>31.5</v>
+        <v>23.7</v>
       </c>
       <c r="I8" t="n">
-        <v>13.1</v>
+        <v>9.5</v>
       </c>
       <c r="J8" t="n">
-        <v>4.3</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>1.3</v>
+        <v>0.8</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
@@ -821,7 +821,7 @@
         <v>6.1</v>
       </c>
       <c r="J9" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="K9" t="n">
         <v>0.7</v>
@@ -900,13 +900,13 @@
         <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>32.8</v>
+        <v>35.7</v>
       </c>
       <c r="H11" t="n">
-        <v>9.699999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="I11" t="n">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
@@ -991,7 +991,7 @@
         <v>16.2</v>
       </c>
       <c r="H13" t="n">
-        <v>5.8</v>
+        <v>6</v>
       </c>
       <c r="I13" t="n">
         <v>0.8</v>
@@ -1032,13 +1032,13 @@
         <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>23.1</v>
+        <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>4.6</v>
+        <v>5.6</v>
       </c>
       <c r="I14" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J14" t="n">
         <v>0.2</v>
@@ -1120,7 +1120,7 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>5.9</v>
+        <v>5.1</v>
       </c>
       <c r="H16" t="n">
         <v>0.5</v>
@@ -1208,22 +1208,22 @@
         <v>100</v>
       </c>
       <c r="G18" t="n">
-        <v>97.8</v>
+        <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>74.5</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>52.4</v>
+        <v>46.7</v>
       </c>
       <c r="J18" t="n">
-        <v>27.5</v>
+        <v>23.9</v>
       </c>
       <c r="K18" t="n">
-        <v>15.6</v>
+        <v>12.2</v>
       </c>
       <c r="L18" t="n">
-        <v>7.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="19">
@@ -1261,10 +1261,10 @@
         <v>49</v>
       </c>
       <c r="J19" t="n">
-        <v>31.9</v>
+        <v>32.4</v>
       </c>
       <c r="K19" t="n">
-        <v>19.6</v>
+        <v>20</v>
       </c>
       <c r="L19" t="n">
         <v>10.8</v>
@@ -1305,13 +1305,13 @@
         <v>37.9</v>
       </c>
       <c r="J20" t="n">
-        <v>21.4</v>
+        <v>22.3</v>
       </c>
       <c r="K20" t="n">
-        <v>11.1</v>
+        <v>11.3</v>
       </c>
       <c r="L20" t="n">
-        <v>5.2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="21">
@@ -1349,10 +1349,10 @@
         <v>15</v>
       </c>
       <c r="J21" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="K21" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L21" t="n">
         <v>0.5</v>
@@ -1390,16 +1390,16 @@
         <v>48.4</v>
       </c>
       <c r="I22" t="n">
-        <v>20.1</v>
+        <v>23.3</v>
       </c>
       <c r="J22" t="n">
-        <v>7.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="L22" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="23">
@@ -1437,10 +1437,10 @@
         <v>3.8</v>
       </c>
       <c r="J23" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="K23" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L23" t="n">
         <v>0.1</v>
@@ -1481,10 +1481,10 @@
         <v>5.4</v>
       </c>
       <c r="J24" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="L24" t="n">
         <v>0.2</v>
@@ -1516,16 +1516,16 @@
         <v>100</v>
       </c>
       <c r="G25" t="n">
-        <v>40.7</v>
+        <v>36.1</v>
       </c>
       <c r="H25" t="n">
-        <v>8.199999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="I25" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="J25" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="K25" t="n">
         <v>0.1</v>
@@ -1560,22 +1560,22 @@
         <v>100</v>
       </c>
       <c r="G26" t="n">
-        <v>59.3</v>
+        <v>63.9</v>
       </c>
       <c r="H26" t="n">
-        <v>17.2</v>
+        <v>21.7</v>
       </c>
       <c r="I26" t="n">
-        <v>7.9</v>
+        <v>10.4</v>
       </c>
       <c r="J26" t="n">
-        <v>2.3</v>
+        <v>3.1</v>
       </c>
       <c r="K26" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
@@ -1698,10 +1698,10 @@
         <v>7.6</v>
       </c>
       <c r="I29" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="J29" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K29" t="n">
         <v>0.1</v>
@@ -1742,7 +1742,7 @@
         <v>1.5</v>
       </c>
       <c r="I30" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1868,7 +1868,7 @@
         <v>46.6</v>
       </c>
       <c r="G33" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="H33" t="n">
         <v>0.1</v>
@@ -1912,7 +1912,7 @@
         <v>53.4</v>
       </c>
       <c r="G34" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H34" t="n">
         <v>0.1</v>
@@ -1962,16 +1962,16 @@
         <v>74</v>
       </c>
       <c r="I35" t="n">
-        <v>53.4</v>
+        <v>52.3</v>
       </c>
       <c r="J35" t="n">
-        <v>31.6</v>
+        <v>31.1</v>
       </c>
       <c r="K35" t="n">
-        <v>17.9</v>
+        <v>17</v>
       </c>
       <c r="L35" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="36">
@@ -2003,16 +2003,16 @@
         <v>97.09999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>78.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="I36" t="n">
-        <v>58.5</v>
+        <v>57.4</v>
       </c>
       <c r="J36" t="n">
-        <v>34.9</v>
+        <v>33.9</v>
       </c>
       <c r="K36" t="n">
-        <v>17.5</v>
+        <v>16.9</v>
       </c>
       <c r="L36" t="n">
         <v>9.300000000000001</v>
@@ -2047,19 +2047,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>45.1</v>
+        <v>43.8</v>
       </c>
       <c r="I37" t="n">
-        <v>15.9</v>
+        <v>14.8</v>
       </c>
       <c r="J37" t="n">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="K37" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="38">
@@ -2091,19 +2091,19 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>44.9</v>
+        <v>52.3</v>
       </c>
       <c r="I38" t="n">
-        <v>19</v>
+        <v>23.6</v>
       </c>
       <c r="J38" t="n">
-        <v>9.1</v>
+        <v>11.6</v>
       </c>
       <c r="K38" t="n">
-        <v>3.5</v>
+        <v>4.9</v>
       </c>
       <c r="L38" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="39">
@@ -2132,22 +2132,22 @@
         <v>100</v>
       </c>
       <c r="G39" t="n">
-        <v>72.8</v>
+        <v>71.7</v>
       </c>
       <c r="H39" t="n">
-        <v>40.1</v>
+        <v>32.9</v>
       </c>
       <c r="I39" t="n">
-        <v>14.9</v>
+        <v>11.6</v>
       </c>
       <c r="J39" t="n">
-        <v>5.6</v>
+        <v>4.2</v>
       </c>
       <c r="K39" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="L39" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="40">
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>77.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>46.2</v>
+        <v>47.6</v>
       </c>
       <c r="I40" t="n">
-        <v>16.5</v>
+        <v>18.8</v>
       </c>
       <c r="J40" t="n">
-        <v>6.9</v>
+        <v>7.9</v>
       </c>
       <c r="K40" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="L40" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="41">
@@ -2220,19 +2220,19 @@
         <v>100</v>
       </c>
       <c r="G41" t="n">
-        <v>55.9</v>
+        <v>53.6</v>
       </c>
       <c r="H41" t="n">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="J41" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="K41" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L41" t="n">
         <v>0.1</v>
@@ -2270,7 +2270,7 @@
         <v>12.8</v>
       </c>
       <c r="I42" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="J42" t="n">
         <v>1.3</v>
@@ -2314,16 +2314,16 @@
         <v>11.9</v>
       </c>
       <c r="I43" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K43" t="n">
         <v>0.2</v>
       </c>
       <c r="L43" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2352,16 +2352,16 @@
         <v>100</v>
       </c>
       <c r="G44" t="n">
-        <v>44.1</v>
+        <v>46.4</v>
       </c>
       <c r="H44" t="n">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="I44" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K44" t="n">
         <v>0.2</v>
@@ -2396,7 +2396,7 @@
         <v>30.7</v>
       </c>
       <c r="G45" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="H45" t="n">
         <v>1.4</v>
@@ -2452,7 +2452,7 @@
         <v>0.3</v>
       </c>
       <c r="K46" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2484,10 +2484,10 @@
         <v>100</v>
       </c>
       <c r="G47" t="n">
-        <v>27.2</v>
+        <v>28.3</v>
       </c>
       <c r="H47" t="n">
-        <v>9.699999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="I47" t="n">
         <v>2.1</v>
@@ -2751,19 +2751,19 @@
         <v>97.2</v>
       </c>
       <c r="H53" t="n">
-        <v>77.3</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>58.6</v>
+        <v>59.9</v>
       </c>
       <c r="J53" t="n">
-        <v>41.3</v>
+        <v>42.3</v>
       </c>
       <c r="K53" t="n">
-        <v>27.1</v>
+        <v>28.3</v>
       </c>
       <c r="L53" t="n">
-        <v>17.2</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="54">
@@ -2795,16 +2795,16 @@
         <v>95.3</v>
       </c>
       <c r="H54" t="n">
-        <v>78.59999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>54</v>
+        <v>52.7</v>
       </c>
       <c r="J54" t="n">
-        <v>26.4</v>
+        <v>25.5</v>
       </c>
       <c r="K54" t="n">
-        <v>14.1</v>
+        <v>13.9</v>
       </c>
       <c r="L54" t="n">
         <v>7.6</v>
@@ -2842,16 +2842,16 @@
         <v>56.8</v>
       </c>
       <c r="I55" t="n">
-        <v>25.1</v>
+        <v>27.1</v>
       </c>
       <c r="J55" t="n">
-        <v>10.2</v>
+        <v>10.8</v>
       </c>
       <c r="K55" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="L55" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="56">
@@ -2886,16 +2886,16 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>18.1</v>
+        <v>17.8</v>
       </c>
       <c r="J56" t="n">
-        <v>8.1</v>
+        <v>8</v>
       </c>
       <c r="K56" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="L56" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="57">
@@ -2930,13 +2930,13 @@
         <v>32.6</v>
       </c>
       <c r="I57" t="n">
-        <v>9.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J57" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="K57" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L57" t="n">
         <v>0.3</v>
@@ -2974,7 +2974,7 @@
         <v>30.6</v>
       </c>
       <c r="I58" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="J58" t="n">
         <v>3.7</v>
@@ -3012,22 +3012,22 @@
         <v>100</v>
       </c>
       <c r="G59" t="n">
-        <v>57.5</v>
+        <v>57.7</v>
       </c>
       <c r="H59" t="n">
-        <v>15.1</v>
+        <v>12.7</v>
       </c>
       <c r="I59" t="n">
-        <v>5.4</v>
+        <v>4.2</v>
       </c>
       <c r="J59" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="K59" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="L59" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -3056,13 +3056,13 @@
         <v>100</v>
       </c>
       <c r="G60" t="n">
-        <v>31.9</v>
+        <v>33.6</v>
       </c>
       <c r="H60" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="J60" t="n">
         <v>0.5</v>
@@ -3100,19 +3100,19 @@
         <v>100</v>
       </c>
       <c r="G61" t="n">
-        <v>68.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="H61" t="n">
-        <v>17.1</v>
+        <v>16.7</v>
       </c>
       <c r="I61" t="n">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J61" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="K61" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L61" t="n">
         <v>0.4</v>
@@ -3144,16 +3144,16 @@
         <v>100</v>
       </c>
       <c r="G62" t="n">
-        <v>42.5</v>
+        <v>42.3</v>
       </c>
       <c r="H62" t="n">
-        <v>5.6</v>
+        <v>7.3</v>
       </c>
       <c r="I62" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="J62" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="K62" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-27)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -516,10 +516,10 @@
         <v>42.2</v>
       </c>
       <c r="K2" t="n">
-        <v>27.1</v>
+        <v>26.5</v>
       </c>
       <c r="L2" t="n">
-        <v>15.1</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="3">
@@ -560,10 +560,10 @@
         <v>15.6</v>
       </c>
       <c r="K3" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="L3" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="4">
@@ -604,10 +604,10 @@
         <v>14.5</v>
       </c>
       <c r="K4" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
       <c r="L4" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="5">
@@ -648,10 +648,10 @@
         <v>4.2</v>
       </c>
       <c r="K5" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="L5" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -692,7 +692,7 @@
         <v>10.3</v>
       </c>
       <c r="K6" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="L6" t="n">
         <v>1.4</v>
@@ -736,7 +736,7 @@
         <v>5.5</v>
       </c>
       <c r="K7" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="L7" t="n">
         <v>0.6</v>
@@ -780,7 +780,7 @@
         <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="L8" t="n">
         <v>0.2</v>
@@ -1211,19 +1211,19 @@
         <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>70.59999999999999</v>
+        <v>69.5</v>
       </c>
       <c r="I18" t="n">
-        <v>46.7</v>
+        <v>45.7</v>
       </c>
       <c r="J18" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="K18" t="n">
-        <v>12.2</v>
+        <v>12.1</v>
       </c>
       <c r="L18" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="19">
@@ -1252,22 +1252,22 @@
         <v>100</v>
       </c>
       <c r="G19" t="n">
-        <v>95.09999999999999</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>78.09999999999999</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>49</v>
+        <v>45.9</v>
       </c>
       <c r="J19" t="n">
-        <v>32.4</v>
+        <v>29.5</v>
       </c>
       <c r="K19" t="n">
-        <v>20</v>
+        <v>17.3</v>
       </c>
       <c r="L19" t="n">
-        <v>10.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
@@ -1302,16 +1302,16 @@
         <v>74.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>37.9</v>
+        <v>38.9</v>
       </c>
       <c r="J20" t="n">
-        <v>22.3</v>
+        <v>22.9</v>
       </c>
       <c r="K20" t="n">
-        <v>11.3</v>
+        <v>12.7</v>
       </c>
       <c r="L20" t="n">
-        <v>5.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -1340,22 +1340,22 @@
         <v>100</v>
       </c>
       <c r="G21" t="n">
-        <v>88.3</v>
+        <v>85.3</v>
       </c>
       <c r="H21" t="n">
-        <v>42.6</v>
+        <v>38.5</v>
       </c>
       <c r="I21" t="n">
-        <v>15</v>
+        <v>13.6</v>
       </c>
       <c r="J21" t="n">
-        <v>4.7</v>
+        <v>4.4</v>
       </c>
       <c r="K21" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22">
@@ -1387,19 +1387,19 @@
         <v>75.59999999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>48.4</v>
+        <v>51.5</v>
       </c>
       <c r="I22" t="n">
-        <v>23.3</v>
+        <v>24.8</v>
       </c>
       <c r="J22" t="n">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="L22" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="23">
@@ -1434,10 +1434,10 @@
         <v>14.6</v>
       </c>
       <c r="I23" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="J23" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="K23" t="n">
         <v>0.4</v>
@@ -1475,13 +1475,13 @@
         <v>55.7</v>
       </c>
       <c r="H24" t="n">
-        <v>14.7</v>
+        <v>16.2</v>
       </c>
       <c r="I24" t="n">
-        <v>5.4</v>
+        <v>5.9</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="K24" t="n">
         <v>0.7</v>
@@ -1525,7 +1525,7 @@
         <v>2.6</v>
       </c>
       <c r="J25" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K25" t="n">
         <v>0.1</v>
@@ -1563,19 +1563,19 @@
         <v>63.9</v>
       </c>
       <c r="H26" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="I26" t="n">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="J26" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="K26" t="n">
-        <v>1.1</v>
+        <v>1.4</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="27">
@@ -1607,16 +1607,16 @@
         <v>44.3</v>
       </c>
       <c r="H27" t="n">
-        <v>6.9</v>
+        <v>9.4</v>
       </c>
       <c r="I27" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="J27" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -1654,13 +1654,13 @@
         <v>10.2</v>
       </c>
       <c r="I28" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="J28" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K28" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -1695,10 +1695,10 @@
         <v>24.4</v>
       </c>
       <c r="H29" t="n">
-        <v>7.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I29" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="J29" t="n">
         <v>0.4</v>
@@ -1736,13 +1736,13 @@
         <v>100</v>
       </c>
       <c r="G30" t="n">
-        <v>11.7</v>
+        <v>14.7</v>
       </c>
       <c r="H30" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1824,10 +1824,10 @@
         <v>100</v>
       </c>
       <c r="G32" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="H32" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
@@ -1968,10 +1968,10 @@
         <v>31.1</v>
       </c>
       <c r="K35" t="n">
-        <v>17</v>
+        <v>16.9</v>
       </c>
       <c r="L35" t="n">
-        <v>9.699999999999999</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="36">
@@ -2012,10 +2012,10 @@
         <v>33.9</v>
       </c>
       <c r="K36" t="n">
-        <v>16.9</v>
+        <v>17.1</v>
       </c>
       <c r="L36" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="37">
@@ -2056,7 +2056,7 @@
         <v>5.9</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L37" t="n">
         <v>0.6</v>
@@ -2188,10 +2188,10 @@
         <v>7.9</v>
       </c>
       <c r="K40" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="L40" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
@@ -2323,7 +2323,7 @@
         <v>0.2</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
@@ -2452,7 +2452,7 @@
         <v>0.3</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
@@ -2754,16 +2754,16 @@
         <v>77.40000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>59.9</v>
+        <v>61.4</v>
       </c>
       <c r="J53" t="n">
-        <v>42.3</v>
+        <v>43.6</v>
       </c>
       <c r="K53" t="n">
-        <v>28.3</v>
+        <v>29.2</v>
       </c>
       <c r="L53" t="n">
-        <v>17.9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="54">
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>95.3</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>79.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="I54" t="n">
-        <v>52.7</v>
+        <v>51.9</v>
       </c>
       <c r="J54" t="n">
-        <v>25.5</v>
+        <v>24.9</v>
       </c>
       <c r="K54" t="n">
-        <v>13.9</v>
+        <v>13.1</v>
       </c>
       <c r="L54" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="55">
@@ -2842,16 +2842,16 @@
         <v>56.8</v>
       </c>
       <c r="I55" t="n">
-        <v>27.1</v>
+        <v>25.9</v>
       </c>
       <c r="J55" t="n">
-        <v>10.8</v>
+        <v>10.2</v>
       </c>
       <c r="K55" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="L55" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="56">
@@ -2886,13 +2886,13 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>17.8</v>
+        <v>16.1</v>
       </c>
       <c r="J56" t="n">
-        <v>8</v>
+        <v>7.2</v>
       </c>
       <c r="K56" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="L56" t="n">
         <v>1.2</v>
@@ -2933,7 +2933,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="J57" t="n">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="K57" t="n">
         <v>0.9</v>
@@ -2974,10 +2974,10 @@
         <v>30.6</v>
       </c>
       <c r="I58" t="n">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="J58" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="K58" t="n">
         <v>1.3</v>
@@ -3015,19 +3015,19 @@
         <v>57.7</v>
       </c>
       <c r="H59" t="n">
-        <v>12.7</v>
+        <v>15.9</v>
       </c>
       <c r="I59" t="n">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
       <c r="J59" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="K59" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L59" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="60">
@@ -3062,10 +3062,10 @@
         <v>5.7</v>
       </c>
       <c r="I60" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="J60" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K60" t="n">
         <v>0.1</v>
@@ -3112,7 +3112,7 @@
         <v>3.6</v>
       </c>
       <c r="K61" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="L61" t="n">
         <v>0.4</v>
@@ -3147,13 +3147,13 @@
         <v>42.3</v>
       </c>
       <c r="H62" t="n">
-        <v>7.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I62" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
       <c r="J62" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K62" t="n">
         <v>0.1</v>
@@ -3194,7 +3194,7 @@
         <v>3.8</v>
       </c>
       <c r="I63" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
         <v>0.2</v>
@@ -3238,13 +3238,13 @@
         <v>7.4</v>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="J64" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K64" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="H67" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="I67" t="n">
         <v>0.1</v>
@@ -3408,7 +3408,7 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>4.7</v>
+        <v>4.9</v>
       </c>
       <c r="H68" t="n">
         <v>0.7</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-28)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -510,16 +510,16 @@
         <v>78</v>
       </c>
       <c r="I2" t="n">
-        <v>58.9</v>
+        <v>59.7</v>
       </c>
       <c r="J2" t="n">
-        <v>42.2</v>
+        <v>43.4</v>
       </c>
       <c r="K2" t="n">
-        <v>26.5</v>
+        <v>27.6</v>
       </c>
       <c r="L2" t="n">
-        <v>14.4</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="3">
@@ -548,22 +548,22 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>94.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>66.40000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="I3" t="n">
-        <v>37.2</v>
+        <v>36.8</v>
       </c>
       <c r="J3" t="n">
-        <v>15.6</v>
+        <v>15</v>
       </c>
       <c r="K3" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="L3" t="n">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="4">
@@ -595,19 +595,19 @@
         <v>82.40000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>51.4</v>
+        <v>51.7</v>
       </c>
       <c r="I4" t="n">
-        <v>31.6</v>
+        <v>31.9</v>
       </c>
       <c r="J4" t="n">
-        <v>14.5</v>
+        <v>14.3</v>
       </c>
       <c r="K4" t="n">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="L4" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="5">
@@ -645,10 +645,10 @@
         <v>10.5</v>
       </c>
       <c r="J5" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="K5" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="L5" t="n">
         <v>0.4</v>
@@ -683,19 +683,19 @@
         <v>83.8</v>
       </c>
       <c r="H6" t="n">
-        <v>54.4</v>
+        <v>54.3</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>19.1</v>
       </c>
       <c r="J6" t="n">
-        <v>10.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="L6" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         <v>72.40000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36.1</v>
+        <v>35.7</v>
       </c>
       <c r="I7" t="n">
         <v>15.6</v>
@@ -771,16 +771,16 @@
         <v>64.3</v>
       </c>
       <c r="H8" t="n">
-        <v>23.7</v>
+        <v>24</v>
       </c>
       <c r="I8" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="K8" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L8" t="n">
         <v>0.2</v>
@@ -903,10 +903,10 @@
         <v>35.7</v>
       </c>
       <c r="H11" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="J11" t="n">
         <v>0.5</v>
@@ -953,7 +953,7 @@
         <v>2.6</v>
       </c>
       <c r="J12" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="K12" t="n">
         <v>0.1</v>
@@ -1035,7 +1035,7 @@
         <v>25.8</v>
       </c>
       <c r="H14" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="I14" t="n">
         <v>0.9</v>
@@ -1120,7 +1120,7 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>5.1</v>
+        <v>5.9</v>
       </c>
       <c r="H16" t="n">
         <v>0.5</v>
@@ -1223,7 +1223,7 @@
         <v>12.1</v>
       </c>
       <c r="L18" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="19">
@@ -1264,10 +1264,10 @@
         <v>29.5</v>
       </c>
       <c r="K19" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="L19" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1355,7 +1355,7 @@
         <v>1.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22">
@@ -1572,7 +1572,7 @@
         <v>3.5</v>
       </c>
       <c r="K26" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L26" t="n">
         <v>0.4</v>
@@ -1959,19 +1959,19 @@
         <v>91.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I35" t="n">
-        <v>52.3</v>
+        <v>54.8</v>
       </c>
       <c r="J35" t="n">
-        <v>31.1</v>
+        <v>35.9</v>
       </c>
       <c r="K35" t="n">
-        <v>16.9</v>
+        <v>20.3</v>
       </c>
       <c r="L35" t="n">
-        <v>9.9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="36">
@@ -2000,22 +2000,22 @@
         <v>100</v>
       </c>
       <c r="G36" t="n">
-        <v>97.09999999999999</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>79.2</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>57.4</v>
+        <v>46.1</v>
       </c>
       <c r="J36" t="n">
-        <v>33.9</v>
+        <v>24.7</v>
       </c>
       <c r="K36" t="n">
-        <v>17.1</v>
+        <v>11.4</v>
       </c>
       <c r="L36" t="n">
-        <v>9.4</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="37">
@@ -2047,19 +2047,19 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>43.8</v>
+        <v>43.5</v>
       </c>
       <c r="I37" t="n">
-        <v>14.8</v>
+        <v>18.2</v>
       </c>
       <c r="J37" t="n">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="K37" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="L37" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="38">
@@ -2091,19 +2091,19 @@
         <v>77</v>
       </c>
       <c r="H38" t="n">
-        <v>52.3</v>
+        <v>46.7</v>
       </c>
       <c r="I38" t="n">
-        <v>23.6</v>
+        <v>20.8</v>
       </c>
       <c r="J38" t="n">
-        <v>11.6</v>
+        <v>10.4</v>
       </c>
       <c r="K38" t="n">
-        <v>4.9</v>
+        <v>4.1</v>
       </c>
       <c r="L38" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="39">
@@ -2135,19 +2135,19 @@
         <v>71.7</v>
       </c>
       <c r="H39" t="n">
-        <v>32.9</v>
+        <v>38.2</v>
       </c>
       <c r="I39" t="n">
-        <v>11.6</v>
+        <v>12.4</v>
       </c>
       <c r="J39" t="n">
-        <v>4.2</v>
+        <v>5</v>
       </c>
       <c r="K39" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="L39" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="40">
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>77.40000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="H40" t="n">
-        <v>47.6</v>
+        <v>48.2</v>
       </c>
       <c r="I40" t="n">
-        <v>18.8</v>
+        <v>24.2</v>
       </c>
       <c r="J40" t="n">
-        <v>7.9</v>
+        <v>10.6</v>
       </c>
       <c r="K40" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="L40" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="41">
@@ -2223,13 +2223,13 @@
         <v>53.6</v>
       </c>
       <c r="H41" t="n">
-        <v>11.3</v>
+        <v>14</v>
       </c>
       <c r="I41" t="n">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
       <c r="J41" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="K41" t="n">
         <v>0.4</v>
@@ -2267,13 +2267,13 @@
         <v>53</v>
       </c>
       <c r="H42" t="n">
-        <v>12.8</v>
+        <v>11.7</v>
       </c>
       <c r="I42" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="J42" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="K42" t="n">
         <v>0.4</v>
@@ -2311,19 +2311,19 @@
         <v>47</v>
       </c>
       <c r="H43" t="n">
-        <v>11.9</v>
+        <v>11.1</v>
       </c>
       <c r="I43" t="n">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="J43" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
         <v>0.2</v>
       </c>
       <c r="L43" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2355,16 +2355,16 @@
         <v>46.4</v>
       </c>
       <c r="H44" t="n">
-        <v>9.1</v>
+        <v>12.2</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>3.9</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="K44" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L44" t="n">
         <v>0.1</v>
@@ -2440,13 +2440,13 @@
         <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>16.8</v>
+        <v>15.9</v>
       </c>
       <c r="H46" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="I46" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="J46" t="n">
         <v>0.3</v>
@@ -2487,13 +2487,13 @@
         <v>28.3</v>
       </c>
       <c r="H47" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I47" t="n">
         <v>2.1</v>
       </c>
       <c r="J47" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2578,7 +2578,7 @@
         <v>1.7</v>
       </c>
       <c r="I49" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2616,13 +2616,13 @@
         <v>100</v>
       </c>
       <c r="G50" t="n">
-        <v>2.9</v>
+        <v>4.9</v>
       </c>
       <c r="H50" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2760,10 +2760,10 @@
         <v>43.6</v>
       </c>
       <c r="K53" t="n">
-        <v>29.2</v>
+        <v>28.9</v>
       </c>
       <c r="L53" t="n">
-        <v>19</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="54">
@@ -2804,10 +2804,10 @@
         <v>24.9</v>
       </c>
       <c r="K54" t="n">
-        <v>13.1</v>
+        <v>13.8</v>
       </c>
       <c r="L54" t="n">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="55">
@@ -2848,10 +2848,10 @@
         <v>10.2</v>
       </c>
       <c r="K55" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="L55" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="56">
@@ -2980,7 +2980,7 @@
         <v>3.8</v>
       </c>
       <c r="K58" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="L58" t="n">
         <v>0.4</v>
@@ -3112,7 +3112,7 @@
         <v>3.6</v>
       </c>
       <c r="K61" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="L61" t="n">
         <v>0.4</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-29)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -607,7 +607,7 @@
         <v>6.7</v>
       </c>
       <c r="L4" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="5">
@@ -1211,19 +1211,19 @@
         <v>97.2</v>
       </c>
       <c r="H18" t="n">
-        <v>69.5</v>
+        <v>73.5</v>
       </c>
       <c r="I18" t="n">
-        <v>45.7</v>
+        <v>48.3</v>
       </c>
       <c r="J18" t="n">
-        <v>23.8</v>
+        <v>25.1</v>
       </c>
       <c r="K18" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
       <c r="L18" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="19">
@@ -1258,16 +1258,16 @@
         <v>74.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>45.9</v>
+        <v>44.5</v>
       </c>
       <c r="J19" t="n">
-        <v>29.5</v>
+        <v>28.6</v>
       </c>
       <c r="K19" t="n">
-        <v>17.1</v>
+        <v>16.5</v>
       </c>
       <c r="L19" t="n">
-        <v>8.699999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="20">
@@ -1302,16 +1302,16 @@
         <v>74.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>38.9</v>
+        <v>40.2</v>
       </c>
       <c r="J20" t="n">
-        <v>22.9</v>
+        <v>23.5</v>
       </c>
       <c r="K20" t="n">
-        <v>12.7</v>
+        <v>13</v>
       </c>
       <c r="L20" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="21">
@@ -1390,13 +1390,13 @@
         <v>51.5</v>
       </c>
       <c r="I22" t="n">
-        <v>24.8</v>
+        <v>24.6</v>
       </c>
       <c r="J22" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K22" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="L22" t="n">
         <v>1.5</v>
@@ -1563,19 +1563,19 @@
         <v>63.9</v>
       </c>
       <c r="H26" t="n">
-        <v>22.8</v>
+        <v>18.8</v>
       </c>
       <c r="I26" t="n">
-        <v>11.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>3.5</v>
+        <v>2.6</v>
       </c>
       <c r="K26" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
@@ -1968,10 +1968,10 @@
         <v>35.9</v>
       </c>
       <c r="K35" t="n">
-        <v>20.3</v>
+        <v>20</v>
       </c>
       <c r="L35" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="36">
@@ -2012,10 +2012,10 @@
         <v>24.7</v>
       </c>
       <c r="K36" t="n">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="L36" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="37">
@@ -2100,10 +2100,10 @@
         <v>10.4</v>
       </c>
       <c r="K38" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="L38" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="39">
@@ -2323,7 +2323,7 @@
         <v>0.2</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="44">
@@ -2757,13 +2757,13 @@
         <v>61.4</v>
       </c>
       <c r="J53" t="n">
-        <v>43.6</v>
+        <v>44.1</v>
       </c>
       <c r="K53" t="n">
-        <v>28.9</v>
+        <v>29.6</v>
       </c>
       <c r="L53" t="n">
-        <v>18.7</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="54">
@@ -2792,22 +2792,22 @@
         <v>100</v>
       </c>
       <c r="G54" t="n">
-        <v>95.09999999999999</v>
+        <v>94.3</v>
       </c>
       <c r="H54" t="n">
-        <v>75.2</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>51.9</v>
+        <v>49.1</v>
       </c>
       <c r="J54" t="n">
-        <v>24.9</v>
+        <v>23.3</v>
       </c>
       <c r="K54" t="n">
-        <v>13.8</v>
+        <v>12.8</v>
       </c>
       <c r="L54" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="55">
@@ -2842,16 +2842,16 @@
         <v>56.8</v>
       </c>
       <c r="I55" t="n">
-        <v>25.9</v>
+        <v>28.1</v>
       </c>
       <c r="J55" t="n">
-        <v>10.2</v>
+        <v>11.1</v>
       </c>
       <c r="K55" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="L55" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -2889,7 +2889,7 @@
         <v>16.1</v>
       </c>
       <c r="J56" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="K56" t="n">
         <v>2.9</v>
@@ -2933,10 +2933,10 @@
         <v>8.800000000000001</v>
       </c>
       <c r="J57" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="K57" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
         <v>0.3</v>
@@ -2974,13 +2974,13 @@
         <v>30.6</v>
       </c>
       <c r="I58" t="n">
-        <v>11.3</v>
+        <v>11.4</v>
       </c>
       <c r="J58" t="n">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="K58" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L58" t="n">
         <v>0.4</v>
@@ -3015,13 +3015,13 @@
         <v>57.7</v>
       </c>
       <c r="H59" t="n">
-        <v>15.9</v>
+        <v>16.3</v>
       </c>
       <c r="I59" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="J59" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="K59" t="n">
         <v>0.3</v>
@@ -3068,7 +3068,7 @@
         <v>0.6</v>
       </c>
       <c r="K60" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -3147,7 +3147,7 @@
         <v>42.3</v>
       </c>
       <c r="H62" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="I62" t="n">
         <v>2.4</v>
@@ -3238,7 +3238,7 @@
         <v>7.4</v>
       </c>
       <c r="I64" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="J64" t="n">
         <v>0.6</v>
@@ -3408,10 +3408,10 @@
         <v>100</v>
       </c>
       <c r="G68" t="n">
-        <v>4.9</v>
+        <v>5.7</v>
       </c>
       <c r="H68" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I68" t="n">
         <v>0.1</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-03-30)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -507,19 +507,19 @@
         <v>95.2</v>
       </c>
       <c r="H2" t="n">
-        <v>78</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>59.7</v>
+        <v>58.1</v>
       </c>
       <c r="J2" t="n">
-        <v>43.4</v>
+        <v>40.9</v>
       </c>
       <c r="K2" t="n">
-        <v>27.6</v>
+        <v>24.4</v>
       </c>
       <c r="L2" t="n">
-        <v>15.3</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="3">
@@ -551,19 +551,19 @@
         <v>94.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>65.8</v>
+        <v>66</v>
       </c>
       <c r="I3" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="J3" t="n">
-        <v>15</v>
+        <v>16.2</v>
       </c>
       <c r="K3" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="L3" t="n">
-        <v>2.4</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="4">
@@ -601,10 +601,10 @@
         <v>31.9</v>
       </c>
       <c r="J4" t="n">
-        <v>14.3</v>
+        <v>14.7</v>
       </c>
       <c r="K4" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
       <c r="L4" t="n">
         <v>2.7</v>
@@ -642,13 +642,13 @@
         <v>34</v>
       </c>
       <c r="I5" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="J5" t="n">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="K5" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L5" t="n">
         <v>0.4</v>
@@ -686,13 +686,13 @@
         <v>54.3</v>
       </c>
       <c r="I6" t="n">
-        <v>19.1</v>
+        <v>20.2</v>
       </c>
       <c r="J6" t="n">
-        <v>9.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="K6" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="L6" t="n">
         <v>1.3</v>
@@ -730,13 +730,13 @@
         <v>35.7</v>
       </c>
       <c r="I7" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="J7" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="K7" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="L7" t="n">
         <v>0.6</v>
@@ -771,16 +771,16 @@
         <v>64.3</v>
       </c>
       <c r="H8" t="n">
-        <v>24</v>
+        <v>23.8</v>
       </c>
       <c r="I8" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="J8" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="K8" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="L8" t="n">
         <v>0.2</v>
@@ -859,13 +859,13 @@
         <v>44.4</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="J10" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>0.2</v>
@@ -994,7 +994,7 @@
         <v>6</v>
       </c>
       <c r="I13" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J13" t="n">
         <v>0.2</v>
@@ -1220,10 +1220,10 @@
         <v>25.1</v>
       </c>
       <c r="K18" t="n">
-        <v>12.8</v>
+        <v>13.9</v>
       </c>
       <c r="L18" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="19">
@@ -1264,10 +1264,10 @@
         <v>28.6</v>
       </c>
       <c r="K19" t="n">
-        <v>16.5</v>
+        <v>16.9</v>
       </c>
       <c r="L19" t="n">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="20">
@@ -1308,7 +1308,7 @@
         <v>23.5</v>
       </c>
       <c r="K20" t="n">
-        <v>13</v>
+        <v>13.2</v>
       </c>
       <c r="L20" t="n">
         <v>6.1</v>
@@ -1396,7 +1396,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="K22" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="L22" t="n">
         <v>1.5</v>
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27">
@@ -1956,22 +1956,22 @@
         <v>100</v>
       </c>
       <c r="G35" t="n">
-        <v>91.09999999999999</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>76</v>
+        <v>79.2</v>
       </c>
       <c r="I35" t="n">
-        <v>54.8</v>
+        <v>58.3</v>
       </c>
       <c r="J35" t="n">
-        <v>35.9</v>
+        <v>39.6</v>
       </c>
       <c r="K35" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="L35" t="n">
-        <v>11.9</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="36">
@@ -2006,16 +2006,16 @@
         <v>73.09999999999999</v>
       </c>
       <c r="I36" t="n">
-        <v>46.1</v>
+        <v>49.6</v>
       </c>
       <c r="J36" t="n">
-        <v>24.7</v>
+        <v>25.7</v>
       </c>
       <c r="K36" t="n">
-        <v>11.3</v>
+        <v>11.8</v>
       </c>
       <c r="L36" t="n">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="37">
@@ -2047,13 +2047,13 @@
         <v>88.3</v>
       </c>
       <c r="H37" t="n">
-        <v>43.5</v>
+        <v>45.5</v>
       </c>
       <c r="I37" t="n">
-        <v>18.2</v>
+        <v>19.1</v>
       </c>
       <c r="J37" t="n">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="K37" t="n">
         <v>2.3</v>
@@ -2094,16 +2094,16 @@
         <v>46.7</v>
       </c>
       <c r="I38" t="n">
-        <v>20.8</v>
+        <v>19.2</v>
       </c>
       <c r="J38" t="n">
-        <v>10.4</v>
+        <v>9.5</v>
       </c>
       <c r="K38" t="n">
-        <v>4.2</v>
+        <v>3.8</v>
       </c>
       <c r="L38" t="n">
-        <v>1.9</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="39">
@@ -2138,10 +2138,10 @@
         <v>38.2</v>
       </c>
       <c r="I39" t="n">
-        <v>12.4</v>
+        <v>11.9</v>
       </c>
       <c r="J39" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="K39" t="n">
         <v>1.4</v>
@@ -2176,22 +2176,22 @@
         <v>100</v>
       </c>
       <c r="G40" t="n">
-        <v>78.3</v>
+        <v>76</v>
       </c>
       <c r="H40" t="n">
-        <v>48.2</v>
+        <v>45.5</v>
       </c>
       <c r="I40" t="n">
-        <v>24.2</v>
+        <v>19.5</v>
       </c>
       <c r="J40" t="n">
-        <v>10.6</v>
+        <v>7.6</v>
       </c>
       <c r="K40" t="n">
-        <v>4.3</v>
+        <v>2.9</v>
       </c>
       <c r="L40" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="41">
@@ -2229,7 +2229,7 @@
         <v>5.8</v>
       </c>
       <c r="J41" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="K41" t="n">
         <v>0.4</v>
@@ -2267,16 +2267,16 @@
         <v>53</v>
       </c>
       <c r="H42" t="n">
-        <v>11.7</v>
+        <v>10.3</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
       <c r="J42" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="K42" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L42" t="n">
         <v>0.1</v>
@@ -2311,19 +2311,19 @@
         <v>47</v>
       </c>
       <c r="H43" t="n">
-        <v>11.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="I43" t="n">
-        <v>3.9</v>
+        <v>3.5</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K43" t="n">
         <v>0.2</v>
       </c>
       <c r="L43" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2358,7 +2358,7 @@
         <v>12.2</v>
       </c>
       <c r="I44" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="J44" t="n">
         <v>1.2</v>
@@ -2396,13 +2396,13 @@
         <v>30.7</v>
       </c>
       <c r="G45" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="H45" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="I45" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
@@ -2440,13 +2440,13 @@
         <v>69.3</v>
       </c>
       <c r="G46" t="n">
-        <v>15.9</v>
+        <v>16.8</v>
       </c>
       <c r="H46" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="I46" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="J46" t="n">
         <v>0.3</v>
@@ -2490,10 +2490,10 @@
         <v>9.800000000000001</v>
       </c>
       <c r="I47" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="J47" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="K47" t="n">
         <v>0.1</v>
@@ -2534,7 +2534,7 @@
         <v>5.3</v>
       </c>
       <c r="I48" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="J48" t="n">
         <v>0.1</v>
@@ -2660,13 +2660,13 @@
         <v>59.4</v>
       </c>
       <c r="G51" t="n">
-        <v>7</v>
+        <v>3.4</v>
       </c>
       <c r="H51" t="n">
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="I51" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
@@ -2704,10 +2704,10 @@
         <v>40.6</v>
       </c>
       <c r="G52" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2760,10 +2760,10 @@
         <v>44.1</v>
       </c>
       <c r="K53" t="n">
-        <v>29.6</v>
+        <v>29</v>
       </c>
       <c r="L53" t="n">
-        <v>19.3</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="54">
@@ -2804,7 +2804,7 @@
         <v>23.3</v>
       </c>
       <c r="K54" t="n">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="L54" t="n">
         <v>7</v>
@@ -2851,7 +2851,7 @@
         <v>5</v>
       </c>
       <c r="L55" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="56">
@@ -3068,7 +3068,7 @@
         <v>0.6</v>
       </c>
       <c r="K60" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update bracket sim outputs (2026-04-05)
</commit_message>
<xml_diff>
--- a/2026_bracket_preds.xlsx
+++ b/2026_bracket_preds.xlsx
@@ -516,10 +516,10 @@
         <v>40.9</v>
       </c>
       <c r="K2" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="L2" t="n">
-        <v>12.8</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="3">
@@ -554,16 +554,16 @@
         <v>66</v>
       </c>
       <c r="I3" t="n">
-        <v>36.9</v>
+        <v>37.9</v>
       </c>
       <c r="J3" t="n">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="K3" t="n">
-        <v>7</v>
+        <v>7.4</v>
       </c>
       <c r="L3" t="n">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="4">
@@ -598,13 +598,13 @@
         <v>51.7</v>
       </c>
       <c r="I4" t="n">
-        <v>31.9</v>
+        <v>30.9</v>
       </c>
       <c r="J4" t="n">
-        <v>14.7</v>
+        <v>14.3</v>
       </c>
       <c r="K4" t="n">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="L4" t="n">
         <v>2.7</v>
@@ -651,7 +651,7 @@
         <v>1.4</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -692,10 +692,10 @@
         <v>10.1</v>
       </c>
       <c r="K6" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="L6" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -956,7 +956,7 @@
         <v>0.7</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1220,10 +1220,10 @@
         <v>25.1</v>
       </c>
       <c r="K18" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="L18" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="19">
@@ -1258,16 +1258,16 @@
         <v>74.09999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>44.5</v>
+        <v>45.9</v>
       </c>
       <c r="J19" t="n">
-        <v>28.6</v>
+        <v>29.5</v>
       </c>
       <c r="K19" t="n">
-        <v>16.9</v>
+        <v>17.3</v>
       </c>
       <c r="L19" t="n">
-        <v>8.6</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="20">
@@ -1299,19 +1299,19 @@
         <v>94.2</v>
       </c>
       <c r="H20" t="n">
-        <v>74.09999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>40.2</v>
+        <v>38.8</v>
       </c>
       <c r="J20" t="n">
-        <v>23.5</v>
+        <v>21.7</v>
       </c>
       <c r="K20" t="n">
-        <v>13.2</v>
+        <v>11.8</v>
       </c>
       <c r="L20" t="n">
-        <v>6.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="21">
@@ -1349,10 +1349,10 @@
         <v>13.6</v>
       </c>
       <c r="J21" t="n">
-        <v>4.4</v>
+        <v>4.7</v>
       </c>
       <c r="K21" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="L21" t="n">
         <v>0.5</v>
@@ -1393,13 +1393,13 @@
         <v>24.6</v>
       </c>
       <c r="J22" t="n">
-        <v>9.699999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="K22" t="n">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="L22" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="23">
@@ -1572,10 +1572,10 @@
         <v>2.6</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="27">
@@ -1651,7 +1651,7 @@
         <v>44.5</v>
       </c>
       <c r="H28" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="I28" t="n">
         <v>2.4</v>
@@ -1959,19 +1959,19 @@
         <v>95.09999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>79.2</v>
+        <v>80.8</v>
       </c>
       <c r="I35" t="n">
-        <v>58.3</v>
+        <v>61.5</v>
       </c>
       <c r="J35" t="n">
-        <v>39.6</v>
+        <v>42.7</v>
       </c>
       <c r="K35" t="n">
-        <v>22.5</v>
+        <v>25.9</v>
       </c>
       <c r="L35" t="n">
-        <v>14.2</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="36">
@@ -2009,13 +2009,13 @@
         <v>49.6</v>
       </c>
       <c r="J36" t="n">
-        <v>25.7</v>
+        <v>25.3</v>
       </c>
       <c r="K36" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="L36" t="n">
-        <v>6.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="37">
@@ -2053,13 +2053,13 @@
         <v>19.1</v>
       </c>
       <c r="J37" t="n">
-        <v>6.9</v>
+        <v>6.3</v>
       </c>
       <c r="K37" t="n">
         <v>2.3</v>
       </c>
       <c r="L37" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="38">
@@ -2094,13 +2094,13 @@
         <v>46.7</v>
       </c>
       <c r="I38" t="n">
-        <v>19.2</v>
+        <v>18</v>
       </c>
       <c r="J38" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="K38" t="n">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="L38" t="n">
         <v>1.7</v>
@@ -2138,16 +2138,16 @@
         <v>38.2</v>
       </c>
       <c r="I39" t="n">
-        <v>11.9</v>
+        <v>10.4</v>
       </c>
       <c r="J39" t="n">
-        <v>4.7</v>
+        <v>4.1</v>
       </c>
       <c r="K39" t="n">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L39" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="40">
@@ -2185,10 +2185,10 @@
         <v>19.5</v>
       </c>
       <c r="J40" t="n">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
       <c r="K40" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="L40" t="n">
         <v>1.1</v>
@@ -2229,7 +2229,7 @@
         <v>5.8</v>
       </c>
       <c r="J41" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="K41" t="n">
         <v>0.4</v>
@@ -2311,13 +2311,13 @@
         <v>47</v>
       </c>
       <c r="H43" t="n">
-        <v>9.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I43" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="J43" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="K43" t="n">
         <v>0.2</v>
@@ -2361,7 +2361,7 @@
         <v>4</v>
       </c>
       <c r="J44" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K44" t="n">
         <v>0.3</v>
@@ -2748,22 +2748,22 @@
         <v>100</v>
       </c>
       <c r="G53" t="n">
-        <v>97.2</v>
+        <v>95.2</v>
       </c>
       <c r="H53" t="n">
-        <v>77.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="I53" t="n">
-        <v>61.4</v>
+        <v>57.6</v>
       </c>
       <c r="J53" t="n">
-        <v>44.1</v>
+        <v>41</v>
       </c>
       <c r="K53" t="n">
-        <v>29</v>
+        <v>26.3</v>
       </c>
       <c r="L53" t="n">
-        <v>19.1</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="54">
@@ -2801,13 +2801,13 @@
         <v>49.1</v>
       </c>
       <c r="J54" t="n">
-        <v>23.3</v>
+        <v>24</v>
       </c>
       <c r="K54" t="n">
-        <v>12.7</v>
+        <v>11.9</v>
       </c>
       <c r="L54" t="n">
-        <v>7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="55">
@@ -2845,10 +2845,10 @@
         <v>28.1</v>
       </c>
       <c r="J55" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="K55" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="L55" t="n">
         <v>2.1</v>
@@ -2886,13 +2886,13 @@
         <v>52</v>
       </c>
       <c r="I56" t="n">
-        <v>16.1</v>
+        <v>17.6</v>
       </c>
       <c r="J56" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="K56" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="L56" t="n">
         <v>1.2</v>
@@ -2930,10 +2930,10 @@
         <v>32.6</v>
       </c>
       <c r="I57" t="n">
-        <v>8.800000000000001</v>
+        <v>10.1</v>
       </c>
       <c r="J57" t="n">
-        <v>3.2</v>
+        <v>3.6</v>
       </c>
       <c r="K57" t="n">
         <v>1</v>
@@ -2977,7 +2977,7 @@
         <v>11.4</v>
       </c>
       <c r="J58" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="K58" t="n">
         <v>1.3</v>
@@ -3021,7 +3021,7 @@
         <v>5.4</v>
       </c>
       <c r="J59" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="K59" t="n">
         <v>0.3</v>
@@ -3059,16 +3059,16 @@
         <v>33.6</v>
       </c>
       <c r="H60" t="n">
-        <v>5.7</v>
+        <v>7</v>
       </c>
       <c r="I60" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="J60" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K60" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
@@ -3103,16 +3103,16 @@
         <v>66.40000000000001</v>
       </c>
       <c r="H61" t="n">
-        <v>16.7</v>
+        <v>17.6</v>
       </c>
       <c r="I61" t="n">
-        <v>8.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="J61" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="K61" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="L61" t="n">
         <v>0.4</v>
@@ -3197,7 +3197,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="K63" t="n">
         <v>0</v>
@@ -3282,7 +3282,7 @@
         <v>10.7</v>
       </c>
       <c r="I65" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="J65" t="n">
         <v>0.4</v>
@@ -3452,10 +3452,10 @@
         <v>100</v>
       </c>
       <c r="G69" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="H69" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>

</xml_diff>